<commit_message>
initial commit for CG0464
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -1,39 +1,161 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/negative/01/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAEA5BF1-BB9C-0048-959C-62D404ABEEF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Library" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Datasets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Validation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Library" sheetId="1" r:id="rId1"/>
+    <sheet name="Datasets" sheetId="2" r:id="rId2"/>
+    <sheet name="Validation" sheetId="3" r:id="rId3"/>
+    <sheet name="zz.xpt" sheetId="4" r:id="rId4"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>sdtmig</t>
+  </si>
+  <si>
+    <t>3-4</t>
+  </si>
+  <si>
+    <t>Filename</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <t>Error group</t>
+  </si>
+  <si>
+    <t>Sheet</t>
+  </si>
+  <si>
+    <t>Error level</t>
+  </si>
+  <si>
+    <t>Row num</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Error value</t>
+  </si>
+  <si>
+    <t>zz.xpt</t>
+  </si>
+  <si>
+    <t>Custom Dataset</t>
+  </si>
+  <si>
+    <t>STUDYID</t>
+  </si>
+  <si>
+    <t>DOMAIN</t>
+  </si>
+  <si>
+    <t>Study Identifier</t>
+  </si>
+  <si>
+    <t>Domain Abbreviation</t>
+  </si>
+  <si>
+    <t>Char</t>
+  </si>
+  <si>
+    <t>Num</t>
+  </si>
+  <si>
+    <t>CDISCPILOT01</t>
+  </si>
+  <si>
+    <t>USUBJID</t>
+  </si>
+  <si>
+    <t>ZZSEQ</t>
+  </si>
+  <si>
+    <t>ZZTERM</t>
+  </si>
+  <si>
+    <t>Sequence Number</t>
+  </si>
+  <si>
+    <t>Unique Subject Identifier</t>
+  </si>
+  <si>
+    <t>ZZ</t>
+  </si>
+  <si>
+    <t>CDISC001</t>
+  </si>
+  <si>
+    <t>[ABSENT]</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -48,81 +170,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -410,36 +482,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>sdtmig</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>3-4</t>
-        </is>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -448,29 +508,28 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Filename</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Label</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -478,55 +537,132 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Error group</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Sheet</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Error level</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Row num</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Error value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF4426AC-ADD3-6641-9A03-C7226EFF36E9}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="2">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2">
+        <v>8</v>
+      </c>
+      <c r="D4" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
changes to match CG0464
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6295F79-5394-C743-8F50-BD2C4A491F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA3EDB8B-BD04-A146-89AB-DF37436B7581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="33">
   <si>
     <t>Product</t>
   </si>
@@ -110,6 +110,18 @@
   </si>
   <si>
     <t>ZZTRT</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>define_dataset_class</t>
+  </si>
+  <si>
+    <t>INTERVENTIONS</t>
+  </si>
+  <si>
+    <t>domain</t>
   </si>
 </sst>
 </file>
@@ -538,7 +550,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -571,8 +583,8 @@
       <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="D2">
-        <v>1</v>
+      <c r="D2" t="s">
+        <v>29</v>
       </c>
       <c r="E2" t="s">
         <v>28</v>
@@ -581,8 +593,49 @@
         <v>27</v>
       </c>
     </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
updates after engine fixes
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E743C5E-484D-BC4D-BA38-E8F09BB0DBFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA918AA-83DB-9941-A97A-66F0153672B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="18" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="91">
   <si>
     <t>Product</t>
   </si>
@@ -307,6 +307,12 @@
   </si>
   <si>
     <t>DUMMY EPOCH</t>
+  </si>
+  <si>
+    <t>Mismatched Role</t>
+  </si>
+  <si>
+    <t>Timing</t>
   </si>
 </sst>
 </file>
@@ -433,34 +439,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal 3 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <font>
-        <i/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFCC"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color rgb="FFD9D9D9"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFD9D9D9"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFD9D9D9"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFD9D9D9"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <i/>
@@ -883,7 +862,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E456D595-1A57-0943-B18E-D88401008EB3}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -984,6 +963,86 @@
       </c>
       <c r="F5" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E7" t="s">
+        <v>62</v>
+      </c>
+      <c r="F7" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" t="s">
+        <v>63</v>
+      </c>
+      <c r="F8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1343,7 +1402,7 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="A2:M4">
-    <cfRule type="notContainsBlanks" dxfId="2" priority="1">
+    <cfRule type="notContainsBlanks" dxfId="1" priority="1">
       <formula>LEN(TRIM(A2))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1559,14 +1618,9 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:B4">
-    <cfRule type="notContainsBlanks" dxfId="1" priority="3">
+  <conditionalFormatting sqref="A2:L4">
+    <cfRule type="notContainsBlanks" dxfId="0" priority="1">
       <formula>LEN(TRIM(A2))&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:L4">
-    <cfRule type="notContainsBlanks" dxfId="0" priority="1">
-      <formula>LEN(TRIM(C2))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1575,6 +1629,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Comment xmlns="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010090ADB40D834AE945B19FCDA4041AC0CB" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c09bae7b217a3930fedb3a6204001e96">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xmlns:ns3="63ea592b-d684-45c7-8cdc-fad8f8e6bb41" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac018b55a0c98af8ca0cc741473a0b1c" ns2:_="" ns3:_="">
     <xsd:import namespace="9dee18c2-6da5-44c1-913e-bf7f393fe0e8"/>
@@ -1797,24 +1868,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Comment xmlns="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{173E2EFD-8922-4D2E-BE2E-AE460DA159D0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F7876C8-4097-41AA-906A-130684BD3FE8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9dee18c2-6da5-44c1-913e-bf7f393fe0e8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{35E82A84-6886-48D7-851E-66994726A649}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1831,22 +1903,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F7876C8-4097-41AA-906A-130684BD3FE8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9dee18c2-6da5-44c1-913e-bf7f393fe0e8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{173E2EFD-8922-4D2E-BE2E-AE460DA159D0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
filter ce first + 2 errors per ce usubjid 001 + death / death
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -37,7 +37,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -91,12 +91,8 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -116,6 +112,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -155,12 +163,6 @@
         <bgColor/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -181,7 +183,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -189,13 +191,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -589,7 +592,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F10"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -628,7 +631,7 @@
         <v>CEDECOD</v>
       </c>
       <c r="F2" s="2" t="str">
-        <v>LAST CONTACT</v>
+        <v>DEATH</v>
       </c>
     </row>
     <row r="3">
@@ -652,63 +655,63 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="str">
+      <c r="B4" s="2" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C4" s="3" t="str">
+      <c r="C4" s="2" t="str">
         <v>Record</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="str">
+      <c r="E4" s="2" t="str">
         <v>DTHFL</v>
       </c>
-      <c r="F4" s="3" t="str">
+      <c r="F4" s="2" t="str">
         <v>N</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2">
+      <c r="A5" s="3">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="3" t="str">
         <v>ce.xpt</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C5" s="3" t="str">
         <v>Record</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="3">
         <v>6</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E5" s="3" t="str">
         <v>CEDECOD</v>
       </c>
-      <c r="F5" s="2" t="str">
+      <c r="F5" s="3" t="str">
+        <v>LAST CONTACT</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="str">
+        <v>ce.xpt</v>
+      </c>
+      <c r="C6" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D6" s="3">
+        <v>6</v>
+      </c>
+      <c r="E6" s="3" t="str">
+        <v>CETERM</v>
+      </c>
+      <c r="F6" s="3" t="str">
         <v>DEATH</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>2</v>
-      </c>
-      <c r="B6" s="2" t="str">
-        <v>ce.xpt</v>
-      </c>
-      <c r="C6" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D6" s="2">
-        <v>6</v>
-      </c>
-      <c r="E6" s="2" t="str">
-        <v>CETERM</v>
-      </c>
-      <c r="F6" s="2" t="str">
-        <v>PROGRESSIVE DISEASE</v>
       </c>
     </row>
     <row r="7">
@@ -722,7 +725,7 @@
         <v>Record</v>
       </c>
       <c r="D7" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E7" s="3" t="str">
         <v>DTHFL</v>
@@ -731,16 +734,76 @@
         <v>N</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3" t="str">
+        <v>ce.xpt</v>
+      </c>
+      <c r="C8" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D8" s="3">
+        <v>7</v>
+      </c>
+      <c r="E8" s="3" t="str">
+        <v>CEDECOD</v>
+      </c>
+      <c r="F8" s="3" t="str">
+        <v>DEATH</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>3</v>
+      </c>
+      <c r="B9" s="3" t="str">
+        <v>ce.xpt</v>
+      </c>
+      <c r="C9" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D9" s="3">
+        <v>7</v>
+      </c>
+      <c r="E9" s="3" t="str">
+        <v>CETERM</v>
+      </c>
+      <c r="F9" s="3" t="str">
+        <v>PROGRESSIVE DISEASE</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>3</v>
+      </c>
+      <c r="B10" s="3" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C10" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D10" s="3">
+        <v>6</v>
+      </c>
+      <c r="E10" s="3" t="str">
+        <v>DTHFL</v>
+      </c>
+      <c r="F10" s="3" t="str">
+        <v>N</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H9"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="str">
@@ -847,28 +910,28 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="str">
+      <c r="A5" s="2" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="3" t="str">
+      <c r="B5" s="2" t="str">
         <v>CE</v>
       </c>
-      <c r="C5" s="3" t="str">
+      <c r="C5" s="2" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>1</v>
       </c>
       <c r="E5" s="7" t="str">
-        <v>LAST CONTACT</v>
+        <v>DEATH</v>
       </c>
       <c r="F5" s="8" t="str">
         <v>DEATH</v>
       </c>
-      <c r="G5" s="3" t="str">
+      <c r="G5" s="2" t="str">
         <v>CTCAE 4.03</v>
       </c>
-      <c r="H5" s="3" t="str">
+      <c r="H5" s="2" t="str">
         <v>GRADE 1</v>
       </c>
     </row>
@@ -880,22 +943,22 @@
         <v>CE</v>
       </c>
       <c r="C6" s="3" t="str">
-        <v>CDISC002</v>
+        <v>CDISC001</v>
       </c>
       <c r="D6" s="3">
         <v>2</v>
       </c>
-      <c r="E6" s="7" t="str">
+      <c r="E6" s="9" t="str">
+        <v>LAST CONTACT</v>
+      </c>
+      <c r="F6" s="10" t="str">
         <v>DEATH</v>
-      </c>
-      <c r="F6" s="7" t="str">
-        <v>PROGRESSIVE DISEASE</v>
       </c>
       <c r="G6" s="3" t="str">
         <v>CTCAE 4.03</v>
       </c>
       <c r="H6" s="3" t="str">
-        <v>GRADE 2</v>
+        <v>GRADE 1</v>
       </c>
     </row>
     <row r="7">
@@ -906,27 +969,79 @@
         <v>CE</v>
       </c>
       <c r="C7" s="3" t="str">
-        <v>CDISC003</v>
+        <v>CDISC002</v>
       </c>
       <c r="D7" s="3">
         <v>3</v>
       </c>
-      <c r="E7" s="3" t="str">
-        <v>COMPLETED</v>
-      </c>
-      <c r="F7" s="3" t="str">
-        <v>Migraine</v>
+      <c r="E7" s="10" t="str">
+        <v>DEATH</v>
+      </c>
+      <c r="F7" s="10" t="str">
+        <v>PROGRESSIVE DISEASE</v>
       </c>
       <c r="G7" s="3" t="str">
         <v>CTCAE 4.03</v>
       </c>
       <c r="H7" s="3" t="str">
+        <v>GRADE 2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B8" s="2" t="str">
+        <v>CE</v>
+      </c>
+      <c r="C8" s="2" t="str">
+        <v>CDISC002</v>
+      </c>
+      <c r="D8" s="2">
+        <v>4</v>
+      </c>
+      <c r="E8" s="2" t="str">
+        <v>LAST CONTACT</v>
+      </c>
+      <c r="F8" s="2" t="str">
+        <v>PROGRESSIVE DISEASE</v>
+      </c>
+      <c r="G8" s="2" t="str">
+        <v>CTCAE 4.03</v>
+      </c>
+      <c r="H8" s="2" t="str">
+        <v>GRADE 2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B9" s="3" t="str">
+        <v>CE</v>
+      </c>
+      <c r="C9" s="3" t="str">
+        <v>CDISC003</v>
+      </c>
+      <c r="D9" s="3">
+        <v>5</v>
+      </c>
+      <c r="E9" s="3" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="F9" s="3" t="str">
+        <v>Migraine</v>
+      </c>
+      <c r="G9" s="3" t="str">
+        <v>CTCAE 4.03</v>
+      </c>
+      <c r="H9" s="3" t="str">
         <v>GRADE 1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -966,7 +1081,7 @@
       <c r="J1" s="4" t="str">
         <v>RFPENDTC</v>
       </c>
-      <c r="K1" s="9" t="str">
+      <c r="K1" s="11" t="str">
         <v>DTHDTC</v>
       </c>
       <c r="L1" s="4" t="str">
@@ -993,19 +1108,19 @@
       <c r="S1" s="4" t="str">
         <v>ETHNIC</v>
       </c>
-      <c r="T1" s="10" t="str">
+      <c r="T1" s="12" t="str">
         <v>ARMCD</v>
       </c>
       <c r="U1" s="4" t="str">
         <v>ARM</v>
       </c>
-      <c r="V1" s="10" t="str">
+      <c r="V1" s="12" t="str">
         <v>ACTARMCD</v>
       </c>
-      <c r="W1" s="10" t="str">
+      <c r="W1" s="12" t="str">
         <v>ACTARM</v>
       </c>
-      <c r="X1" s="10" t="str">
+      <c r="X1" s="12" t="str">
         <v>ARMNRS</v>
       </c>
       <c r="Y1" s="4" t="str">
@@ -1286,10 +1401,10 @@
       <c r="J5" s="3" t="str">
         <v>2021-02-18</v>
       </c>
-      <c r="K5" s="11" t="str">
+      <c r="K5" s="13" t="str">
         <v>2021-02-18</v>
       </c>
-      <c r="L5" s="8" t="str">
+      <c r="L5" s="10" t="str">
         <v>N</v>
       </c>
       <c r="M5" s="3" t="str">
@@ -1298,10 +1413,10 @@
       <c r="N5" s="3" t="str">
         <v>1940-01-14</v>
       </c>
-      <c r="O5" s="12" t="str">
+      <c r="O5" s="14" t="str">
         <v>78</v>
       </c>
-      <c r="P5" s="12" t="str">
+      <c r="P5" s="14" t="str">
         <v>YEARS</v>
       </c>
       <c r="Q5" s="3" t="str">
@@ -1313,19 +1428,19 @@
       <c r="S5" s="3" t="str">
         <v>HISPANIC OR LATINO</v>
       </c>
-      <c r="T5" s="12" t="str">
+      <c r="T5" s="14" t="str">
         <v>IKD</v>
       </c>
-      <c r="U5" s="12" t="str">
+      <c r="U5" s="14" t="str">
         <v>IKd</v>
       </c>
-      <c r="V5" s="12" t="str">
+      <c r="V5" s="14" t="str">
         <v>IKD</v>
       </c>
-      <c r="W5" s="12" t="str">
+      <c r="W5" s="14" t="str">
         <v>IKd</v>
       </c>
-      <c r="X5" s="12" t="str">
+      <c r="X5" s="14" t="str">
         <v/>
       </c>
       <c r="Y5" s="3" t="str">
@@ -1366,10 +1481,10 @@
       <c r="J6" s="3" t="str">
         <v>2021-11-25</v>
       </c>
-      <c r="K6" s="12" t="str">
+      <c r="K6" s="14" t="str">
         <v>2021-11-25</v>
       </c>
-      <c r="L6" s="13" t="str">
+      <c r="L6" s="10" t="str">
         <v>N</v>
       </c>
       <c r="M6" s="3" t="str">
@@ -1378,10 +1493,10 @@
       <c r="N6" s="3" t="str">
         <v>1946-09-13</v>
       </c>
-      <c r="O6" s="12" t="str">
+      <c r="O6" s="14" t="str">
         <v>71</v>
       </c>
-      <c r="P6" s="12" t="str">
+      <c r="P6" s="14" t="str">
         <v>YEARS</v>
       </c>
       <c r="Q6" s="3" t="str">
@@ -1393,19 +1508,19 @@
       <c r="S6" s="3" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T6" s="12" t="str">
+      <c r="T6" s="14" t="str">
         <v>IKD</v>
       </c>
-      <c r="U6" s="12" t="str">
+      <c r="U6" s="14" t="str">
         <v>IKd</v>
       </c>
-      <c r="V6" s="12" t="str">
+      <c r="V6" s="14" t="str">
         <v>IKD</v>
       </c>
-      <c r="W6" s="12" t="str">
+      <c r="W6" s="14" t="str">
         <v>IKd</v>
       </c>
-      <c r="X6" s="12" t="str">
+      <c r="X6" s="14" t="str">
         <v/>
       </c>
       <c r="Y6" s="3" t="str">
@@ -1446,7 +1561,7 @@
       <c r="J7" s="3" t="str">
         <v>2018-09-04</v>
       </c>
-      <c r="K7" s="12" t="str">
+      <c r="K7" s="14" t="str">
         <v>2018-09-04</v>
       </c>
       <c r="L7" s="3" t="str">
@@ -1458,10 +1573,10 @@
       <c r="N7" s="3" t="str">
         <v>1947-12-23</v>
       </c>
-      <c r="O7" s="12" t="str">
+      <c r="O7" s="14" t="str">
         <v>70</v>
       </c>
-      <c r="P7" s="12" t="str">
+      <c r="P7" s="14" t="str">
         <v>YEARS</v>
       </c>
       <c r="Q7" s="3" t="str">
@@ -1473,19 +1588,19 @@
       <c r="S7" s="3" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T7" s="12" t="str">
+      <c r="T7" s="14" t="str">
         <v>IKD</v>
       </c>
-      <c r="U7" s="12" t="str">
+      <c r="U7" s="14" t="str">
         <v>IKd</v>
       </c>
-      <c r="V7" s="12" t="str">
+      <c r="V7" s="14" t="str">
         <v>IKD</v>
       </c>
-      <c r="W7" s="12" t="str">
+      <c r="W7" s="14" t="str">
         <v>IKd</v>
       </c>
-      <c r="X7" s="12" t="str">
+      <c r="X7" s="14" t="str">
         <v/>
       </c>
       <c r="Y7" s="3" t="str">

</xml_diff>

<commit_message>
Created rule (YAML) and test data and performed validation
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -1,42 +1,149 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\els_janssens\CORE\Rule_Authoring\core-contributor\rules\NEW-RULE\negative\01\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{766970D4-8034-4F70-B86D-28AD8FE5D9E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
     <sheet name="Datasets" sheetId="2" r:id="rId2"/>
     <sheet name="Validation" sheetId="3" r:id="rId3"/>
     <sheet name="cm.xpt" sheetId="4" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="38">
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>sdtmig</t>
+  </si>
+  <si>
+    <t>3-4</t>
+  </si>
+  <si>
+    <t>Filename</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <t>cm.xpt</t>
+  </si>
+  <si>
+    <t>Concomitant and Prior Medications</t>
+  </si>
+  <si>
+    <t>Error group</t>
+  </si>
+  <si>
+    <t>Sheet</t>
+  </si>
+  <si>
+    <t>Error level</t>
+  </si>
+  <si>
+    <t>Row num</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Error value</t>
+  </si>
+  <si>
+    <t>Dataset</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>define_variable_origin_type</t>
+  </si>
+  <si>
+    <t>Protocol</t>
+  </si>
+  <si>
+    <t>variable_name</t>
+  </si>
+  <si>
+    <t>CMTRT</t>
+  </si>
+  <si>
+    <t>STUDYID</t>
+  </si>
+  <si>
+    <t>DOMAIN</t>
+  </si>
+  <si>
+    <t>USUBJID</t>
+  </si>
+  <si>
+    <t>CMSEQ</t>
+  </si>
+  <si>
+    <t>Study Identifier</t>
+  </si>
+  <si>
+    <t>Domain Abbreviation</t>
+  </si>
+  <si>
+    <t>Unique Subject Identifier</t>
+  </si>
+  <si>
+    <t>Sequence Number</t>
+  </si>
+  <si>
+    <t>Reported Name of Drug, Med, or Therapy</t>
+  </si>
+  <si>
+    <t>Char</t>
+  </si>
+  <si>
+    <t>Num</t>
+  </si>
+  <si>
+    <t>ABC</t>
+  </si>
+  <si>
+    <t>CM</t>
+  </si>
+  <si>
+    <t>ABC-001</t>
+  </si>
+  <si>
+    <t>Ibuprofen</t>
+  </si>
+  <si>
+    <t>Paracetamol</t>
+  </si>
+  <si>
+    <t>define_variable_source_type</t>
+  </si>
+  <si>
+    <t>Investigator</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -46,41 +153,25 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <i/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none">
-        <bgColor/>
-      </patternFill>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125">
-        <bgColor/>
-      </patternFill>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
-        <bgColor/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -89,21 +180,28 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs>
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -428,253 +526,295 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="str">
-        <v>Product</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>Version</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="str">
-        <v>sdtmig</v>
-      </c>
-      <c r="B2" s="3" t="str">
-        <v>3-4</v>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
+    <ignoredError sqref="A1:B2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="str">
-        <v>Filename</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>Label</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="str">
-        <v>cm.xpt</v>
-      </c>
-      <c r="B2" s="3" t="str">
-        <v>Concomitant and Prior Medications</v>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
+    <ignoredError sqref="A1:B2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="31.42578125" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="str">
-        <v>Error group</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>Sheet</v>
-      </c>
-      <c r="C1" s="3" t="str">
-        <v>Error level</v>
-      </c>
-      <c r="D1" s="3" t="str">
-        <v>Row num</v>
-      </c>
-      <c r="E1" s="3" t="str">
-        <v>Variable</v>
-      </c>
-      <c r="F1" s="3" t="str">
-        <v>Error value</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
-        <v>cm.xpt</v>
-      </c>
-      <c r="C2" s="2" t="str">
-        <v>Dataset</v>
-      </c>
-      <c r="D2" s="2" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="E2" s="2" t="str">
-        <v>define_variable_origin_type</v>
-      </c>
-      <c r="F2" s="2" t="str">
-        <v>Protocol</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2">
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
-        <v>cm.xpt</v>
-      </c>
-      <c r="C3" s="2" t="str">
-        <v>Dataset</v>
-      </c>
-      <c r="D3" s="2" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="E3" s="2" t="str">
-        <v>variable_name</v>
-      </c>
-      <c r="F3" s="2" t="str">
-        <v>CMTRT</v>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError sqref="A3:F3 A1:F1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.85546875" customWidth="1"/>
+    <col min="2" max="2" width="27.5703125" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="5" max="5" width="38.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="str">
-        <v>STUDYID</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>DOMAIN</v>
-      </c>
-      <c r="C1" s="3" t="str">
-        <v>USUBJID</v>
-      </c>
-      <c r="D1" s="3" t="str">
-        <v>CMSEQ</v>
-      </c>
-      <c r="E1" s="3" t="str">
-        <v>CMTRT</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="str">
-        <v>Study Identifier</v>
-      </c>
-      <c r="B2" s="4" t="str">
-        <v>Domain Abbreviation</v>
-      </c>
-      <c r="C2" s="4" t="str">
-        <v>Unique Subject Identifier</v>
-      </c>
-      <c r="D2" s="4" t="str">
-        <v>Sequence Number</v>
-      </c>
-      <c r="E2" s="4" t="str">
-        <v>Reported Name of Drug, Med, or Therapy</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="4" t="str">
-        <v>Num</v>
-      </c>
-      <c r="E3" s="4" t="str">
-        <v>Char</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
         <v>10</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="2">
         <v>2</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="2">
         <v>14</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="2">
         <v>8</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="str">
-        <v>ABC</v>
-      </c>
-      <c r="B5" s="3" t="str">
-        <v>CM</v>
-      </c>
-      <c r="C5" s="3" t="str">
-        <v>ABC-001</v>
-      </c>
-      <c r="D5" s="3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="1">
         <v>1</v>
       </c>
-      <c r="E5" s="3" t="str">
-        <v>Ibuprofen</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="str">
-        <v>ABC</v>
-      </c>
-      <c r="B6" s="3" t="str">
-        <v>CM</v>
-      </c>
-      <c r="C6" s="3" t="str">
-        <v>ABC-001</v>
-      </c>
-      <c r="D6" s="3">
+      <c r="E5" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="1">
         <v>2</v>
       </c>
-      <c r="E6" s="3" t="str">
-        <v>Paracetamol</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="str">
-        <v>ABC</v>
-      </c>
-      <c r="B7" s="3" t="str">
-        <v>CM</v>
-      </c>
-      <c r="C7" s="3" t="str">
-        <v>ABC-001</v>
-      </c>
-      <c r="D7" s="3">
+      <c r="E6" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="1">
         <v>3</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError sqref="A1:E7" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updates after engine fix
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0250BA51-D202-F143-B178-0440B52C856D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19211613-0E17-5349-A6DF-4D6C030F367A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="181">
   <si>
     <t>Product</t>
   </si>
@@ -560,16 +560,13 @@
     <t>Record</t>
   </si>
   <si>
-    <t>1000398888888880</t>
-  </si>
-  <si>
     <t>Medical History</t>
   </si>
   <si>
     <t>Adverse Events</t>
   </si>
   <si>
-    <t>10046318</t>
+    <t>1004631800</t>
   </si>
 </sst>
 </file>
@@ -640,7 +637,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -715,21 +712,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="6"/>
-      </left>
-      <right style="thin">
-        <color theme="6"/>
-      </right>
-      <top style="thin">
-        <color theme="6"/>
-      </top>
-      <bottom style="thin">
-        <color theme="6"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -780,9 +762,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1178,20 +1158,20 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>175</v>
       </c>
-      <c r="B2" s="18" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>176</v>
       </c>
-      <c r="B3" s="18" t="s">
-        <v>180</v>
+      <c r="B3" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -1243,8 +1223,8 @@
       <c r="E2" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="17">
-        <v>10049663</v>
+      <c r="F2" s="18">
+        <v>1004966300</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -1263,7 +1243,7 @@
       <c r="E3" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="17"/>
+      <c r="F3" s="18"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
@@ -1281,8 +1261,8 @@
       <c r="E4" t="s">
         <v>102</v>
       </c>
-      <c r="F4" s="17">
-        <v>10046318</v>
+      <c r="F4" s="18">
+        <v>1004631800</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -1301,7 +1281,7 @@
       <c r="E5" t="s">
         <v>102</v>
       </c>
-      <c r="F5" s="17"/>
+      <c r="F5" s="18"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
@@ -1320,7 +1300,7 @@
         <v>102</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -1353,6 +1333,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93E8F0DE-CD04-B340-8520-6F5AE3E29670}">
   <dimension ref="A1:T9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="8" max="8" width="11.1640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -1625,7 +1608,7 @@
         <v>59</v>
       </c>
       <c r="H5" s="7">
-        <v>10049663</v>
+        <v>1004966300</v>
       </c>
       <c r="I5" t="s">
         <v>60</v>
@@ -1922,6 +1905,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C53B671-2300-4443-9C35-3D147F6F9A59}">
   <dimension ref="A1:AA10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="8" max="8" width="10.1640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
@@ -2278,7 +2264,7 @@
         <v>138</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="I5" s="12" t="s">
         <v>139</v>

</xml_diff>

<commit_message>
use dummy data term DI(DEHYDROABIETYL)AMINE ACETATE
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -62,9 +62,18 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -78,6 +87,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -107,7 +128,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -115,6 +136,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -559,7 +582,7 @@
         <v>TSVAL</v>
       </c>
       <c r="F3" s="4" t="str">
-        <v>DUMMYSRSTERM</v>
+        <v>FAKEUNIITERM</v>
       </c>
     </row>
   </sheetData>
@@ -612,104 +635,104 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Group ID</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Trial Summary Parameter Short Name</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Trial Summary Parameter</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Parameter Value</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Parameter Null Flavor</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Parameter Value Code</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Name of the Reference Terminology</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="6" t="str">
         <v>Version of the Reference Terminology</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="D3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="5" t="str">
+      <c r="D3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>10</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>8</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="6">
         <v>5</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="6">
         <v>8</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="6">
         <v>40</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="6">
         <v>149</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="6">
         <v>2</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="6">
         <v>11</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="6">
         <v>18</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="6">
         <v>10</v>
       </c>
     </row>
@@ -726,16 +749,19 @@
       <c r="D5" s="4" t="str">
         <v/>
       </c>
-      <c r="E5" s="6" t="str">
+      <c r="E5" s="7" t="str">
         <v>CURTRT</v>
       </c>
       <c r="F5" s="4" t="str">
         <v>Extension Trial Indicator</v>
       </c>
-      <c r="G5" s="6" t="str">
+      <c r="G5" s="8" t="str">
         <v>FAKEUNIITERM</v>
       </c>
-      <c r="I5" s="2" t="str">
+      <c r="H5" s="2" t="str">
+        <v/>
+      </c>
+      <c r="I5" s="4" t="str">
         <v>00000UNII1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
re-ran tests with updated is_not_ordered_set
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -62,18 +62,9 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -87,18 +78,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -128,7 +107,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -136,8 +115,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -832,95 +809,95 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="5" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="5" t="str">
         <v>Description of Planned Arm</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Planned Order of Element within Arm</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="5" t="str">
         <v>Element Code</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="5" t="str">
         <v>Description of Element</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="5" t="str">
         <v>Branch</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="5" t="str">
         <v>Transition Rule</v>
       </c>
-      <c r="J2" s="6" t="str">
+      <c r="J2" s="5" t="str">
         <v>Epoch</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
+      <c r="A3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="B3" s="6" t="str">
+      <c r="B3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="C3" s="6" t="str">
+      <c r="C3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="D3" s="6" t="str">
+      <c r="D3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="E3" s="6" t="str">
+      <c r="E3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="F3" s="6" t="str">
+      <c r="F3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="G3" s="6" t="str">
+      <c r="G3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="H3" s="6" t="str">
+      <c r="H3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="I3" s="6" t="str">
+      <c r="I3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="J3" s="6" t="str">
+      <c r="J3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="str">
+      <c r="A4" s="5" t="str">
         <v>12</v>
       </c>
-      <c r="B4" s="6" t="str">
+      <c r="B4" s="5" t="str">
         <v>2</v>
       </c>
-      <c r="C4" s="6" t="str">
+      <c r="C4" s="5" t="str">
         <v>8</v>
       </c>
-      <c r="D4" s="6" t="str">
+      <c r="D4" s="5" t="str">
         <v>28</v>
       </c>
-      <c r="E4" s="6" t="str">
+      <c r="E4" s="5" t="str">
         <v>8</v>
       </c>
-      <c r="F4" s="6" t="str">
+      <c r="F4" s="5" t="str">
         <v>7</v>
       </c>
-      <c r="G4" s="6" t="str">
+      <c r="G4" s="5" t="str">
         <v>26</v>
       </c>
-      <c r="H4" s="6" t="str">
+      <c r="H4" s="5" t="str">
         <v>200</v>
       </c>
-      <c r="I4" s="6" t="str">
+      <c r="I4" s="5" t="str">
         <v>200</v>
       </c>
-      <c r="J4" s="6" t="str">
+      <c r="J4" s="5" t="str">
         <v>9</v>
       </c>
     </row>
@@ -1059,13 +1036,13 @@
       <c r="B9" s="3" t="str">
         <v>TA</v>
       </c>
-      <c r="C9" s="7" t="str">
+      <c r="C9" s="6" t="str">
         <v>ZAN_HIGH</v>
       </c>
-      <c r="D9" s="8" t="str">
+      <c r="D9" s="6" t="str">
         <v>Zanomaline High Dose (81 mg)</v>
       </c>
-      <c r="E9" s="8" t="str">
+      <c r="E9" s="6" t="str">
         <v>1</v>
       </c>
       <c r="F9" s="3" t="str">
@@ -1091,13 +1068,13 @@
       <c r="B10" s="3" t="str">
         <v>TA</v>
       </c>
-      <c r="C10" s="8" t="str">
+      <c r="C10" s="6" t="str">
         <v>ZAN_HIGH</v>
       </c>
-      <c r="D10" s="8" t="str">
+      <c r="D10" s="6" t="str">
         <v>Zanomaline High Dose (81 mg)</v>
       </c>
-      <c r="E10" s="8" t="str">
+      <c r="E10" s="6" t="str">
         <v>3</v>
       </c>
       <c r="F10" s="3" t="str">
@@ -1123,13 +1100,13 @@
       <c r="B11" s="3" t="str">
         <v>TA</v>
       </c>
-      <c r="C11" s="8" t="str">
+      <c r="C11" s="6" t="str">
         <v>ZAN_HIGH</v>
       </c>
-      <c r="D11" s="8" t="str">
+      <c r="D11" s="6" t="str">
         <v>Zanomaline High Dose (81 mg)</v>
       </c>
-      <c r="E11" s="8" t="str">
+      <c r="E11" s="6" t="str">
         <v>2</v>
       </c>
       <c r="F11" s="3" t="str">
@@ -1155,13 +1132,13 @@
       <c r="B12" s="3" t="str">
         <v>TA</v>
       </c>
-      <c r="C12" s="8" t="str">
+      <c r="C12" s="6" t="str">
         <v>ZAN_HIGH</v>
       </c>
-      <c r="D12" s="8" t="str">
+      <c r="D12" s="6" t="str">
         <v>Zanomaline High Dose (81 mg)</v>
       </c>
-      <c r="E12" s="8" t="str">
+      <c r="E12" s="6" t="str">
         <v>4</v>
       </c>
       <c r="F12" s="3" t="str">

</xml_diff>

<commit_message>
better negative test cases + grammar in rule description + output var testcd
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Library" sheetId="1" r:id="rId1"/>
     <sheet name="Datasets" sheetId="2" r:id="rId2"/>
     <sheet name="Validation" sheetId="3" r:id="rId3"/>
-    <sheet name="ie.xpt" sheetId="4" r:id="rId4"/>
+    <sheet name="lb.xpt" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -57,8 +57,7 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <b/>
-      <color rgb="FF000000"/>
+      <i/>
     </font>
     <font>
       <sz val="11"/>
@@ -68,10 +67,17 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FF000000"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -85,6 +91,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -114,15 +138,17 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -493,10 +519,10 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="str">
-        <v>ie.xpt</v>
+        <v>lb.xpt</v>
       </c>
       <c r="B2" s="3" t="str">
-        <v>Inclusion Exclusion</v>
+        <v>Laboratory</v>
       </c>
     </row>
   </sheetData>
@@ -508,7 +534,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F10"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="str">
@@ -535,7 +561,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="str">
-        <v>ie.xpt</v>
+        <v>lb.xpt</v>
       </c>
       <c r="C2" s="3" t="str">
         <v>Record</v>
@@ -544,22 +570,182 @@
         <v>5</v>
       </c>
       <c r="E2" s="3" t="str">
-        <v>IELOINC</v>
+        <v>LBLOINC</v>
       </c>
       <c r="F2" s="3" t="str">
+        <v>999999-9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="str">
+        <v>lb.xpt</v>
+      </c>
+      <c r="C3" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D3" s="3">
+        <v>5</v>
+      </c>
+      <c r="E3" s="3" t="str">
+        <v>LBTESTCD</v>
+      </c>
+      <c r="F3" s="3" t="str">
+        <v>ALB</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="str">
+        <v>lb.xpt</v>
+      </c>
+      <c r="C4" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D4" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E4" s="3" t="str">
+        <v>$define_loinc_version</v>
+      </c>
+      <c r="F4" s="3">
+        <v>2.74</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="str">
+        <v>lb.xpt</v>
+      </c>
+      <c r="C5" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D5" s="3">
+        <v>6</v>
+      </c>
+      <c r="E5" s="3" t="str">
+        <v>LBLOINC</v>
+      </c>
+      <c r="F5" s="3" t="str">
+        <v>Health informatics pioneer and the father of LOINC</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="str">
+        <v>lb.xpt</v>
+      </c>
+      <c r="C6" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D6" s="3">
+        <v>6</v>
+      </c>
+      <c r="E6" s="3" t="str">
+        <v>LBTESTCD</v>
+      </c>
+      <c r="F6" s="3" t="str">
+        <v>ALP</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>2</v>
+      </c>
+      <c r="B7" s="3" t="str">
+        <v>lb.xpt</v>
+      </c>
+      <c r="C7" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D7" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E7" s="3" t="str">
+        <v>$define_loinc_version</v>
+      </c>
+      <c r="F7" s="3">
+        <v>2.74</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3" t="str">
+        <v>lb.xpt</v>
+      </c>
+      <c r="C8" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D8" s="2">
+        <v>7</v>
+      </c>
+      <c r="E8" s="3" t="str">
+        <v>LBLOINC</v>
+      </c>
+      <c r="F8" s="3" t="str">
         <v>100002-5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <v>3</v>
+      </c>
+      <c r="B9" s="3" t="str">
+        <v>lb.xpt</v>
+      </c>
+      <c r="C9" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D9" s="2">
+        <v>7</v>
+      </c>
+      <c r="E9" s="3" t="str">
+        <v>LBTESTCD</v>
+      </c>
+      <c r="F9" s="3" t="str">
+        <v>ALT</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2">
+        <v>3</v>
+      </c>
+      <c r="B10" s="3" t="str">
+        <v>lb.xpt</v>
+      </c>
+      <c r="C10" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D10" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E10" s="3" t="str">
+        <v>$define_loinc_version</v>
+      </c>
+      <c r="F10" s="3">
+        <v>2.74</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:Y7"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="str">
@@ -572,38 +758,74 @@
         <v>USUBJID</v>
       </c>
       <c r="D1" s="4" t="str">
-        <v>IESEQ</v>
+        <v>LBSEQ</v>
       </c>
       <c r="E1" s="4" t="str">
-        <v>IETESTCD</v>
+        <v>LBTESTCD</v>
       </c>
       <c r="F1" s="4" t="str">
-        <v>IETEST</v>
+        <v>LBTEST</v>
       </c>
       <c r="G1" s="4" t="str">
-        <v>IECAT</v>
+        <v>LBCAT</v>
       </c>
       <c r="H1" s="4" t="str">
-        <v>IEORRES</v>
+        <v>LBORRES</v>
       </c>
       <c r="I1" s="4" t="str">
-        <v>IESTRESC</v>
+        <v>LBORRESU</v>
       </c>
       <c r="J1" s="4" t="str">
+        <v>LBORNRLO</v>
+      </c>
+      <c r="K1" s="4" t="str">
+        <v>LBORNRHI</v>
+      </c>
+      <c r="L1" s="4" t="str">
+        <v>LBSTRESC</v>
+      </c>
+      <c r="M1" s="4" t="str">
+        <v>LBSTRESN</v>
+      </c>
+      <c r="N1" s="4" t="str">
+        <v>LBSTRESU</v>
+      </c>
+      <c r="O1" s="4" t="str">
+        <v>LBSTNRLO</v>
+      </c>
+      <c r="P1" s="4" t="str">
+        <v>LBSTNRHI</v>
+      </c>
+      <c r="Q1" s="4" t="str">
+        <v>LBNRIND</v>
+      </c>
+      <c r="R1" s="4" t="str">
+        <v>LBLOBXFL</v>
+      </c>
+      <c r="S1" s="4" t="str">
+        <v>LBDRVFL</v>
+      </c>
+      <c r="T1" s="4" t="str">
+        <v>VISITNUM</v>
+      </c>
+      <c r="U1" s="4" t="str">
+        <v>VISIT</v>
+      </c>
+      <c r="V1" s="4" t="str">
         <v>EPOCH</v>
       </c>
-      <c r="K1" s="4" t="str">
-        <v>IEDTC</v>
-      </c>
-      <c r="L1" s="4" t="str">
-        <v>IEDY</v>
-      </c>
-      <c r="M1" s="5" t="str">
-        <v>IELOINC</v>
+      <c r="W1" s="4" t="str">
+        <v>LBDTC</v>
+      </c>
+      <c r="X1" s="4" t="str">
+        <v>LBDY</v>
+      </c>
+      <c r="Y1" s="4" t="str">
+        <v>LBLOINC</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
       <c r="B2" s="6" t="str">
@@ -616,30 +838,66 @@
         <v>Sequence Number</v>
       </c>
       <c r="E2" s="6" t="str">
-        <v>Inclusion/Exclusion Criterion Short Name</v>
+        <v>Lab Test or Examination Short Name</v>
       </c>
       <c r="F2" s="6" t="str">
-        <v>Inclusion/Exclusion Criterion</v>
+        <v>Lab Test or Examination Name</v>
       </c>
       <c r="G2" s="6" t="str">
-        <v>Inclusion/Exclusion Category</v>
+        <v>Category for Lab Test</v>
       </c>
       <c r="H2" s="6" t="str">
-        <v>I/E Criterion Original Result</v>
+        <v>Result or Finding in Original Units</v>
       </c>
       <c r="I2" s="6" t="str">
-        <v>I/E Criterion Result in Std Format</v>
+        <v>Original Units</v>
       </c>
       <c r="J2" s="6" t="str">
+        <v>Reference Range Lower Limit in Orig Unit</v>
+      </c>
+      <c r="K2" s="6" t="str">
+        <v>Reference Range Upper Limit in Orig Unit</v>
+      </c>
+      <c r="L2" s="6" t="str">
+        <v>Character Result/Finding in Std Format</v>
+      </c>
+      <c r="M2" s="6" t="str">
+        <v>Numeric Result/Finding in Standard Units</v>
+      </c>
+      <c r="N2" s="6" t="str">
+        <v>Standard Units</v>
+      </c>
+      <c r="O2" s="6" t="str">
+        <v>Reference Range Lower Limit-Std Units</v>
+      </c>
+      <c r="P2" s="6" t="str">
+        <v>Reference Range Upper Limit-Std Units</v>
+      </c>
+      <c r="Q2" s="6" t="str">
+        <v>Reference Range Indicator</v>
+      </c>
+      <c r="R2" s="6" t="str">
+        <v>Last Observation Before Exposure Flag</v>
+      </c>
+      <c r="S2" s="6" t="str">
+        <v>Derived Flag</v>
+      </c>
+      <c r="T2" s="6" t="str">
+        <v>Visit Number</v>
+      </c>
+      <c r="U2" s="6" t="str">
+        <v>Visit Name</v>
+      </c>
+      <c r="V2" s="6" t="str">
         <v>Epoch</v>
       </c>
-      <c r="K2" s="6" t="str">
-        <v>Date/Time of Collection</v>
-      </c>
-      <c r="L2" s="6" t="str">
-        <v>Study Day of Collection</v>
-      </c>
-      <c r="M2" s="6" t="str">
+      <c r="W2" s="6" t="str">
+        <v>Date/Time of Specimen Collection</v>
+      </c>
+      <c r="X2" s="6" t="str">
+        <v>Study Day of Specimen Collection</v>
+      </c>
+      <c r="Y2" s="6" t="str">
         <v>LOINC Code</v>
       </c>
     </row>
@@ -678,9 +936,45 @@
         <v>Char</v>
       </c>
       <c r="L3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="M3" s="6" t="str">
+      <c r="N3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="O3" s="6" t="str">
+        <v>Num</v>
+      </c>
+      <c r="P3" s="6" t="str">
+        <v>Num</v>
+      </c>
+      <c r="Q3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="R3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="S3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="T3" s="6" t="str">
+        <v>Num</v>
+      </c>
+      <c r="U3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="V3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="W3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="X3" s="6" t="str">
+        <v>Num</v>
+      </c>
+      <c r="Y3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
@@ -701,27 +995,63 @@
         <v>7</v>
       </c>
       <c r="F4" s="6">
-        <v>196</v>
+        <v>39</v>
       </c>
       <c r="G4" s="6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H4" s="6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I4" s="6">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J4" s="6">
-        <v>9</v>
+        <v>200</v>
       </c>
       <c r="K4" s="6">
-        <v>10</v>
+        <v>200</v>
       </c>
       <c r="L4" s="6">
         <v>8</v>
       </c>
       <c r="M4" s="6">
+        <v>8</v>
+      </c>
+      <c r="N4" s="6">
+        <v>7</v>
+      </c>
+      <c r="O4" s="6">
+        <v>8</v>
+      </c>
+      <c r="P4" s="6">
+        <v>8</v>
+      </c>
+      <c r="Q4" s="6">
+        <v>8</v>
+      </c>
+      <c r="R4" s="6">
+        <v>1</v>
+      </c>
+      <c r="S4" s="6">
+        <v>10</v>
+      </c>
+      <c r="T4" s="6">
+        <v>8</v>
+      </c>
+      <c r="U4" s="6">
+        <v>200</v>
+      </c>
+      <c r="V4" s="6">
+        <v>9</v>
+      </c>
+      <c r="W4" s="6">
+        <v>19</v>
+      </c>
+      <c r="X4" s="6">
+        <v>8</v>
+      </c>
+      <c r="Y4" s="6">
         <v>8</v>
       </c>
     </row>
@@ -730,45 +1060,235 @@
         <v>CDISCPILOT01</v>
       </c>
       <c r="B5" s="3" t="str">
-        <v>IE</v>
+        <v>LB</v>
       </c>
       <c r="C5" s="3" t="str">
-        <v>CDISC01</v>
+        <v>CDISC001</v>
       </c>
       <c r="D5" s="3">
         <v>1</v>
       </c>
-      <c r="E5" s="3" t="str">
-        <v>INCL01</v>
+      <c r="E5" s="7" t="str">
+        <v>ALB</v>
       </c>
       <c r="F5" s="3" t="str">
-        <v>Is not pregnant or nursing.</v>
+        <v>Albumin</v>
       </c>
       <c r="G5" s="3" t="str">
-        <v>INCLUSION</v>
+        <v>CHEMISTRY</v>
       </c>
       <c r="H5" s="3" t="str">
+        <v>3.9</v>
+      </c>
+      <c r="I5" s="3" t="str">
+        <v>g/dL</v>
+      </c>
+      <c r="J5" s="3" t="str">
+        <v>3.5</v>
+      </c>
+      <c r="K5" s="3" t="str">
+        <v>4.6</v>
+      </c>
+      <c r="L5" s="3" t="str">
+        <v>39</v>
+      </c>
+      <c r="M5" s="3">
+        <v>39</v>
+      </c>
+      <c r="N5" s="3" t="str">
+        <v>g/L</v>
+      </c>
+      <c r="O5" s="3">
+        <v>35</v>
+      </c>
+      <c r="P5" s="3">
+        <v>46</v>
+      </c>
+      <c r="Q5" s="3" t="str">
+        <v>NORMAL</v>
+      </c>
+      <c r="R5" s="3" t="str">
         <v>Y</v>
       </c>
-      <c r="I5" s="3" t="str">
+      <c r="S5" s="2" t="str">
+        <v/>
+      </c>
+      <c r="T5" s="3">
+        <v>1</v>
+      </c>
+      <c r="U5" s="3" t="str">
+        <v>SCREENING 1</v>
+      </c>
+      <c r="V5" s="3" t="str">
+        <v>SCREENING</v>
+      </c>
+      <c r="W5" s="3" t="str">
+        <v>2012-11-23T11:20</v>
+      </c>
+      <c r="X5" s="3">
+        <v>-7</v>
+      </c>
+      <c r="Y5" s="8" t="str">
+        <v>999999-9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B6" s="3" t="str">
+        <v>LB</v>
+      </c>
+      <c r="C6" s="3" t="str">
+        <v>CDISC001</v>
+      </c>
+      <c r="D6" s="3">
+        <v>2</v>
+      </c>
+      <c r="E6" s="7" t="str">
+        <v>ALP</v>
+      </c>
+      <c r="F6" s="3" t="str">
+        <v>Alkaline Phosphatase</v>
+      </c>
+      <c r="G6" s="3" t="str">
+        <v>CHEMISTRY</v>
+      </c>
+      <c r="H6" s="3" t="str">
+        <v>93</v>
+      </c>
+      <c r="I6" s="3" t="str">
+        <v>U/L</v>
+      </c>
+      <c r="J6" s="3" t="str">
+        <v>35</v>
+      </c>
+      <c r="K6" s="3" t="str">
+        <v>115</v>
+      </c>
+      <c r="L6" s="3" t="str">
+        <v>93</v>
+      </c>
+      <c r="M6" s="3">
+        <v>93</v>
+      </c>
+      <c r="N6" s="3" t="str">
+        <v>U/L</v>
+      </c>
+      <c r="O6" s="3">
+        <v>35</v>
+      </c>
+      <c r="P6" s="3">
+        <v>115</v>
+      </c>
+      <c r="Q6" s="3" t="str">
+        <v>NORMAL</v>
+      </c>
+      <c r="R6" s="3" t="str">
         <v>Y</v>
       </c>
-      <c r="J5" s="3" t="str">
+      <c r="S6" s="3" t="str">
+        <v/>
+      </c>
+      <c r="T6" s="3">
+        <v>1</v>
+      </c>
+      <c r="U6" s="3" t="str">
+        <v>SCREENING 1</v>
+      </c>
+      <c r="V6" s="3" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="K5" s="3" t="str">
-        <v>2014-03-17</v>
-      </c>
-      <c r="L5" s="3" t="str">
+      <c r="W6" s="3" t="str">
+        <v>2012-11-23T11:20</v>
+      </c>
+      <c r="X6" s="3">
+        <v>-7</v>
+      </c>
+      <c r="Y6" s="9" t="str">
+        <v>Health informatics pioneer and the father of LOINC</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B7" s="3" t="str">
+        <v>LB</v>
+      </c>
+      <c r="C7" s="3" t="str">
+        <v>CDISC001</v>
+      </c>
+      <c r="D7" s="3">
+        <v>3</v>
+      </c>
+      <c r="E7" s="7" t="str">
+        <v>ALT</v>
+      </c>
+      <c r="F7" s="3" t="str">
+        <v>Alanine Aminotransferase</v>
+      </c>
+      <c r="G7" s="3" t="str">
+        <v>CHEMISTRY</v>
+      </c>
+      <c r="H7" s="3" t="str">
         <v/>
       </c>
-      <c r="M5" s="7" t="str">
+      <c r="I7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="J7" s="3" t="str">
+        <v>6</v>
+      </c>
+      <c r="K7" s="3" t="str">
+        <v>35</v>
+      </c>
+      <c r="L7" s="3" t="str">
+        <v>18</v>
+      </c>
+      <c r="M7" s="3">
+        <v>18</v>
+      </c>
+      <c r="N7" s="3" t="str">
+        <v>U/L</v>
+      </c>
+      <c r="O7" s="3">
+        <v>6</v>
+      </c>
+      <c r="P7" s="3">
+        <v>35</v>
+      </c>
+      <c r="Q7" s="3" t="str">
+        <v>NORMAL</v>
+      </c>
+      <c r="R7" s="3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="S7" s="3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="T7" s="3">
+        <v>1</v>
+      </c>
+      <c r="U7" s="3" t="str">
+        <v>SCREENING 1</v>
+      </c>
+      <c r="V7" s="3" t="str">
+        <v>SCREENING</v>
+      </c>
+      <c r="W7" s="3" t="str">
+        <v>2012-11-23T11:20</v>
+      </c>
+      <c r="X7" s="3">
+        <v>-7</v>
+      </c>
+      <c r="Y7" s="9" t="str">
         <v>100002-5</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add PPTEST to output
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -36,7 +36,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -63,8 +67,12 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -84,6 +92,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -113,14 +127,16 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -455,26 +471,26 @@
   <dimension ref="A1:B3"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
+      <c r="A1" s="3" t="str">
         <v>Product</v>
       </c>
-      <c r="B1" s="2" t="str">
+      <c r="B1" s="3" t="str">
         <v>Version</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="3" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="3" t="str">
         <v>3-4</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="3" t="str">
         <v>sdtmct</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="3" t="str">
         <v>2025-03-28</v>
       </c>
     </row>
@@ -490,18 +506,18 @@
   <dimension ref="A1:B2"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
+      <c r="A1" s="3" t="str">
         <v>Filename</v>
       </c>
-      <c r="B1" s="2" t="str">
+      <c r="B1" s="3" t="str">
         <v>Label</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="3" t="str">
         <v>pp.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="3" t="str">
         <v>Pharmacokinetics Parameters</v>
       </c>
     </row>
@@ -514,25 +530,25 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
+      <c r="A1" s="3" t="str">
         <v>Error group</v>
       </c>
-      <c r="B1" s="2" t="str">
+      <c r="B1" s="3" t="str">
         <v>Sheet</v>
       </c>
-      <c r="C1" s="2" t="str">
+      <c r="C1" s="3" t="str">
         <v>Error level</v>
       </c>
-      <c r="D1" s="2" t="str">
+      <c r="D1" s="3" t="str">
         <v>Row num</v>
       </c>
-      <c r="E1" s="2" t="str">
+      <c r="E1" s="3" t="str">
         <v>Variable</v>
       </c>
-      <c r="F1" s="2" t="str">
+      <c r="F1" s="3" t="str">
         <v>Error value</v>
       </c>
     </row>
@@ -556,9 +572,29 @@
         <v>pgEq/mL</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="str">
+        <v>pp.xpt</v>
+      </c>
+      <c r="C3" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D3" s="3">
+        <v>5</v>
+      </c>
+      <c r="E3" s="3" t="str">
+        <v>PPTEST</v>
+      </c>
+      <c r="F3" s="3" t="str">
+        <v>AURC Infinity Obs Norm by Dose</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -568,237 +604,237 @@
   <dimension ref="A1:O5"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="str">
+      <c r="A1" s="4" t="str">
         <v>STUDYID</v>
       </c>
-      <c r="B1" s="3" t="str">
+      <c r="B1" s="4" t="str">
         <v>DOMAIN</v>
       </c>
-      <c r="C1" s="3" t="str">
+      <c r="C1" s="4" t="str">
         <v>USUBJID</v>
       </c>
-      <c r="D1" s="3" t="str">
+      <c r="D1" s="4" t="str">
         <v>PPSEQ</v>
       </c>
-      <c r="E1" s="3" t="str">
+      <c r="E1" s="4" t="str">
         <v>PPGRPID</v>
       </c>
-      <c r="F1" s="3" t="str">
+      <c r="F1" s="4" t="str">
         <v>PPTESTCD</v>
       </c>
-      <c r="G1" s="3" t="str">
+      <c r="G1" s="4" t="str">
         <v>PPTEST</v>
       </c>
-      <c r="H1" s="3" t="str">
+      <c r="H1" s="4" t="str">
         <v>PPCAT</v>
       </c>
-      <c r="I1" s="3" t="str">
+      <c r="I1" s="4" t="str">
         <v>PPORRES</v>
       </c>
-      <c r="J1" s="3" t="str">
+      <c r="J1" s="4" t="str">
         <v>PPORRESU</v>
       </c>
-      <c r="K1" s="3" t="str">
+      <c r="K1" s="4" t="str">
         <v>PPSTRESC</v>
       </c>
-      <c r="L1" s="3" t="str">
+      <c r="L1" s="4" t="str">
         <v>PPSTRESN</v>
       </c>
-      <c r="M1" s="3" t="str">
+      <c r="M1" s="4" t="str">
         <v>PPSTRESU</v>
       </c>
-      <c r="N1" s="3" t="str">
+      <c r="N1" s="4" t="str">
         <v>PPSPEC</v>
       </c>
-      <c r="O1" s="3" t="str">
+      <c r="O1" s="4" t="str">
         <v>PPRFTDTC</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="4" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="4" t="str">
+      <c r="D2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="4" t="str">
+      <c r="E2" s="5" t="str">
         <v>Group ID</v>
       </c>
-      <c r="F2" s="4" t="str">
+      <c r="F2" s="5" t="str">
         <v>Parameter Short Name</v>
       </c>
-      <c r="G2" s="4" t="str">
+      <c r="G2" s="5" t="str">
         <v>Parameter Name</v>
       </c>
-      <c r="H2" s="4" t="str">
+      <c r="H2" s="5" t="str">
         <v>Parameter Category</v>
       </c>
-      <c r="I2" s="4" t="str">
+      <c r="I2" s="5" t="str">
         <v>Result or Finding in Original Units</v>
       </c>
-      <c r="J2" s="4" t="str">
+      <c r="J2" s="5" t="str">
         <v>Original Units</v>
       </c>
-      <c r="K2" s="4" t="str">
+      <c r="K2" s="5" t="str">
         <v>Character Result/Finding in Std Format</v>
       </c>
-      <c r="L2" s="4" t="str">
+      <c r="L2" s="5" t="str">
         <v>Numeric Result/Finding in Standard Units</v>
       </c>
-      <c r="M2" s="4" t="str">
+      <c r="M2" s="5" t="str">
         <v>Standard Units</v>
       </c>
-      <c r="N2" s="4" t="str">
+      <c r="N2" s="5" t="str">
         <v>Specimen Material Type</v>
       </c>
-      <c r="O2" s="4" t="str">
+      <c r="O2" s="5" t="str">
         <v>Date/Time of Reference Point</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="4" t="str">
+      <c r="A3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="4" t="str">
+      <c r="E3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="M3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="N3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="O3" s="4" t="str">
+      <c r="M3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="N3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="O3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="str">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="str">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4" t="str">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4" t="str">
+      <c r="A4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5" t="str">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="str">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4" t="str">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4" t="str">
-        <v>50</v>
-      </c>
-      <c r="H4" s="4" t="str">
-        <v>50</v>
-      </c>
-      <c r="I4" s="4" t="str">
-        <v>50</v>
-      </c>
-      <c r="J4" s="4" t="str">
-        <v>50</v>
-      </c>
-      <c r="K4" s="4" t="str">
-        <v>50</v>
-      </c>
-      <c r="L4" s="4" t="str">
+      <c r="E4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="G4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="H4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="I4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="J4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="K4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="L4" s="5" t="str">
         <v>8</v>
       </c>
-      <c r="M4" s="4" t="str">
-        <v>50</v>
-      </c>
-      <c r="N4" s="4" t="str">
-        <v>50</v>
-      </c>
-      <c r="O4" s="4" t="str">
+      <c r="M4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="N4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="O4" s="5" t="str">
         <v>50</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="str">
+      <c r="A5" s="6" t="str">
         <v>Sample001</v>
       </c>
-      <c r="B5" s="5" t="str">
+      <c r="B5" s="6" t="str">
         <v>PP</v>
       </c>
-      <c r="C5" s="5" t="str">
+      <c r="C5" s="6" t="str">
         <v>01-004</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="6">
         <v>1</v>
       </c>
-      <c r="E5" s="5" t="str">
+      <c r="E5" s="6" t="str">
         <v>Part A Period 1</v>
       </c>
-      <c r="F5" s="5" t="str">
+      <c r="F5" s="6" t="str">
         <v>AUCIFP</v>
       </c>
-      <c r="G5" s="5" t="str">
+      <c r="G5" s="7" t="str">
         <v>AURC Infinity Obs Norm by Dose</v>
       </c>
-      <c r="H5" s="5" t="str">
+      <c r="H5" s="6" t="str">
         <v>PPCAT01</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="6">
         <v>1194.546</v>
       </c>
-      <c r="J5" s="6" t="str">
+      <c r="J5" s="8" t="str">
         <v>pgEq/mL</v>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="6">
         <v>1195</v>
       </c>
-      <c r="L5" s="5">
+      <c r="L5" s="6">
         <v>1195</v>
       </c>
-      <c r="M5" s="5" t="str">
+      <c r="M5" s="6" t="str">
         <v>pgEq/mL</v>
       </c>
-      <c r="N5" s="5" t="str">
+      <c r="N5" s="6" t="str">
         <v>PLASMA</v>
       </c>
-      <c r="O5" s="5" t="str">
+      <c r="O5" s="6" t="str">
         <v>2018-04-09T09:05</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update test data and add version
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -62,7 +62,6 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <i/>
     </font>
     <font>
       <sz val="11"/>
@@ -88,7 +87,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -624,104 +623,104 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="5" t="str">
         <v>Group ID</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Trial Summary Parameter Short Name</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="5" t="str">
         <v>Trial Summary Parameter</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="5" t="str">
         <v>Parameter Value</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="5" t="str">
         <v>Parameter Null Flavor</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="5" t="str">
         <v>Parameter Value Code</v>
       </c>
-      <c r="J2" s="6" t="str">
+      <c r="J2" s="5" t="str">
         <v>Name of the Reference Terminology</v>
       </c>
-      <c r="K2" s="6" t="str">
+      <c r="K2" s="5" t="str">
         <v>Version of the Reference Terminology</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
+      <c r="A3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="D3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="6" t="str">
+      <c r="D3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
+      <c r="A4" s="5">
         <v>10</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>8</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <v>5</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>8</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <v>40</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="5">
         <v>149</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="5">
         <v>2</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="5">
         <v>11</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="5">
         <v>18</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="5">
         <v>10</v>
       </c>
     </row>
@@ -738,7 +737,7 @@
       <c r="D5" s="4" t="str">
         <v/>
       </c>
-      <c r="E5" s="7" t="str">
+      <c r="E5" s="6" t="str">
         <v>TRT</v>
       </c>
       <c r="F5" s="4" t="str">
@@ -747,10 +746,10 @@
       <c r="G5" s="4" t="str">
         <v>UNIITERM1</v>
       </c>
-      <c r="H5" s="2" t="str">
+      <c r="H5" s="4" t="str">
         <v/>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="7">
         <v>9999999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix test cases and add version
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -62,7 +62,6 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <i/>
     </font>
     <font>
       <sz val="11"/>
@@ -88,7 +87,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -624,104 +623,104 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="5" t="str">
         <v>Group ID</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Trial Summary Parameter Short Name</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="5" t="str">
         <v>Trial Summary Parameter</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="5" t="str">
         <v>Parameter Value</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="5" t="str">
         <v>Parameter Null Flavor</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="5" t="str">
         <v>Parameter Value Code</v>
       </c>
-      <c r="J2" s="6" t="str">
+      <c r="J2" s="5" t="str">
         <v>Name of the Reference Terminology</v>
       </c>
-      <c r="K2" s="6" t="str">
+      <c r="K2" s="5" t="str">
         <v>Version of the Reference Terminology</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
+      <c r="A3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="D3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="6" t="str">
+      <c r="D3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
+      <c r="A4" s="5">
         <v>10</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>8</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <v>5</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>8</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <v>40</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="5">
         <v>149</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="5">
         <v>2</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="5">
         <v>11</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="5">
         <v>18</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="5">
         <v>10</v>
       </c>
     </row>
@@ -738,7 +737,7 @@
       <c r="D5" s="4" t="str">
         <v/>
       </c>
-      <c r="E5" s="7" t="str">
+      <c r="E5" s="6" t="str">
         <v>COMPTRT</v>
       </c>
       <c r="F5" s="4" t="str">
@@ -747,10 +746,10 @@
       <c r="G5" s="4" t="str">
         <v>UNIITERM1</v>
       </c>
-      <c r="H5" s="2" t="str">
+      <c r="H5" s="4" t="str">
         <v/>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="7">
         <v>9999999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
strict incremental sort adjustments
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9206F61-F54D-8E4B-BADE-47538BB29F00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F6D775A-84C4-CD41-BFB1-593B47365942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-8560" windowWidth="51200" windowHeight="28200" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="86">
   <si>
     <t>Product</t>
   </si>
@@ -249,6 +249,39 @@
   </si>
   <si>
     <t>Record</t>
+  </si>
+  <si>
+    <t>HYPO1</t>
+  </si>
+  <si>
+    <t>HYPO3</t>
+  </si>
+  <si>
+    <t>HYPO</t>
+  </si>
+  <si>
+    <t>2008-01-01</t>
+  </si>
+  <si>
+    <t>2008-01-02</t>
+  </si>
+  <si>
+    <t>2008-01-03</t>
+  </si>
+  <si>
+    <t>005</t>
+  </si>
+  <si>
+    <t>HYPOGLYCEMIC EVENT</t>
+  </si>
+  <si>
+    <t>Occurrence of a hypoglycemic event</t>
+  </si>
+  <si>
+    <t>006</t>
+  </si>
+  <si>
+    <t>HYPO2</t>
   </si>
 </sst>
 </file>
@@ -319,7 +352,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -334,6 +367,15 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -698,7 +740,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -812,13 +854,13 @@
         <v>74</v>
       </c>
       <c r="D6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E6" t="s">
         <v>20</v>
       </c>
       <c r="F6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -832,7 +874,7 @@
         <v>74</v>
       </c>
       <c r="D7">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E7" t="s">
         <v>21</v>
@@ -872,13 +914,13 @@
         <v>74</v>
       </c>
       <c r="D9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E9" t="s">
         <v>22</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -892,13 +934,13 @@
         <v>74</v>
       </c>
       <c r="D10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E10" t="s">
         <v>20</v>
       </c>
       <c r="F10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -912,7 +954,7 @@
         <v>74</v>
       </c>
       <c r="D11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E11" t="s">
         <v>21</v>
@@ -952,13 +994,13 @@
         <v>74</v>
       </c>
       <c r="D13">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E13" t="s">
         <v>22</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -1132,13 +1174,13 @@
         <v>74</v>
       </c>
       <c r="D22">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E22" t="s">
         <v>20</v>
       </c>
       <c r="F22" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -1152,7 +1194,7 @@
         <v>74</v>
       </c>
       <c r="D23">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E23" t="s">
         <v>21</v>
@@ -1192,13 +1234,13 @@
         <v>74</v>
       </c>
       <c r="D25">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E25" t="s">
         <v>22</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -1212,13 +1254,13 @@
         <v>74</v>
       </c>
       <c r="D26">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E26" t="s">
         <v>20</v>
       </c>
       <c r="F26" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
@@ -1232,7 +1274,7 @@
         <v>74</v>
       </c>
       <c r="D27">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E27" t="s">
         <v>21</v>
@@ -1272,13 +1314,13 @@
         <v>74</v>
       </c>
       <c r="D29">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E29" t="s">
         <v>22</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
@@ -1292,13 +1334,13 @@
         <v>74</v>
       </c>
       <c r="D30">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E30" t="s">
         <v>20</v>
       </c>
       <c r="F30" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
@@ -1312,7 +1354,7 @@
         <v>74</v>
       </c>
       <c r="D31">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E31" t="s">
         <v>21</v>
@@ -1352,13 +1394,13 @@
         <v>74</v>
       </c>
       <c r="D33">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E33" t="s">
         <v>22</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
@@ -1372,13 +1414,13 @@
         <v>74</v>
       </c>
       <c r="D34">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E34" t="s">
         <v>20</v>
       </c>
       <c r="F34" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
@@ -1392,13 +1434,13 @@
         <v>74</v>
       </c>
       <c r="D35">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E35" t="s">
         <v>21</v>
       </c>
       <c r="F35" t="s">
-        <v>45</v>
+        <v>82</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -1412,7 +1454,7 @@
         <v>74</v>
       </c>
       <c r="D36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E36" t="s">
         <v>41</v>
@@ -1432,13 +1474,173 @@
         <v>74</v>
       </c>
       <c r="D37">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E37" t="s">
         <v>22</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>73</v>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>10</v>
+      </c>
+      <c r="B38" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38" t="s">
+        <v>74</v>
+      </c>
+      <c r="D38">
+        <v>19</v>
+      </c>
+      <c r="E38" t="s">
+        <v>20</v>
+      </c>
+      <c r="F38" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>10</v>
+      </c>
+      <c r="B39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" t="s">
+        <v>74</v>
+      </c>
+      <c r="D39">
+        <v>19</v>
+      </c>
+      <c r="E39" t="s">
+        <v>21</v>
+      </c>
+      <c r="F39" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>10</v>
+      </c>
+      <c r="B40" t="s">
+        <v>14</v>
+      </c>
+      <c r="C40" t="s">
+        <v>74</v>
+      </c>
+      <c r="D40">
+        <v>6</v>
+      </c>
+      <c r="E40" t="s">
+        <v>41</v>
+      </c>
+      <c r="F40" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>10</v>
+      </c>
+      <c r="B41" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" t="s">
+        <v>74</v>
+      </c>
+      <c r="D41">
+        <v>19</v>
+      </c>
+      <c r="E41" t="s">
+        <v>22</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>11</v>
+      </c>
+      <c r="B42" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" t="s">
+        <v>74</v>
+      </c>
+      <c r="D42">
+        <v>21</v>
+      </c>
+      <c r="E42" t="s">
+        <v>20</v>
+      </c>
+      <c r="F42" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>11</v>
+      </c>
+      <c r="B43" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" t="s">
+        <v>74</v>
+      </c>
+      <c r="D43">
+        <v>21</v>
+      </c>
+      <c r="E43" t="s">
+        <v>21</v>
+      </c>
+      <c r="F43" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>11</v>
+      </c>
+      <c r="B44" t="s">
+        <v>14</v>
+      </c>
+      <c r="C44" t="s">
+        <v>74</v>
+      </c>
+      <c r="D44">
+        <v>6</v>
+      </c>
+      <c r="E44" t="s">
+        <v>41</v>
+      </c>
+      <c r="F44" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>11</v>
+      </c>
+      <c r="B45" t="s">
+        <v>12</v>
+      </c>
+      <c r="C45" t="s">
+        <v>74</v>
+      </c>
+      <c r="D45">
+        <v>21</v>
+      </c>
+      <c r="E45" t="s">
+        <v>22</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1449,7 +1651,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6491AEE8-38DB-694C-957E-E74E9CCBDB4E}">
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -1639,13 +1841,13 @@
       <c r="D7">
         <v>3</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="6" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1685,13 +1887,13 @@
       <c r="D9">
         <v>5</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" t="s">
         <v>57</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" t="s">
         <v>45</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="4" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1754,13 +1956,13 @@
       <c r="D12">
         <v>6</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" t="s">
         <v>64</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" t="s">
         <v>45</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G12" s="4" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1831,6 +2033,144 @@
       </c>
       <c r="G15" s="6" t="s">
         <v>73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D17">
+        <v>2</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D18">
+        <v>3</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D20">
+        <v>2</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="32" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D21">
+        <v>3</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1841,7 +2181,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{824A2302-6193-3F4E-A78A-27E305DD7F6A}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -1929,7 +2269,25 @@
         <v>47</v>
       </c>
     </row>
+    <row r="6" spans="1:5" ht="64" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
full-run with workgin test cases
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -36,7 +36,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -58,13 +62,14 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <i/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -72,6 +77,12 @@
     </fill>
     <fill>
       <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -107,14 +118,15 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -449,18 +461,18 @@
   <dimension ref="A1:B2"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
+      <c r="A1" s="3" t="str">
         <v>Product</v>
       </c>
-      <c r="B1" s="2" t="str">
+      <c r="B1" s="3" t="str">
         <v>Version</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="3" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="3" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -476,18 +488,18 @@
   <dimension ref="A1:B2"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
+      <c r="A1" s="3" t="str">
         <v>Filename</v>
       </c>
-      <c r="B1" s="2" t="str">
+      <c r="B1" s="3" t="str">
         <v>Label</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="3" t="str">
         <v>ts.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="3" t="str">
         <v>Trial Summary Parameters</v>
       </c>
     </row>
@@ -503,83 +515,83 @@
   <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
+      <c r="A1" s="3" t="str">
         <v>Error group</v>
       </c>
-      <c r="B1" s="2" t="str">
+      <c r="B1" s="3" t="str">
         <v>Sheet</v>
       </c>
-      <c r="C1" s="2" t="str">
+      <c r="C1" s="3" t="str">
         <v>Error level</v>
       </c>
-      <c r="D1" s="2" t="str">
+      <c r="D1" s="3" t="str">
         <v>Row num</v>
       </c>
-      <c r="E1" s="2" t="str">
+      <c r="E1" s="3" t="str">
         <v>Variable</v>
       </c>
-      <c r="F1" s="2" t="str">
+      <c r="F1" s="3" t="str">
         <v>Error value</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="3" t="str">
         <v>ts.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="3" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="3">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="3" t="str">
         <v>TSPARMCD</v>
       </c>
-      <c r="F2" s="2" t="str">
+      <c r="F2" s="3" t="str">
         <v>SSTDTC</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="3" t="str">
         <v>ts.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="3" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="3">
         <v>5</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E3" s="3" t="str">
         <v>TSVAL</v>
       </c>
-      <c r="F3" s="2" t="str">
-        <v>2025-11-01</v>
+      <c r="F3" s="3" t="str">
+        <v>2026-03-02</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
+      <c r="A4" s="3">
         <v>1</v>
       </c>
-      <c r="B4" s="2" t="str">
+      <c r="B4" s="3" t="str">
         <v>ts.xpt</v>
       </c>
-      <c r="C4" s="2" t="str">
+      <c r="C4" s="3" t="str">
         <v>Record</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="3">
         <v>5</v>
       </c>
-      <c r="E4" s="2" t="str">
+      <c r="E4" s="3" t="str">
         <v>$define_meddra_version</v>
       </c>
-      <c r="F4" s="2" t="str">
-        <v>2025-11-01</v>
+      <c r="F4" s="3">
+        <v>28.1</v>
       </c>
     </row>
   </sheetData>
@@ -594,174 +606,174 @@
   <dimension ref="A1:K5"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="str">
+      <c r="A1" s="4" t="str">
         <v>STUDYID</v>
       </c>
-      <c r="B1" s="3" t="str">
+      <c r="B1" s="4" t="str">
         <v>DOMAIN</v>
       </c>
-      <c r="C1" s="3" t="str">
+      <c r="C1" s="4" t="str">
         <v>TSSEQ</v>
       </c>
-      <c r="D1" s="3" t="str">
+      <c r="D1" s="4" t="str">
         <v>TSGRPID</v>
       </c>
-      <c r="E1" s="3" t="str">
+      <c r="E1" s="4" t="str">
         <v>TSPARMCD</v>
       </c>
-      <c r="F1" s="3" t="str">
+      <c r="F1" s="4" t="str">
         <v>TSPARM</v>
       </c>
-      <c r="G1" s="3" t="str">
+      <c r="G1" s="4" t="str">
         <v>TSVAL</v>
       </c>
-      <c r="H1" s="3" t="str">
+      <c r="H1" s="4" t="str">
         <v>TSVALNF</v>
       </c>
-      <c r="I1" s="3" t="str">
+      <c r="I1" s="4" t="str">
         <v>TSVALCD</v>
       </c>
-      <c r="J1" s="3" t="str">
+      <c r="J1" s="4" t="str">
         <v>TSVCDREF</v>
       </c>
-      <c r="K1" s="3" t="str">
+      <c r="K1" s="4" t="str">
         <v>TSVCDVER</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="4" t="str">
+      <c r="C2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="D2" s="4" t="str">
+      <c r="D2" s="5" t="str">
         <v>Group ID</v>
       </c>
-      <c r="E2" s="4" t="str">
+      <c r="E2" s="6" t="str">
         <v>Trial Summary Parameter Short Name</v>
       </c>
-      <c r="F2" s="4" t="str">
+      <c r="F2" s="6" t="str">
         <v>Trial Summary Parameter</v>
       </c>
-      <c r="G2" s="4" t="str">
+      <c r="G2" s="6" t="str">
         <v>Parameter Value</v>
       </c>
-      <c r="H2" s="4" t="str">
+      <c r="H2" s="6" t="str">
         <v>Parameter Null Flavor</v>
       </c>
-      <c r="I2" s="4" t="str">
+      <c r="I2" s="6" t="str">
         <v>Parameter Value Code</v>
       </c>
-      <c r="J2" s="4" t="str">
+      <c r="J2" s="6" t="str">
         <v>Name of the Reference Terminology</v>
       </c>
-      <c r="K2" s="4" t="str">
+      <c r="K2" s="6" t="str">
         <v>Version of the Reference Terminology</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="4" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="D3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="4" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="4" t="str">
+      <c r="D3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4">
+      <c r="A4" s="6">
         <v>12</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="6">
         <v>8</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="6">
         <v>200</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="6">
         <v>8</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="6">
         <v>40</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="6">
         <v>200</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="6">
         <v>4</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="6">
         <v>200</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="6">
         <v>200</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="6">
         <v>200</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="str">
+      <c r="A5" s="3" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="5" t="str">
+      <c r="B5" s="3" t="str">
         <v>TS</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="3">
         <v>1</v>
       </c>
-      <c r="D5" s="2" t="str">
+      <c r="D5" s="3" t="str">
         <v/>
       </c>
-      <c r="E5" s="6" t="str">
+      <c r="E5" s="7" t="str">
         <v>SSTDTC</v>
       </c>
-      <c r="F5" s="5" t="str">
+      <c r="F5" s="3" t="str">
         <v>Study Start Date</v>
       </c>
-      <c r="G5" s="6" t="str">
-        <v>2025-11-01</v>
-      </c>
-      <c r="H5" s="2" t="str">
+      <c r="G5" s="7" t="str">
+        <v>2026-03-02</v>
+      </c>
+      <c r="H5" s="3" t="str">
         <v/>
       </c>
-      <c r="I5" s="2" t="str">
+      <c r="I5" s="3" t="str">
         <v/>
       </c>
-      <c r="J5" s="5" t="str">
+      <c r="J5" s="3" t="str">
         <v>ISO 8601</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add ACTARMCD to output
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5878A1DB-10D8-3E4C-A735-91E47EF53355}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA3FEA3-9DCA-1D45-A690-DEA410116FA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38460" yWindow="-1360" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="137">
   <si>
     <t>Product</t>
   </si>
@@ -578,7 +578,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -605,10 +605,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -623,6 +619,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -987,8 +986,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="5" max="5" width="9.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -1032,7 +1034,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>12</v>
@@ -1041,18 +1043,18 @@
         <v>136</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>12</v>
@@ -1061,7 +1063,7 @@
         <v>136</v>
       </c>
       <c r="D4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E4" t="s">
         <v>28</v>
@@ -1072,7 +1074,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" t="s">
         <v>12</v>
@@ -1081,18 +1083,18 @@
         <v>136</v>
       </c>
       <c r="D5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B6" t="s">
         <v>12</v>
@@ -1101,12 +1103,112 @@
         <v>136</v>
       </c>
       <c r="D6">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E6" t="s">
         <v>28</v>
       </c>
       <c r="F6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>136</v>
+      </c>
+      <c r="D7">
+        <v>7</v>
+      </c>
+      <c r="E7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>136</v>
+      </c>
+      <c r="D8">
+        <v>8</v>
+      </c>
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>136</v>
+      </c>
+      <c r="D9">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>136</v>
+      </c>
+      <c r="D10">
+        <v>9</v>
+      </c>
+      <c r="E10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>136</v>
+      </c>
+      <c r="D11">
+        <v>9</v>
+      </c>
+      <c r="E11" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1125,61 +1227,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="L1" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="14" t="s">
+      <c r="M1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="N1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="14" t="s">
+      <c r="O1" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="14" t="s">
+      <c r="P1" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="14" t="s">
+      <c r="Q1" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="R1" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="S1" s="11" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1367,10 +1469,10 @@
       <c r="B5" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="13">
         <v>76000300003</v>
       </c>
       <c r="E5" s="4" t="s">
@@ -1395,13 +1497,13 @@
       <c r="L5" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="M5" s="16" t="s">
+      <c r="M5" s="14" t="s">
         <v>65</v>
       </c>
       <c r="N5" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="O5" s="5" t="s">
+      <c r="O5" s="14" t="s">
         <v>67</v>
       </c>
       <c r="P5" s="5" t="s">
@@ -1420,10 +1522,10 @@
       <c r="B6" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="13" t="s">
         <v>135</v>
       </c>
       <c r="E6" s="6" t="s">
@@ -1448,13 +1550,13 @@
       <c r="L6" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="M6" s="16" t="s">
+      <c r="M6" s="14" t="s">
         <v>65</v>
       </c>
       <c r="N6" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="O6" s="16" t="s">
         <v>67</v>
       </c>
       <c r="P6" s="7" t="s">
@@ -1475,10 +1577,10 @@
       <c r="B7" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="13">
         <v>99900049999</v>
       </c>
       <c r="E7" s="6" t="s">
@@ -1503,13 +1605,13 @@
       <c r="L7" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="M7" s="16" t="s">
+      <c r="M7" s="14" t="s">
         <v>65</v>
       </c>
       <c r="N7" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="O7" s="16" t="s">
         <v>67</v>
       </c>
       <c r="P7" s="7" t="s">
@@ -1530,10 +1632,10 @@
       <c r="B8" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="13">
         <v>88800088888</v>
       </c>
       <c r="E8" s="6" t="s">
@@ -1558,13 +1660,13 @@
       <c r="L8" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="M8" s="16" t="s">
+      <c r="M8" s="14" t="s">
         <v>79</v>
       </c>
       <c r="N8" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="O8" s="7" t="s">
+      <c r="O8" s="16" t="s">
         <v>79</v>
       </c>
       <c r="P8" s="7" t="s">
@@ -1588,7 +1690,7 @@
       <c r="C9" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="13">
         <v>88800088888</v>
       </c>
       <c r="E9" s="6" t="s">
@@ -1613,13 +1715,13 @@
       <c r="L9" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="M9" s="16" t="s">
+      <c r="M9" s="14" t="s">
         <v>79</v>
       </c>
       <c r="N9" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="O9" s="16" t="s">
         <v>79</v>
       </c>
       <c r="P9" s="7" t="s">
@@ -1648,58 +1750,58 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:18" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="L1" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="M1" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="N1" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="O1" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="P1" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="Q1" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="R1" s="11" t="s">
         <v>100</v>
       </c>
     </row>
@@ -1906,16 +2008,16 @@
       <c r="L5" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="M5" s="10">
+      <c r="M5">
         <v>0.1</v>
       </c>
-      <c r="N5" s="11" t="s">
+      <c r="N5" t="s">
         <v>122</v>
       </c>
-      <c r="O5" s="12">
+      <c r="O5" s="10">
         <v>40557</v>
       </c>
-      <c r="P5" s="12">
+      <c r="P5" s="10">
         <v>40571</v>
       </c>
       <c r="Q5" s="1">
@@ -1960,16 +2062,16 @@
       <c r="L6" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="M6" s="10">
+      <c r="M6">
         <v>0.1</v>
       </c>
-      <c r="N6" s="11" t="s">
+      <c r="N6" t="s">
         <v>122</v>
       </c>
-      <c r="O6" s="12">
+      <c r="O6" s="10">
         <v>40557</v>
       </c>
-      <c r="P6" s="12">
+      <c r="P6" s="10">
         <v>40571</v>
       </c>
       <c r="Q6" s="1">
@@ -2014,12 +2116,10 @@
       <c r="L7" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="12">
+      <c r="O7" s="10">
         <v>40557</v>
       </c>
-      <c r="P7" s="12">
+      <c r="P7" s="10">
         <v>40566</v>
       </c>
       <c r="Q7" s="1">
@@ -2066,10 +2166,10 @@
       </c>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
-      <c r="O8" s="12">
+      <c r="O8" s="10">
         <v>40568</v>
       </c>
-      <c r="P8" s="12">
+      <c r="P8" s="10">
         <v>40571</v>
       </c>
       <c r="Q8" s="1">

</xml_diff>

<commit_message>
Els' fixes and flipping rule direction
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87F0F39A-5848-7548-9C11-9E4A494FF374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC94EF39-FDD0-7B4C-B8BC-481DAEFB5B6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37840" yWindow="-3860" windowWidth="30240" windowHeight="18980" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -710,7 +710,7 @@
         <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F2" t="s">
         <v>49</v>
@@ -730,7 +730,7 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s">
         <v>51</v>
@@ -750,7 +750,7 @@
         <v>6</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F4" t="s">
         <v>49</v>
@@ -770,7 +770,7 @@
         <v>6</v>
       </c>
       <c r="E5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F5" t="s">
         <v>52</v>
@@ -790,7 +790,7 @@
         <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F6" t="s">
         <v>53</v>
@@ -810,7 +810,7 @@
         <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F7" t="s">
         <v>54</v>
@@ -830,7 +830,7 @@
         <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F8" t="s">
         <v>50</v>
@@ -850,7 +850,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F9" t="s">
         <v>44</v>
@@ -870,7 +870,7 @@
         <v>11</v>
       </c>
       <c r="E10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F10" t="s">
         <v>50</v>
@@ -890,7 +890,7 @@
         <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F11" t="s">
         <v>45</v>
@@ -1012,11 +1012,11 @@
       <c r="D5" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>49</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>51</v>
       </c>
       <c r="G5" s="5"/>
     </row>
@@ -1031,11 +1031,11 @@
       <c r="D6" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>49</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>52</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>33</v>
@@ -1052,11 +1052,11 @@
       <c r="D7" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>49</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>33</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>35</v>
@@ -1073,11 +1073,11 @@
       <c r="D8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="9" t="s">
         <v>53</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>54</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>37</v>
@@ -1094,11 +1094,11 @@
       <c r="D9" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="6" t="s">
         <v>49</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>41</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>42</v>
@@ -1117,11 +1117,11 @@
       <c r="D10" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" s="10" t="s">
         <v>50</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>44</v>
       </c>
       <c r="G10" s="5"/>
     </row>
@@ -1136,11 +1136,11 @@
       <c r="D11" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>50</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>45</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>46</v>

</xml_diff>

<commit_message>
Els' suggestions implemented and rule flipped
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9425C16F-0FA2-0B4C-BEBE-627CD4E427AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17C436DF-CA61-494E-B88F-0492EFA1C3D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37160" yWindow="-2900" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -665,7 +665,7 @@
         <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F2">
         <v>0.1</v>
@@ -685,7 +685,7 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -705,7 +705,7 @@
         <v>6</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F4">
         <v>2.9</v>
@@ -725,7 +725,7 @@
         <v>6</v>
       </c>
       <c r="E5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F5">
         <v>3</v>
@@ -745,7 +745,7 @@
         <v>7</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F6">
         <v>-20</v>
@@ -765,7 +765,7 @@
         <v>7</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F7">
         <v>5</v>
@@ -785,7 +785,7 @@
         <v>8</v>
       </c>
       <c r="E8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F8">
         <v>2000</v>
@@ -805,7 +805,7 @@
         <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F9">
         <v>200000</v>
@@ -958,10 +958,10 @@
         <v>37</v>
       </c>
       <c r="H5" s="6">
+        <v>1</v>
+      </c>
+      <c r="I5" s="6">
         <v>0.1</v>
-      </c>
-      <c r="I5" s="6">
-        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -984,10 +984,10 @@
         <v>40</v>
       </c>
       <c r="H6" s="6">
+        <v>3</v>
+      </c>
+      <c r="I6" s="6">
         <v>2.9</v>
-      </c>
-      <c r="I6" s="6">
-        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -1010,10 +1010,10 @@
         <v>42</v>
       </c>
       <c r="H7" s="6">
+        <v>5</v>
+      </c>
+      <c r="I7" s="6">
         <v>-20</v>
-      </c>
-      <c r="I7" s="6">
-        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -1036,10 +1036,10 @@
         <v>44</v>
       </c>
       <c r="H8" s="6">
+        <v>200000</v>
+      </c>
+      <c r="I8" s="6">
         <v>2000</v>
-      </c>
-      <c r="I8" s="6">
-        <v>200000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
rule condition removed and test data updated
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7356838-EECE-E04E-82CD-8D37908CCAF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BD2D4BE-F0EF-C948-8DCF-41B85B8EA29F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30320" yWindow="-8560" windowWidth="51200" windowHeight="28200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="124">
   <si>
     <t>Product</t>
   </si>
@@ -873,7 +873,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A268467F-CDB7-0842-BD4B-311D887FB169}">
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -1024,17 +1024,17 @@
       <c r="B8" t="s">
         <v>6</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="6" t="s">
         <v>119</v>
       </c>
       <c r="D8">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E8" t="s">
         <v>13</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -1044,17 +1044,17 @@
       <c r="B9" t="s">
         <v>6</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="6" t="s">
         <v>119</v>
       </c>
       <c r="D9">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>16</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -1068,7 +1068,7 @@
         <v>119</v>
       </c>
       <c r="D10">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E10" t="s">
         <v>13</v>
@@ -1088,13 +1088,13 @@
         <v>119</v>
       </c>
       <c r="D11">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>16</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>123</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -1108,13 +1108,13 @@
         <v>119</v>
       </c>
       <c r="D12">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E12" t="s">
         <v>13</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -1128,13 +1128,13 @@
         <v>119</v>
       </c>
       <c r="D13">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>16</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
@@ -1148,13 +1148,13 @@
         <v>119</v>
       </c>
       <c r="D14">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E14" t="s">
         <v>13</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>78</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
@@ -1168,13 +1168,13 @@
         <v>119</v>
       </c>
       <c r="D15">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>16</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
@@ -1188,13 +1188,13 @@
         <v>119</v>
       </c>
       <c r="D16">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E16" t="s">
         <v>13</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -1208,13 +1208,13 @@
         <v>119</v>
       </c>
       <c r="D17">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>16</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -1228,13 +1228,13 @@
         <v>119</v>
       </c>
       <c r="D18">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E18" t="s">
         <v>13</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -1248,13 +1248,13 @@
         <v>119</v>
       </c>
       <c r="D19">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>16</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>121</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -1268,13 +1268,13 @@
         <v>119</v>
       </c>
       <c r="D20">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E20" t="s">
         <v>13</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -1288,13 +1288,13 @@
         <v>119</v>
       </c>
       <c r="D21">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>16</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>84</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -1304,17 +1304,17 @@
       <c r="B22" t="s">
         <v>6</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="6" t="s">
         <v>119</v>
       </c>
       <c r="D22">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E22" t="s">
         <v>13</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -1324,18 +1324,16 @@
       <c r="B23" t="s">
         <v>6</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="6" t="s">
         <v>119</v>
       </c>
       <c r="D23">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F23" s="6" t="s">
-        <v>84</v>
-      </c>
+      <c r="F23" s="6"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24">
@@ -1348,70 +1346,150 @@
         <v>119</v>
       </c>
       <c r="D24">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E24" t="s">
         <v>13</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>12</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" t="s">
         <v>6</v>
       </c>
       <c r="C25" t="s">
         <v>119</v>
       </c>
       <c r="D25">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>16</v>
       </c>
       <c r="F25" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>13</v>
+      </c>
+      <c r="B26" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" t="s">
+        <v>119</v>
+      </c>
+      <c r="D26">
+        <v>23</v>
+      </c>
+      <c r="E26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>13</v>
+      </c>
+      <c r="B27" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" t="s">
+        <v>119</v>
+      </c>
+      <c r="D27">
+        <v>23</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>14</v>
+      </c>
+      <c r="B28" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" t="s">
+        <v>119</v>
+      </c>
+      <c r="D28">
+        <v>24</v>
+      </c>
+      <c r="E28" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>14</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" t="s">
+        <v>119</v>
+      </c>
+      <c r="D29">
+        <v>24</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" s="6" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F27" s="6"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F30" s="6"/>
-    </row>
-    <row r="33" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F33" s="6"/>
-    </row>
-    <row r="36" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F36" s="6"/>
-    </row>
-    <row r="39" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F39" s="6"/>
-    </row>
-    <row r="42" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F42" s="6"/>
-    </row>
-    <row r="45" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F45" s="6"/>
-    </row>
-    <row r="48" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F48" s="6"/>
-    </row>
-    <row r="51" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F51" s="6"/>
-    </row>
-    <row r="54" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F54" s="6"/>
-    </row>
-    <row r="57" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F57" s="6"/>
-    </row>
-    <row r="60" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F60" s="6"/>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F31" s="6"/>
+    </row>
+    <row r="34" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F34" s="6"/>
+    </row>
+    <row r="37" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F37" s="6"/>
+    </row>
+    <row r="40" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F40" s="6"/>
+    </row>
+    <row r="43" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F43" s="6"/>
+    </row>
+    <row r="46" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F46" s="6"/>
+    </row>
+    <row r="49" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F49" s="6"/>
+    </row>
+    <row r="52" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F52" s="6"/>
+    </row>
+    <row r="55" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F55" s="6"/>
+    </row>
+    <row r="58" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F58" s="6"/>
+    </row>
+    <row r="61" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F61" s="6"/>
+    </row>
+    <row r="64" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F64" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2187,7 +2265,7 @@
       <c r="E10" s="3">
         <v>17</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="7" t="s">
         <v>88</v>
       </c>
       <c r="G10" s="3" t="s">
@@ -2196,7 +2274,7 @@
       <c r="H10" s="3">
         <v>10006451</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="I10" s="5" t="s">
         <v>89</v>
       </c>
       <c r="J10" s="3">
@@ -3017,7 +3095,7 @@
       <c r="E20" s="3">
         <v>17</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="F20" s="5" t="s">
         <v>88</v>
       </c>
       <c r="G20" s="3" t="s">
@@ -3026,9 +3104,7 @@
       <c r="H20" s="3">
         <v>10006451</v>
       </c>
-      <c r="I20" s="3" t="s">
-        <v>89</v>
-      </c>
+      <c r="I20" s="5"/>
       <c r="J20" s="3">
         <v>10006451</v>
       </c>
@@ -3419,7 +3495,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:AA4 A6:AA7 A5:E5 G5:AA5 A20:AA23 A19:F19 H19 J19:AA19 A24:H24 J24:AA24 A14:AA18 A13:H13 J13:AA13 A10:AA12 A8:E8 G8:H8 J8:AA8 A9:E9 G9:AA9" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:AA4 A6:AA7 A5:E5 G5:AA5 A21:AA23 A19:F19 H19 J19:AA19 A24:H24 J24:AA24 A14:AA18 A13:H13 J13:AA13 A11:AA12 A8:E8 G8:H8 J8:AA8 A9:E9 G9:AA9 A20:H20 J20:AA20 A10:E10 G10:AA10" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
max value > variable length
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -49,6 +49,10 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <b/>
     </font>
     <font>
@@ -60,10 +64,6 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="4">
@@ -114,9 +114,9 @@
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -451,18 +451,18 @@
   <dimension ref="A1:B2"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
+      <c r="A1" s="3" t="str">
         <v>Product</v>
       </c>
-      <c r="B1" s="2" t="str">
+      <c r="B1" s="3" t="str">
         <v>Version</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="3" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="3" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -478,26 +478,26 @@
   <dimension ref="A1:B3"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
+      <c r="A1" s="3" t="str">
         <v>Filename</v>
       </c>
-      <c r="B1" s="2" t="str">
+      <c r="B1" s="3" t="str">
         <v>Label</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="3" t="str">
         <v>relrec.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="3" t="str">
         <v>Related Records</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="3" t="str">
         <v>suppae.xpt</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="3" t="str">
         <v>Supplemental Qualifiers for AE</v>
       </c>
     </row>
@@ -510,191 +510,351 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F17"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
+      <c r="A1" s="3" t="str">
         <v>Error group</v>
       </c>
-      <c r="B1" s="2" t="str">
+      <c r="B1" s="3" t="str">
         <v>Sheet</v>
       </c>
-      <c r="C1" s="2" t="str">
+      <c r="C1" s="3" t="str">
         <v>Error level</v>
       </c>
-      <c r="D1" s="2" t="str">
+      <c r="D1" s="3" t="str">
         <v>Row num</v>
       </c>
-      <c r="E1" s="2" t="str">
-        <v>Variable</v>
-      </c>
-      <c r="F1" s="2" t="str">
+      <c r="E1" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="F1" s="3" t="str">
         <v>Error value</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="3" t="str">
         <v>relrec.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
-        <v>Variable</v>
-      </c>
-      <c r="D2" s="2" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="E2" s="2" t="str">
+      <c r="C2" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D2" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E2" s="3" t="str">
         <v>variable_name</v>
       </c>
-      <c r="F2" s="2" t="str">
+      <c r="F2" s="3" t="str">
         <v>USUBJID</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="3" t="str">
         <v>relrec.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
-        <v>Variable</v>
-      </c>
-      <c r="D3" s="2" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="E3" s="2" t="str">
+      <c r="C3" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D3" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E3" s="3" t="str">
         <v>variable_value</v>
       </c>
-      <c r="F3" s="2" t="str">
+      <c r="F3" s="3" t="str">
         <v>CDISC0001</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
+      <c r="A4" s="3">
         <v>1</v>
       </c>
-      <c r="B4" s="2" t="str">
+      <c r="B4" s="3" t="str">
         <v>relrec.xpt</v>
       </c>
-      <c r="C4" s="2" t="str">
-        <v>Variable</v>
-      </c>
-      <c r="D4" s="2" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="E4" s="2" t="str">
-        <v>variable_size</v>
-      </c>
-      <c r="F4" s="2">
+      <c r="C4" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D4" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E4" s="3" t="str">
+        <v>variable_length</v>
+      </c>
+      <c r="F4" s="3">
         <v>8</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2">
+      <c r="A5" s="3">
         <v>1</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="3" t="str">
         <v>relrec.xpt</v>
       </c>
-      <c r="C5" s="2" t="str">
-        <v>Variable</v>
-      </c>
-      <c r="D5" s="2" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="E5" s="2" t="str">
+      <c r="C5" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D5" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E5" s="3" t="str">
         <v>variable_value_length</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="3">
         <v>9</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2">
+      <c r="A6" s="3">
         <v>2</v>
       </c>
-      <c r="B6" s="2" t="str">
+      <c r="B6" s="3" t="str">
+        <v>relrec.xpt</v>
+      </c>
+      <c r="C6" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D6" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E6" s="3" t="str">
+        <v>variable_name</v>
+      </c>
+      <c r="F6" s="3" t="str">
+        <v>USUBJID</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>2</v>
+      </c>
+      <c r="B7" s="3" t="str">
+        <v>relrec.xpt</v>
+      </c>
+      <c r="C7" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D7" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E7" s="3" t="str">
+        <v>variable_value</v>
+      </c>
+      <c r="F7" s="3" t="str">
+        <v>CDISC001</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>2</v>
+      </c>
+      <c r="B8" s="3" t="str">
+        <v>relrec.xpt</v>
+      </c>
+      <c r="C8" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D8" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E8" s="3" t="str">
+        <v>variable_length</v>
+      </c>
+      <c r="F8" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>2</v>
+      </c>
+      <c r="B9" s="3" t="str">
+        <v>relrec.xpt</v>
+      </c>
+      <c r="C9" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D9" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E9" s="3" t="str">
+        <v>variable_value_length</v>
+      </c>
+      <c r="F9" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>3</v>
+      </c>
+      <c r="B10" s="3" t="str">
         <v>suppae.xpt</v>
       </c>
-      <c r="C6" s="2" t="str">
-        <v>Variable</v>
-      </c>
-      <c r="D6" s="2" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="E6" s="2" t="str">
+      <c r="C10" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D10" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E10" s="3" t="str">
         <v>variable_name</v>
       </c>
-      <c r="F6" s="2" t="str">
+      <c r="F10" s="3" t="str">
         <v>QVAL</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>2</v>
-      </c>
-      <c r="B7" s="2" t="str">
+    <row r="11">
+      <c r="A11" s="3">
+        <v>3</v>
+      </c>
+      <c r="B11" s="3" t="str">
         <v>suppae.xpt</v>
       </c>
-      <c r="C7" s="2" t="str">
-        <v>Variable</v>
-      </c>
-      <c r="D7" s="2" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="E7" s="2" t="str">
+      <c r="C11" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D11" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E11" s="3" t="str">
         <v>variable_value</v>
       </c>
-      <c r="F7" s="2" t="str">
+      <c r="F11" s="3" t="str">
         <v>TWENTYCHARACTERVALUE</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2">
-        <v>2</v>
-      </c>
-      <c r="B8" s="2" t="str">
+    <row r="12">
+      <c r="A12" s="3">
+        <v>3</v>
+      </c>
+      <c r="B12" s="3" t="str">
         <v>suppae.xpt</v>
       </c>
-      <c r="C8" s="2" t="str">
-        <v>Variable</v>
-      </c>
-      <c r="D8" s="2" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="E8" s="2" t="str">
-        <v>variable_size</v>
-      </c>
-      <c r="F8" s="2">
+      <c r="C12" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D12" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E12" s="3" t="str">
+        <v>variable_length</v>
+      </c>
+      <c r="F12" s="3">
         <v>19</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2">
-        <v>2</v>
-      </c>
-      <c r="B9" s="2" t="str">
+    <row r="13">
+      <c r="A13" s="3">
+        <v>3</v>
+      </c>
+      <c r="B13" s="3" t="str">
         <v>suppae.xpt</v>
       </c>
-      <c r="C9" s="2" t="str">
-        <v>Variable</v>
-      </c>
-      <c r="D9" s="2" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="E9" s="2" t="str">
+      <c r="C13" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D13" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E13" s="3" t="str">
         <v>variable_value_length</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F13" s="3">
         <v>20</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3">
+        <v>4</v>
+      </c>
+      <c r="B14" s="3" t="str">
+        <v>suppae.xpt</v>
+      </c>
+      <c r="C14" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D14" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E14" s="3" t="str">
+        <v>variable_name</v>
+      </c>
+      <c r="F14" s="3" t="str">
+        <v>QVAL</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3">
+        <v>4</v>
+      </c>
+      <c r="B15" s="3" t="str">
+        <v>suppae.xpt</v>
+      </c>
+      <c r="C15" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D15" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E15" s="3" t="str">
+        <v>variable_value</v>
+      </c>
+      <c r="F15" s="3" t="str">
+        <v>MEDDRA VERSION 22.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3">
+        <v>4</v>
+      </c>
+      <c r="B16" s="3" t="str">
+        <v>suppae.xpt</v>
+      </c>
+      <c r="C16" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D16" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E16" s="3" t="str">
+        <v>variable_length</v>
+      </c>
+      <c r="F16" s="3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3">
+        <v>4</v>
+      </c>
+      <c r="B17" s="3" t="str">
+        <v>suppae.xpt</v>
+      </c>
+      <c r="C17" s="3" t="str">
+        <v>Variable</v>
+      </c>
+      <c r="D17" s="3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E17" s="3" t="str">
+        <v>variable_value_length</v>
+      </c>
+      <c r="F17" s="3">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -704,140 +864,140 @@
   <dimension ref="A1:G6"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="str">
+      <c r="A1" s="4" t="str">
         <v>STUDYID</v>
       </c>
-      <c r="B1" s="3" t="str">
+      <c r="B1" s="4" t="str">
         <v>RDOMAIN</v>
       </c>
-      <c r="C1" s="3" t="str">
+      <c r="C1" s="4" t="str">
         <v>USUBJID</v>
       </c>
-      <c r="D1" s="3" t="str">
+      <c r="D1" s="4" t="str">
         <v>IDVAR</v>
       </c>
-      <c r="E1" s="3" t="str">
+      <c r="E1" s="4" t="str">
         <v>IDVARVAL</v>
       </c>
-      <c r="F1" s="3" t="str">
+      <c r="F1" s="4" t="str">
         <v>RELTYPE</v>
       </c>
-      <c r="G1" s="3" t="str">
+      <c r="G1" s="4" t="str">
         <v>RELID</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="6" t="str">
         <v>Related Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Identifying Variable</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Identifying Variable Value</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Relationship Type</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Relationship Identifier</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>12</v>
       </c>
-      <c r="B4" s="5">
-        <v>6</v>
-      </c>
-      <c r="C4" s="5">
+      <c r="B4" s="6">
+        <v>2</v>
+      </c>
+      <c r="C4" s="6">
         <v>8</v>
       </c>
-      <c r="D4" s="5">
-        <v>200</v>
-      </c>
-      <c r="E4" s="5">
-        <v>200</v>
-      </c>
-      <c r="F4" s="5">
+      <c r="D4" s="6">
+        <v>5</v>
+      </c>
+      <c r="E4" s="6">
+        <v>1</v>
+      </c>
+      <c r="F4" s="6">
+        <v>3</v>
+      </c>
+      <c r="G4" s="6">
         <v>4</v>
       </c>
-      <c r="G4" s="5">
-        <v>200</v>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="str">
+      <c r="A5" s="3" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="3" t="str">
         <v>AE</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="3" t="str">
         <v>CDISC0001</v>
       </c>
-      <c r="D5" s="6" t="str">
+      <c r="D5" s="3" t="str">
         <v>AESEQ</v>
       </c>
-      <c r="E5" s="6" t="str">
+      <c r="E5" s="3" t="str">
         <v>1</v>
       </c>
-      <c r="F5" s="6" t="str">
+      <c r="F5" s="3" t="str">
         <v>ONE</v>
       </c>
-      <c r="G5" s="6" t="str">
+      <c r="G5" s="3" t="str">
         <v>AEDS</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="str">
+      <c r="A6" s="3" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="6" t="str">
+      <c r="B6" s="3" t="str">
         <v>DS</v>
       </c>
-      <c r="C6" s="6" t="str">
+      <c r="C6" s="3" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="6" t="str">
+      <c r="D6" s="3" t="str">
         <v>AESEQ</v>
       </c>
-      <c r="E6" s="6" t="str">
+      <c r="E6" s="3" t="str">
         <v>2</v>
       </c>
-      <c r="F6" s="6" t="str">
+      <c r="F6" s="3" t="str">
         <v>ONE</v>
       </c>
-      <c r="G6" s="6" t="str">
+      <c r="G6" s="3" t="str">
         <v>AEDS</v>
       </c>
     </row>
@@ -853,194 +1013,194 @@
   <dimension ref="A1:J6"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="str">
+      <c r="A1" s="4" t="str">
         <v>STUDYID</v>
       </c>
-      <c r="B1" s="3" t="str">
+      <c r="B1" s="4" t="str">
         <v>RDOMAIN</v>
       </c>
-      <c r="C1" s="3" t="str">
+      <c r="C1" s="4" t="str">
         <v>USUBJID</v>
       </c>
-      <c r="D1" s="3" t="str">
+      <c r="D1" s="4" t="str">
         <v>IDVAR</v>
       </c>
-      <c r="E1" s="3" t="str">
+      <c r="E1" s="4" t="str">
         <v>IDVARVAL</v>
       </c>
-      <c r="F1" s="3" t="str">
+      <c r="F1" s="4" t="str">
         <v>QNAM</v>
       </c>
-      <c r="G1" s="3" t="str">
+      <c r="G1" s="4" t="str">
         <v>QLABEL</v>
       </c>
-      <c r="H1" s="3" t="str">
+      <c r="H1" s="4" t="str">
         <v>QVAL</v>
       </c>
-      <c r="I1" s="3" t="str">
+      <c r="I1" s="4" t="str">
         <v>QORIG</v>
       </c>
-      <c r="J1" s="3" t="str">
+      <c r="J1" s="4" t="str">
         <v>QEVAL</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Related Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Identifying Variable</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Identifying Variable Value</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Qualifier Variable Name</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Qualifier Variable Label</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Data Value</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Origin</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Evaluator</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>12</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
-        <v>14</v>
-      </c>
-      <c r="D4" s="5">
+      <c r="C4" s="6">
+        <v>8</v>
+      </c>
+      <c r="D4" s="6">
         <v>6</v>
       </c>
-      <c r="E4" s="5">
-        <v>4</v>
-      </c>
-      <c r="F4" s="5">
+      <c r="E4" s="6">
+        <v>2</v>
+      </c>
+      <c r="F4" s="6">
         <v>7</v>
       </c>
-      <c r="G4" s="5">
-        <v>40</v>
-      </c>
-      <c r="H4" s="5">
+      <c r="G4" s="6">
+        <v>18</v>
+      </c>
+      <c r="H4" s="6">
         <v>19</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="6">
         <v>8</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="6">
         <v>22</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="str">
+      <c r="A5" s="3" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="3" t="str">
         <v>AE</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="3" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="6" t="str">
+      <c r="D5" s="3" t="str">
         <v>AESPID</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="3">
         <v>1</v>
       </c>
-      <c r="F5" s="6" t="str">
+      <c r="F5" s="3" t="str">
         <v>DICTVER</v>
       </c>
-      <c r="G5" s="6" t="str">
+      <c r="G5" s="3" t="str">
         <v>Dictionary Version</v>
       </c>
-      <c r="H5" s="6" t="str">
+      <c r="H5" s="3" t="str">
         <v>TWENTYCHARACTERVALUE</v>
       </c>
-      <c r="I5" s="6" t="str">
+      <c r="I5" s="3" t="str">
         <v>Assigned</v>
       </c>
-      <c r="J5" s="6" t="str">
+      <c r="J5" s="3" t="str">
         <v>CLINICAL STUDY SPONSOR</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="str">
+      <c r="A6" s="3" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="6" t="str">
+      <c r="B6" s="3" t="str">
         <v>AE</v>
       </c>
-      <c r="C6" s="6" t="str">
+      <c r="C6" s="3" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="6" t="str">
+      <c r="D6" s="3" t="str">
         <v>AESPID</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="3">
         <v>11</v>
       </c>
-      <c r="F6" s="6" t="str">
+      <c r="F6" s="3" t="str">
         <v>DICTVER</v>
       </c>
-      <c r="G6" s="6" t="str">
+      <c r="G6" s="3" t="str">
         <v>Dictionary Version</v>
       </c>
-      <c r="H6" s="6" t="str">
+      <c r="H6" s="3" t="str">
         <v>MEDDRA VERSION 22.0</v>
       </c>
-      <c r="I6" s="6" t="str">
+      <c r="I6" s="3" t="str">
         <v>Assigned</v>
       </c>
-      <c r="J6" s="6" t="str">
+      <c r="J6" s="3" t="str">
         <v>CLINICAL STUDY SPONSOR</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Changed sensitivity to Dataset in YAML file and completed the Validation sheets in the Excel files
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AF5F2F3-4F3E-D846-877A-05314940B99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17B85662-5133-0746-A235-239505F51CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1400" yWindow="660" windowWidth="28800" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="304">
   <si>
     <t>Product</t>
   </si>
@@ -1398,7 +1398,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="4" width="10.33203125" customWidth="1"/>
@@ -1523,6 +1523,206 @@
         <v>55</v>
       </c>
       <c r="F6" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>297</v>
+      </c>
+      <c r="C7" t="s">
+        <v>300</v>
+      </c>
+      <c r="D7" t="s">
+        <v>299</v>
+      </c>
+      <c r="E7" t="s">
+        <v>301</v>
+      </c>
+      <c r="F7" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>297</v>
+      </c>
+      <c r="C8" t="s">
+        <v>300</v>
+      </c>
+      <c r="D8" t="s">
+        <v>299</v>
+      </c>
+      <c r="E8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>297</v>
+      </c>
+      <c r="C9" t="s">
+        <v>300</v>
+      </c>
+      <c r="D9" t="s">
+        <v>299</v>
+      </c>
+      <c r="E9" t="s">
+        <v>302</v>
+      </c>
+      <c r="F9" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>297</v>
+      </c>
+      <c r="C10" t="s">
+        <v>300</v>
+      </c>
+      <c r="D10" t="s">
+        <v>299</v>
+      </c>
+      <c r="E10" t="s">
+        <v>120</v>
+      </c>
+      <c r="F10" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="8">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>297</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>300</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>299</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>300</v>
+      </c>
+      <c r="D12" t="s">
+        <v>299</v>
+      </c>
+      <c r="E12" t="s">
+        <v>301</v>
+      </c>
+      <c r="F12" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" t="s">
+        <v>300</v>
+      </c>
+      <c r="D13" t="s">
+        <v>299</v>
+      </c>
+      <c r="E13" t="s">
+        <v>91</v>
+      </c>
+      <c r="F13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" t="s">
+        <v>300</v>
+      </c>
+      <c r="D14" t="s">
+        <v>299</v>
+      </c>
+      <c r="E14" t="s">
+        <v>302</v>
+      </c>
+      <c r="F14" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>3</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s">
+        <v>300</v>
+      </c>
+      <c r="D15" t="s">
+        <v>299</v>
+      </c>
+      <c r="E15" t="s">
+        <v>120</v>
+      </c>
+      <c r="F15" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="8">
+        <v>3</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>300</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>299</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="F16" s="8" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
codes instead of names
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -73,7 +73,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -93,12 +93,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -134,7 +128,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -144,7 +138,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -609,7 +602,7 @@
         <v>TSVALCD</v>
       </c>
       <c r="F4" s="3" t="str">
-        <v>atlantis-code</v>
+        <v>ATL</v>
       </c>
     </row>
     <row r="5">
@@ -669,7 +662,7 @@
         <v>TSVAL</v>
       </c>
       <c r="F7" s="3" t="str">
-        <v>Curacao</v>
+        <v>Akrotiri</v>
       </c>
     </row>
     <row r="8">
@@ -689,7 +682,7 @@
         <v>TSVALCD</v>
       </c>
       <c r="F8" s="3" t="str">
-        <v>curacao-code</v>
+        <v>XQZ</v>
       </c>
     </row>
     <row r="9">
@@ -713,82 +706,82 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2">
+      <c r="A10" s="3">
         <v>3</v>
       </c>
-      <c r="B10" s="2" t="str">
-        <v>ts.xpt</v>
-      </c>
-      <c r="C10" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D10" s="2">
+      <c r="B10" s="3" t="str">
+        <v>ts.xpt</v>
+      </c>
+      <c r="C10" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D10" s="3">
         <v>7</v>
       </c>
-      <c r="E10" s="2" t="str">
+      <c r="E10" s="3" t="str">
         <v>TSPARMCD</v>
       </c>
-      <c r="F10" s="2" t="str">
+      <c r="F10" s="3" t="str">
         <v>FCNTRY</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2">
+      <c r="A11" s="3">
         <v>3</v>
       </c>
-      <c r="B11" s="2" t="str">
-        <v>ts.xpt</v>
-      </c>
-      <c r="C11" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D11" s="2">
+      <c r="B11" s="3" t="str">
+        <v>ts.xpt</v>
+      </c>
+      <c r="C11" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D11" s="3">
         <v>7</v>
       </c>
-      <c r="E11" s="2" t="str">
+      <c r="E11" s="3" t="str">
         <v>TSVAL</v>
       </c>
-      <c r="F11" s="2" t="str">
-        <v>Bahamas</v>
+      <c r="F11" s="3" t="str">
+        <v>Åland Islands</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2">
+      <c r="A12" s="3">
         <v>3</v>
       </c>
-      <c r="B12" s="2" t="str">
-        <v>ts.xpt</v>
-      </c>
-      <c r="C12" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D12" s="2">
+      <c r="B12" s="3" t="str">
+        <v>ts.xpt</v>
+      </c>
+      <c r="C12" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D12" s="3">
         <v>7</v>
       </c>
-      <c r="E12" s="2" t="str">
+      <c r="E12" s="3" t="str">
         <v>TSVALCD</v>
       </c>
-      <c r="F12" s="2" t="str">
-        <v>bahamas-code</v>
+      <c r="F12" s="3" t="str">
+        <v>ALA</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2">
+      <c r="A13" s="3">
         <v>3</v>
       </c>
-      <c r="B13" s="2" t="str">
-        <v>ts.xpt</v>
-      </c>
-      <c r="C13" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D13" s="2">
+      <c r="B13" s="3" t="str">
+        <v>ts.xpt</v>
+      </c>
+      <c r="C13" s="3" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D13" s="3">
         <v>7</v>
       </c>
-      <c r="E13" s="2" t="str">
+      <c r="E13" s="3" t="str">
         <v>TSVCDREF</v>
       </c>
-      <c r="F13" s="2" t="str">
+      <c r="F13" s="3" t="str">
         <v>GENC</v>
       </c>
     </row>
@@ -848,16 +841,16 @@
       <c r="C2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Group ID</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Trial Summary Parameter Short Name</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Trial Summary Parameter</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Parameter Value</v>
       </c>
       <c r="H2" s="6" t="str">
@@ -969,9 +962,9 @@
         <v>NA</v>
       </c>
       <c r="I5" s="7" t="str">
-        <v>atlantis-code</v>
-      </c>
-      <c r="J5" s="7" t="str">
+        <v>ATL</v>
+      </c>
+      <c r="J5" s="8" t="str">
         <v>GENC</v>
       </c>
     </row>
@@ -988,51 +981,54 @@
       <c r="D6" s="3" t="str">
         <v/>
       </c>
-      <c r="E6" s="7" t="str">
+      <c r="E6" s="8" t="str">
         <v>FCNTRY</v>
       </c>
       <c r="F6" s="3" t="str">
         <v>Planned Country of Investigational Sites</v>
       </c>
-      <c r="G6" s="7" t="str">
-        <v>Curacao</v>
+      <c r="G6" s="8" t="str">
+        <v>Akrotiri</v>
       </c>
       <c r="H6" s="3" t="str">
         <v>NA</v>
       </c>
-      <c r="I6" s="7" t="str">
-        <v>curacao-code</v>
+      <c r="I6" s="8" t="str">
+        <v>XQZ</v>
       </c>
       <c r="J6" s="8" t="str">
         <v>ISO 3166</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="str">
+      <c r="A7" s="3" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B7" s="2" t="str">
+      <c r="B7" s="3" t="str">
         <v>TS</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="3">
         <v>3</v>
       </c>
-      <c r="E7" s="9" t="str">
+      <c r="D7" s="3" t="str">
+        <v/>
+      </c>
+      <c r="E7" s="8" t="str">
         <v>FCNTRY</v>
       </c>
-      <c r="F7" s="2" t="str">
+      <c r="F7" s="3" t="str">
         <v>Planned Country of Investigational Sites</v>
       </c>
-      <c r="G7" s="9" t="str">
-        <v>Bahamas</v>
-      </c>
-      <c r="H7" s="2" t="str">
+      <c r="G7" s="7" t="str">
+        <v>Åland Islands</v>
+      </c>
+      <c r="H7" s="3" t="str">
         <v>NA</v>
       </c>
-      <c r="I7" s="9" t="str">
-        <v>bahamas-code</v>
-      </c>
-      <c r="J7" s="9" t="str">
+      <c r="I7" s="8" t="str">
+        <v>ALA</v>
+      </c>
+      <c r="J7" s="8" t="str">
         <v>GENC</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added TESTCD as output variable
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D1A3406-943A-3745-AC34-0461430A0192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0BC13D3-05FC-C442-9EB7-F25884D88E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="185">
   <si>
     <t>Product</t>
   </si>
@@ -686,7 +686,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -710,11 +710,6 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1077,7 +1072,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC590268-A813-7E46-A402-7CCF030F7149}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -1096,7 +1091,7 @@
       <c r="E1" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="10" t="s">
         <v>183</v>
       </c>
     </row>
@@ -1116,7 +1111,7 @@
       <c r="E2" t="s">
         <v>118</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="4" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1136,11 +1131,10 @@
       <c r="E3" t="s">
         <v>117</v>
       </c>
-      <c r="F3" s="13"/>
-    </row>
-    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
         <v>175</v>
@@ -1149,16 +1143,16 @@
         <v>184</v>
       </c>
       <c r="D4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E4" t="s">
-        <v>118</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+      <c r="F4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2</v>
       </c>
@@ -1172,13 +1166,15 @@
         <v>6</v>
       </c>
       <c r="E5" t="s">
-        <v>117</v>
-      </c>
-      <c r="F5" s="13"/>
-    </row>
-    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B6" t="s">
         <v>175</v>
@@ -1187,18 +1183,15 @@
         <v>184</v>
       </c>
       <c r="D6">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E6" t="s">
-        <v>118</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>177</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B7" t="s">
         <v>175</v>
@@ -1207,12 +1200,71 @@
         <v>184</v>
       </c>
       <c r="D7">
+        <v>6</v>
+      </c>
+      <c r="E7" t="s">
+        <v>101</v>
+      </c>
+      <c r="F7" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>175</v>
+      </c>
+      <c r="C8" t="s">
+        <v>184</v>
+      </c>
+      <c r="D8">
         <v>8</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E8" t="s">
+        <v>118</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>175</v>
+      </c>
+      <c r="C9" t="s">
+        <v>184</v>
+      </c>
+      <c r="D9">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
         <v>117</v>
       </c>
-      <c r="F7" s="13"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>175</v>
+      </c>
+      <c r="C10" t="s">
+        <v>184</v>
+      </c>
+      <c r="D10">
+        <v>8</v>
+      </c>
+      <c r="E10" t="s">
+        <v>101</v>
+      </c>
+      <c r="F10" t="s">
+        <v>154</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2139,7 +2191,7 @@
       <c r="D5" s="4">
         <v>1</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="9" t="s">
         <v>142</v>
       </c>
       <c r="F5" s="4" t="s">
@@ -2214,7 +2266,7 @@
       <c r="D6" s="4">
         <v>2</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="9" t="s">
         <v>154</v>
       </c>
       <c r="F6" s="4" t="s">
@@ -2372,7 +2424,7 @@
       <c r="D8" s="4">
         <v>4</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="9" t="s">
         <v>154</v>
       </c>
       <c r="F8" s="4" t="s">

</xml_diff>

<commit_message>
included negative case where DTC variable is missing
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0BC13D3-05FC-C442-9EB7-F25884D88E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E7740AA-0655-9B41-B718-B8734C1195B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="186">
   <si>
     <t>Product</t>
   </si>
@@ -440,9 +440,6 @@
     <t>Visit Name</t>
   </si>
   <si>
-    <t>Date/Time of Specimen Collection</t>
-  </si>
-  <si>
     <t>End Date/Time of Specimen Collection</t>
   </si>
   <si>
@@ -579,6 +576,12 @@
   </si>
   <si>
     <t>Record</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>[ABSENT]</t>
   </si>
 </sst>
 </file>
@@ -686,7 +689,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -710,6 +713,9 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1059,10 +1065,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B3" t="s">
         <v>175</v>
-      </c>
-      <c r="B3" t="s">
-        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -1072,27 +1078,27 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC590268-A813-7E46-A402-7CCF030F7149}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="C1" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="D1" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="E1" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="F1" s="10" t="s">
         <v>182</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1100,10 +1106,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D2">
         <v>5</v>
@@ -1120,27 +1126,30 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C3" t="s">
+        <v>181</v>
+      </c>
+      <c r="D3" t="s">
         <v>184</v>
-      </c>
-      <c r="D3">
-        <v>5</v>
       </c>
       <c r="E3" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D4">
         <v>5</v>
@@ -1148,8 +1157,8 @@
       <c r="E4" t="s">
         <v>101</v>
       </c>
-      <c r="F4" t="s">
-        <v>142</v>
+      <c r="F4" s="4" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1157,10 +1166,10 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D5">
         <v>6</v>
@@ -1168,8 +1177,8 @@
       <c r="E5" t="s">
         <v>118</v>
       </c>
-      <c r="F5" s="4" t="s">
-        <v>177</v>
+      <c r="F5" s="11" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -1177,27 +1186,30 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C6" t="s">
+        <v>181</v>
+      </c>
+      <c r="D6" t="s">
         <v>184</v>
-      </c>
-      <c r="D6">
-        <v>6</v>
       </c>
       <c r="E6" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F6" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D7">
         <v>6</v>
@@ -1205,8 +1217,8 @@
       <c r="E7" t="s">
         <v>101</v>
       </c>
-      <c r="F7" t="s">
-        <v>154</v>
+      <c r="F7" s="11" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1214,19 +1226,19 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E8" t="s">
         <v>118</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>177</v>
+      <c r="F8" s="11" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -1234,36 +1246,159 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C9" t="s">
+        <v>181</v>
+      </c>
+      <c r="D9" t="s">
         <v>184</v>
-      </c>
-      <c r="D9">
-        <v>8</v>
       </c>
       <c r="E9" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F9" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D10">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E10" t="s">
         <v>101</v>
       </c>
-      <c r="F10" t="s">
-        <v>154</v>
+      <c r="F10" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>174</v>
+      </c>
+      <c r="C11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D11">
+        <v>8</v>
+      </c>
+      <c r="E11" t="s">
+        <v>118</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>174</v>
+      </c>
+      <c r="C12" t="s">
+        <v>181</v>
+      </c>
+      <c r="D12" t="s">
+        <v>184</v>
+      </c>
+      <c r="E12" t="s">
+        <v>117</v>
+      </c>
+      <c r="F12" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>174</v>
+      </c>
+      <c r="C13" t="s">
+        <v>183</v>
+      </c>
+      <c r="D13">
+        <v>8</v>
+      </c>
+      <c r="E13" t="s">
+        <v>101</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>5</v>
+      </c>
+      <c r="B14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C14" t="s">
+        <v>183</v>
+      </c>
+      <c r="D14">
+        <v>9</v>
+      </c>
+      <c r="E14" t="s">
+        <v>118</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>5</v>
+      </c>
+      <c r="B15" t="s">
+        <v>174</v>
+      </c>
+      <c r="C15" t="s">
+        <v>181</v>
+      </c>
+      <c r="D15" t="s">
+        <v>184</v>
+      </c>
+      <c r="E15" t="s">
+        <v>117</v>
+      </c>
+      <c r="F15" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>5</v>
+      </c>
+      <c r="B16" t="s">
+        <v>174</v>
+      </c>
+      <c r="C16" t="s">
+        <v>183</v>
+      </c>
+      <c r="D16">
+        <v>9</v>
+      </c>
+      <c r="E16" t="s">
+        <v>101</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -1843,10 +1978,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8C96987-FD28-5544-826B-B09F38914901}">
-  <dimension ref="A1:AA9"/>
+  <dimension ref="A1:Z9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:27" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:26" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>7</v>
       </c>
@@ -1911,25 +2046,22 @@
         <v>10</v>
       </c>
       <c r="V1" s="7" t="s">
-        <v>117</v>
+        <v>172</v>
       </c>
       <c r="W1" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="X1" s="7" t="s">
         <v>118</v>
       </c>
+      <c r="X1" s="2" t="s">
+        <v>119</v>
+      </c>
       <c r="Y1" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="Z1" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="AA1" s="7" t="s">
+      <c r="Z1" s="7" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="2" spans="1:27" ht="80" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:26" ht="80" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>11</v>
       </c>
@@ -1994,25 +2126,22 @@
         <v>15</v>
       </c>
       <c r="V2" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="W2" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="W2" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="X2" s="8" t="s">
+      <c r="X2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z2" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="Y2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="Z2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="AA2" s="8" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" ht="16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:26" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
         <v>18</v>
       </c>
@@ -2082,20 +2211,17 @@
       <c r="W3" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="X3" s="8" t="s">
+      <c r="X3" s="3" t="s">
         <v>18</v>
       </c>
       <c r="Y3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="Z3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="AA3" s="8" t="s">
+      <c r="Z3" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A4" s="8">
         <v>12</v>
       </c>
@@ -2165,25 +2291,22 @@
       <c r="W4" s="8">
         <v>19</v>
       </c>
-      <c r="X4" s="8">
-        <v>19</v>
+      <c r="X4" s="3">
+        <v>50</v>
       </c>
       <c r="Y4" s="3">
         <v>50</v>
       </c>
-      <c r="Z4" s="3">
-        <v>50</v>
-      </c>
-      <c r="AA4" s="8">
+      <c r="Z4" s="8">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="32" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>20</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>21</v>
@@ -2192,37 +2315,37 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="H5" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="I5" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="J5" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="K5" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="L5" s="4" t="s">
         <v>148</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>149</v>
       </c>
       <c r="M5" s="4">
         <v>39</v>
       </c>
       <c r="N5" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="Q5" s="4" t="s">
         <v>150</v>
-      </c>
-      <c r="Q5" s="4" t="s">
-        <v>151</v>
       </c>
       <c r="R5" s="4" t="s">
         <v>25</v>
@@ -2231,34 +2354,33 @@
         <v>1</v>
       </c>
       <c r="T5" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="U5" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="U5" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="V5" s="9"/>
-      <c r="W5" s="4" t="s">
+      <c r="V5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="X5" s="9" t="s">
+      <c r="W5" s="9" t="s">
         <v>27</v>
       </c>
+      <c r="X5" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="Y5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z5" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="AA5" s="4">
+        <v>151</v>
+      </c>
+      <c r="Z5" s="4">
         <v>-7</v>
       </c>
     </row>
-    <row r="6" spans="1:27" ht="32" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:26" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>21</v>
@@ -2267,43 +2389,43 @@
         <v>2</v>
       </c>
       <c r="E6" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="G6" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="G6" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="H6" s="4" t="s">
+      <c r="I6" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="J6" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="K6" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="K6" s="4" t="s">
-        <v>159</v>
-      </c>
       <c r="L6" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="M6" s="4">
         <v>93</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O6" s="4">
         <v>35</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="R6" s="4" t="s">
         <v>25</v>
@@ -2312,34 +2434,33 @@
         <v>1</v>
       </c>
       <c r="T6" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="U6" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="U6" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="V6" s="9"/>
-      <c r="W6" s="4" t="s">
+      <c r="V6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="X6" s="9" t="s">
-        <v>177</v>
+      <c r="W6" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="X6" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z6" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="AA6" s="4">
+        <v>151</v>
+      </c>
+      <c r="Z6" s="4">
         <v>-7</v>
       </c>
     </row>
-    <row r="7" spans="1:27" ht="32" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>20</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>22</v>
@@ -2347,41 +2468,41 @@
       <c r="D7" s="4">
         <v>3</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="G7" s="4" t="s">
-        <v>144</v>
-      </c>
       <c r="H7" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="J7" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="K7" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="J7" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>158</v>
-      </c>
       <c r="L7" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="M7" s="4">
         <v>18</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O7" s="4">
         <v>6</v>
       </c>
       <c r="Q7" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="R7" s="4" t="s">
         <v>25</v>
@@ -2390,33 +2511,30 @@
         <v>1</v>
       </c>
       <c r="T7" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="U7" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="U7" s="4" t="s">
-        <v>153</v>
-      </c>
       <c r="V7" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="W7" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="X7" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="Z7" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="AA7" s="4">
+        <v>176</v>
+      </c>
+      <c r="W7" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="Y7" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="Z7" s="4">
         <v>-7</v>
       </c>
     </row>
-    <row r="8" spans="1:27" ht="32" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:26" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>22</v>
@@ -2425,40 +2543,40 @@
         <v>4</v>
       </c>
       <c r="E8" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>155</v>
-      </c>
       <c r="G8" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H8" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="J8" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="I8" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="J8" s="4" t="s">
+      <c r="K8" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="K8" s="4" t="s">
-        <v>164</v>
-      </c>
       <c r="L8" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M8" s="4">
         <v>26</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P8" s="4">
         <v>36</v>
       </c>
       <c r="Q8" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="R8" s="4" t="s">
         <v>25</v>
@@ -2467,34 +2585,33 @@
         <v>1</v>
       </c>
       <c r="T8" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="U8" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="U8" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="V8" s="9"/>
-      <c r="W8" s="4" t="s">
+      <c r="V8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="X8" s="9" t="s">
-        <v>177</v>
+      <c r="W8" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="X8" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="Y8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z8" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="AA8" s="4">
+        <v>151</v>
+      </c>
+      <c r="Z8" s="4">
         <v>-7</v>
       </c>
     </row>
-    <row r="9" spans="1:27" ht="32" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>23</v>
@@ -2502,44 +2619,44 @@
       <c r="D9" s="4">
         <v>5</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="G9" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="H9" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="I9" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="J9" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="J9" s="4" t="s">
+      <c r="K9" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="K9" s="4" t="s">
-        <v>171</v>
-      </c>
       <c r="L9" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="M9" s="4">
         <v>0.03</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O9" s="4">
         <v>0</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Q9" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="R9" s="4" t="s">
         <v>25</v>
@@ -2548,21 +2665,18 @@
         <v>1</v>
       </c>
       <c r="T9" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="U9" s="4" t="s">
         <v>152</v>
-      </c>
-      <c r="U9" s="4" t="s">
-        <v>153</v>
       </c>
       <c r="V9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="W9" s="4" t="s">
+      <c r="W9" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="X9" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="4">
+      <c r="Z9" s="4">
         <v>-7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
merged 2 neg/pos cases into 1
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,23 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E7740AA-0655-9B41-B718-B8734C1195B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF3A9EE3-1E82-6E4E-B797-42E3A65AA09E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
     <sheet name="Datasets" sheetId="2" r:id="rId2"/>
     <sheet name="Validation" sheetId="12" r:id="rId3"/>
     <sheet name="dm.xpt" sheetId="10" r:id="rId4"/>
-    <sheet name="lb.xpt" sheetId="11" r:id="rId5"/>
+    <sheet name="lb1.xpt" sheetId="11" r:id="rId5"/>
+    <sheet name="lb2.xpt" sheetId="13" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="190">
   <si>
     <t>Product</t>
   </si>
@@ -548,9 +549,6 @@
     <t>Start Date/Time of Specimen Collection</t>
   </si>
   <si>
-    <t>lb.xpt</t>
-  </si>
-  <si>
     <t>Laboratory Test Results</t>
   </si>
   <si>
@@ -582,13 +580,28 @@
   </si>
   <si>
     <t>[ABSENT]</t>
+  </si>
+  <si>
+    <t>lb2.xpt</t>
+  </si>
+  <si>
+    <t>lb1.xpt</t>
+  </si>
+  <si>
+    <t>Date/Time of Specimen Collection</t>
+  </si>
+  <si>
+    <t>2012-11-23T15:39:00</t>
+  </si>
+  <si>
+    <t>2012-11-24T15:39:00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -617,6 +630,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -689,7 +709,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -713,7 +733,10 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1044,7 +1067,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -1065,10 +1088,18 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B3" t="s">
         <v>174</v>
       </c>
-      <c r="B3" t="s">
-        <v>175</v>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B4" t="s">
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -1078,27 +1109,30 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC590268-A813-7E46-A402-7CCF030F7149}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="6" max="6" width="17.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="C1" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="D1" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="E1" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="F1" s="10" t="s">
         <v>181</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1106,10 +1140,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D2">
         <v>5</v>
@@ -1126,19 +1160,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E3" t="s">
         <v>117</v>
       </c>
       <c r="F3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1146,10 +1180,10 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D4">
         <v>5</v>
@@ -1166,10 +1200,10 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D5">
         <v>6</v>
@@ -1177,8 +1211,8 @@
       <c r="E5" t="s">
         <v>118</v>
       </c>
-      <c r="F5" s="11" t="s">
-        <v>176</v>
+      <c r="F5" s="4" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -1186,19 +1220,19 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E6" t="s">
         <v>117</v>
       </c>
       <c r="F6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1206,10 +1240,10 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D7">
         <v>6</v>
@@ -1217,7 +1251,7 @@
       <c r="E7" t="s">
         <v>101</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="4" t="s">
         <v>153</v>
       </c>
     </row>
@@ -1226,10 +1260,10 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C8" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D8">
         <v>7</v>
@@ -1237,8 +1271,8 @@
       <c r="E8" t="s">
         <v>118</v>
       </c>
-      <c r="F8" s="11" t="s">
-        <v>176</v>
+      <c r="F8" s="4" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -1246,19 +1280,19 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E9" t="s">
         <v>117</v>
       </c>
       <c r="F9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1266,10 +1300,10 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D10">
         <v>7</v>
@@ -1286,10 +1320,10 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D11">
         <v>8</v>
@@ -1297,8 +1331,8 @@
       <c r="E11" t="s">
         <v>118</v>
       </c>
-      <c r="F11" s="11" t="s">
-        <v>176</v>
+      <c r="F11" s="4" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -1306,19 +1340,19 @@
         <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C12" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E12" t="s">
         <v>117</v>
       </c>
       <c r="F12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1326,10 +1360,10 @@
         <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C13" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D13">
         <v>8</v>
@@ -1337,7 +1371,7 @@
       <c r="E13" t="s">
         <v>101</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="4" t="s">
         <v>153</v>
       </c>
     </row>
@@ -1346,10 +1380,10 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D14">
         <v>9</v>
@@ -1366,19 +1400,19 @@
         <v>5</v>
       </c>
       <c r="B15" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E15" t="s">
         <v>117</v>
       </c>
       <c r="F15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1386,10 +1420,10 @@
         <v>5</v>
       </c>
       <c r="B16" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C16" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D16">
         <v>9</v>
@@ -1398,6 +1432,120 @@
         <v>101</v>
       </c>
       <c r="F16" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>6</v>
+      </c>
+      <c r="B17" t="s">
+        <v>185</v>
+      </c>
+      <c r="C17" t="s">
+        <v>182</v>
+      </c>
+      <c r="D17">
+        <v>6</v>
+      </c>
+      <c r="E17" t="s">
+        <v>118</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>6</v>
+      </c>
+      <c r="B18" t="s">
+        <v>185</v>
+      </c>
+      <c r="C18" t="s">
+        <v>182</v>
+      </c>
+      <c r="D18">
+        <v>6</v>
+      </c>
+      <c r="E18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>6</v>
+      </c>
+      <c r="B19" t="s">
+        <v>185</v>
+      </c>
+      <c r="C19" t="s">
+        <v>182</v>
+      </c>
+      <c r="D19">
+        <v>6</v>
+      </c>
+      <c r="E19" t="s">
+        <v>101</v>
+      </c>
+      <c r="F19" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>7</v>
+      </c>
+      <c r="B20" t="s">
+        <v>185</v>
+      </c>
+      <c r="C20" t="s">
+        <v>182</v>
+      </c>
+      <c r="D20">
+        <v>9</v>
+      </c>
+      <c r="E20" t="s">
+        <v>118</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>7</v>
+      </c>
+      <c r="B21" t="s">
+        <v>185</v>
+      </c>
+      <c r="C21" t="s">
+        <v>182</v>
+      </c>
+      <c r="D21">
+        <v>9</v>
+      </c>
+      <c r="E21" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>7</v>
+      </c>
+      <c r="B22" t="s">
+        <v>185</v>
+      </c>
+      <c r="C22" t="s">
+        <v>182</v>
+      </c>
+      <c r="D22">
+        <v>9</v>
+      </c>
+      <c r="E22" t="s">
+        <v>101</v>
+      </c>
+      <c r="F22" t="s">
         <v>164</v>
       </c>
     </row>
@@ -2443,7 +2591,7 @@
         <v>27</v>
       </c>
       <c r="W6" s="9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="X6" s="4" t="s">
         <v>24</v>
@@ -2517,10 +2665,10 @@
         <v>152</v>
       </c>
       <c r="V7" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="W7" s="9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="Y7" s="4" t="s">
         <v>151</v>
@@ -2594,7 +2742,7 @@
         <v>27</v>
       </c>
       <c r="W8" s="9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="X8" s="4" t="s">
         <v>24</v>
@@ -2677,6 +2825,738 @@
         <v>27</v>
       </c>
       <c r="Z9" s="4">
+        <v>-7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42B766EC-C098-2042-ABBF-939A895C2D4F}">
+  <dimension ref="A1:AA9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:27" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="N1" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="O1" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="P1" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q1" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="R1" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="S1" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="T1" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="U1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="V1" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="W1" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="X1" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AA1" s="7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" ht="80" x14ac:dyDescent="0.2">
+      <c r="A2" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="M2" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="N2" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="P2" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="Q2" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="R2" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="S2" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="T2" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="U2" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="V2" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="W2" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="X2" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA2" s="8" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="P3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="R3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="S3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="T3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="U3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="V3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="W3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="X3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA3" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A4" s="8">
+        <v>12</v>
+      </c>
+      <c r="B4" s="8">
+        <v>2</v>
+      </c>
+      <c r="C4" s="8">
+        <v>8</v>
+      </c>
+      <c r="D4" s="8">
+        <v>8</v>
+      </c>
+      <c r="E4" s="8">
+        <v>7</v>
+      </c>
+      <c r="F4" s="8">
+        <v>39</v>
+      </c>
+      <c r="G4" s="8">
+        <v>10</v>
+      </c>
+      <c r="H4" s="8">
+        <v>6</v>
+      </c>
+      <c r="I4" s="8">
+        <v>7</v>
+      </c>
+      <c r="J4" s="8">
+        <v>200</v>
+      </c>
+      <c r="K4" s="8">
+        <v>200</v>
+      </c>
+      <c r="L4" s="8">
+        <v>8</v>
+      </c>
+      <c r="M4" s="8">
+        <v>8</v>
+      </c>
+      <c r="N4" s="8">
+        <v>7</v>
+      </c>
+      <c r="O4" s="8">
+        <v>8</v>
+      </c>
+      <c r="P4" s="8">
+        <v>8</v>
+      </c>
+      <c r="Q4" s="8">
+        <v>8</v>
+      </c>
+      <c r="R4" s="8">
+        <v>1</v>
+      </c>
+      <c r="S4" s="8">
+        <v>8</v>
+      </c>
+      <c r="T4" s="8">
+        <v>200</v>
+      </c>
+      <c r="U4" s="8">
+        <v>9</v>
+      </c>
+      <c r="V4" s="8">
+        <v>19</v>
+      </c>
+      <c r="W4" s="8">
+        <v>19</v>
+      </c>
+      <c r="X4" s="8">
+        <v>19</v>
+      </c>
+      <c r="Y4" s="3">
+        <v>50</v>
+      </c>
+      <c r="Z4" s="3">
+        <v>50</v>
+      </c>
+      <c r="AA4" s="8">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" ht="48" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="4">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="M5" s="4">
+        <v>39</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="Q5" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="R5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="S5" s="4">
+        <v>1</v>
+      </c>
+      <c r="T5" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="U5" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="V5" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="W5" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="X5" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="Y5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z5" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="AA5" s="4">
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" ht="48" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="4">
+        <v>2</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="M6" s="4">
+        <v>93</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="O6" s="4">
+        <v>35</v>
+      </c>
+      <c r="P6" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="Q6" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="R6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="S6" s="4">
+        <v>1</v>
+      </c>
+      <c r="T6" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="U6" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="V6" s="9"/>
+      <c r="W6" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="X6" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="Y6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z6" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="AA6" s="4">
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" ht="48" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="4">
+        <v>3</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="M7" s="4">
+        <v>18</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="O7" s="4">
+        <v>6</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="R7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="S7" s="4">
+        <v>1</v>
+      </c>
+      <c r="T7" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="U7" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="V7" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="W7" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="X7" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="Z7" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="AA7" s="4">
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" ht="48" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="4">
+        <v>4</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="M8" s="4">
+        <v>26</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="P8" s="4">
+        <v>36</v>
+      </c>
+      <c r="Q8" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="R8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="S8" s="4">
+        <v>1</v>
+      </c>
+      <c r="T8" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="U8" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="V8" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="W8" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="X8" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="Y8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z8" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="AA8" s="4">
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" ht="48" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="4">
+        <v>5</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="M9" s="4">
+        <v>0.03</v>
+      </c>
+      <c r="N9" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="O9" s="4">
+        <v>0</v>
+      </c>
+      <c r="P9" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="Q9" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="R9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="S9" s="4">
+        <v>1</v>
+      </c>
+      <c r="T9" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="U9" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="V9" s="9"/>
+      <c r="W9" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="X9" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="AA9" s="4">
         <v>-7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
included negative case where STINT variable is missing
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B959EADE-457D-9143-8739-A5A9AB4D22C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4424E9B-69CE-DA47-97C7-9FB6A859AE2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,15 @@
     <sheet name="Library" sheetId="1" r:id="rId1"/>
     <sheet name="Datasets" sheetId="2" r:id="rId2"/>
     <sheet name="Validation" sheetId="4" r:id="rId3"/>
-    <sheet name="lb.xpt" sheetId="3" r:id="rId4"/>
+    <sheet name="lb1.xpt" sheetId="3" r:id="rId4"/>
+    <sheet name="lb2.xpt" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="122">
   <si>
     <t>Product</t>
   </si>
@@ -37,9 +38,6 @@
     <t>Label</t>
   </si>
   <si>
-    <t>lb.xpt</t>
-  </si>
-  <si>
     <t>Laboratory Test Results</t>
   </si>
   <si>
@@ -383,6 +381,15 @@
   </si>
   <si>
     <t>Record</t>
+  </si>
+  <si>
+    <t>lb1.xpt</t>
+  </si>
+  <si>
+    <t>lb2.xpt</t>
+  </si>
+  <si>
+    <t>[ABSENT]</t>
   </si>
 </sst>
 </file>
@@ -805,10 +812,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B2" t="s">
         <v>111</v>
-      </c>
-      <c r="B2" t="s">
-        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -818,7 +825,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -831,10 +838,18 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
-        <v>5</v>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -844,27 +859,27 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{353FE4AE-AFB5-ED48-906A-FF16EB0A6114}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>117</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -872,19 +887,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>119</v>
       </c>
       <c r="C2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D2">
         <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -892,16 +907,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>119</v>
       </c>
       <c r="C3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D3">
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -909,19 +924,19 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>119</v>
       </c>
       <c r="C4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D4">
         <v>7</v>
       </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -929,16 +944,136 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>119</v>
       </c>
       <c r="C5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D5">
         <v>7</v>
       </c>
       <c r="E5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6" t="s">
         <v>35</v>
+      </c>
+      <c r="F6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>120</v>
+      </c>
+      <c r="C7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8">
+        <v>6</v>
+      </c>
+      <c r="E8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>120</v>
+      </c>
+      <c r="C9" t="s">
+        <v>116</v>
+      </c>
+      <c r="D9">
+        <v>6</v>
+      </c>
+      <c r="E9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>120</v>
+      </c>
+      <c r="C10" t="s">
+        <v>118</v>
+      </c>
+      <c r="D10">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C11" t="s">
+        <v>116</v>
+      </c>
+      <c r="D11">
+        <v>7</v>
+      </c>
+      <c r="E11" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -953,296 +1088,296 @@
   <sheetData>
     <row r="1" spans="1:32" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AB1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AC1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AD1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AF1" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="AF1" s="3" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:32" ht="96" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="N2" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="O2" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="P2" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="Q2" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="R2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="S2" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="S2" s="5" t="s">
+      <c r="T2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="V2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="W2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="X2" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="Y2" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="Y2" s="4" t="s">
+      <c r="Z2" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="Z2" s="4" t="s">
+      <c r="AA2" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="AA2" s="4" t="s">
+      <c r="AB2" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="AB2" s="4" t="s">
+      <c r="AC2" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="AC2" s="4" t="s">
+      <c r="AD2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="AD2" s="4" t="s">
+      <c r="AE2" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AE2" s="4" t="s">
+      <c r="AF2" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="AF2" s="4" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:32" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="E3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="M3" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="N3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="O3" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="E3" s="4" t="s">
+      <c r="P3" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="Q3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="U3" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="V3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="W3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="X3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="Y3" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="Z3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="AA3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="AB3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="AC3" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="I3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="O3" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="P3" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="R3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="S3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="T3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="U3" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="V3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="W3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="X3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="Y3" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="Z3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="AA3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="AB3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="AC3" s="4" t="s">
-        <v>71</v>
-      </c>
       <c r="AD3" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AE3" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AF3" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:32" ht="16" x14ac:dyDescent="0.2">
@@ -1331,13 +1466,13 @@
         <v>50</v>
       </c>
       <c r="AC4" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="AD4" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="AD4" s="4" t="s">
-        <v>73</v>
-      </c>
       <c r="AE4" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF4" s="4">
         <v>100</v>
@@ -1345,46 +1480,46 @@
     </row>
     <row r="5" spans="1:32" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="6" t="s">
         <v>75</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>76</v>
       </c>
       <c r="D5" s="6">
         <v>1</v>
       </c>
       <c r="E5" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="I5" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="J5" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="K5" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="K5" s="6" t="s">
+      <c r="L5" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="L5" s="6" t="s">
-        <v>84</v>
       </c>
       <c r="M5" s="6">
         <v>39</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="O5" s="6">
         <v>35</v>
@@ -1393,22 +1528,22 @@
         <v>46</v>
       </c>
       <c r="Q5" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="T5" s="6" t="s">
         <v>86</v>
-      </c>
-      <c r="T5" s="6" t="s">
-        <v>87</v>
       </c>
       <c r="U5" s="6">
         <v>1</v>
       </c>
       <c r="V5" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="W5" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="W5" s="6" t="s">
+      <c r="X5" s="6" t="s">
         <v>89</v>
-      </c>
-      <c r="X5" s="6" t="s">
-        <v>90</v>
       </c>
       <c r="Y5" s="6">
         <v>-7</v>
@@ -1417,61 +1552,61 @@
         <v>3</v>
       </c>
       <c r="AB5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AC5" s="2">
         <v>1</v>
       </c>
       <c r="AD5" s="9"/>
       <c r="AE5" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="AF5" t="s">
         <v>93</v>
-      </c>
-      <c r="AF5" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:32" ht="48" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="C6" s="6" t="s">
         <v>75</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>76</v>
       </c>
       <c r="D6" s="6">
         <v>2</v>
       </c>
       <c r="E6" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H6" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="H6" s="6" t="s">
+      <c r="I6" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="J6" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="K6" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="K6" s="6" t="s">
-        <v>100</v>
-      </c>
       <c r="L6" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M6" s="6">
         <v>93</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O6" s="6">
         <v>35</v>
@@ -1480,22 +1615,22 @@
         <v>115</v>
       </c>
       <c r="Q6" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="T6" s="6" t="s">
         <v>86</v>
-      </c>
-      <c r="T6" s="6" t="s">
-        <v>87</v>
       </c>
       <c r="U6" s="6">
         <v>1</v>
       </c>
       <c r="V6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="W6" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="W6" s="6" t="s">
+      <c r="X6" s="6" t="s">
         <v>89</v>
-      </c>
-      <c r="X6" s="6" t="s">
-        <v>90</v>
       </c>
       <c r="Y6" s="6">
         <v>-7</v>
@@ -1504,167 +1639,816 @@
         <v>2</v>
       </c>
       <c r="AB6" t="s">
+        <v>100</v>
+      </c>
+      <c r="AC6" s="2" t="s">
         <v>101</v>
       </c>
+      <c r="AD6" t="s">
+        <v>91</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>92</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32" ht="48" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="N7" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="O7" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="P7" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="T7" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="U7" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="V7" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="W7" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="X7" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y7" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="Z7" s="7"/>
+      <c r="AA7" t="s">
+        <v>105</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>106</v>
+      </c>
+      <c r="AC7" s="2">
+        <v>3</v>
+      </c>
+      <c r="AD7" s="9"/>
+      <c r="AE7" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32" ht="48" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="R8" t="s">
+        <v>107</v>
+      </c>
+      <c r="S8" t="s">
+        <v>108</v>
+      </c>
+      <c r="U8" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="V8" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="W8" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="X8" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="Y8" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="Z8" s="7"/>
+      <c r="AB8" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC8" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>91</v>
+      </c>
+      <c r="AE8" t="s">
+        <v>92</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93FFA24A-A2C7-E749-AD0D-54B47C47A796}">
+  <dimension ref="A1:AE7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:31" ht="32" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="W1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="AC1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="AD1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="AE1" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" ht="96" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="U2" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="V2" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="W2" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="X2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y2" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z2" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA2" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="AB2" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="AC2" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD2" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AE2" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="W3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="X3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="Y3" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="Z3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="AA3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="AB3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="AC3" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="AD3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="AE3" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="4">
+        <v>12</v>
+      </c>
+      <c r="B4" s="4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="4">
+        <v>8</v>
+      </c>
+      <c r="D4" s="4">
+        <v>8</v>
+      </c>
+      <c r="E4" s="4">
+        <v>7</v>
+      </c>
+      <c r="F4" s="4">
+        <v>39</v>
+      </c>
+      <c r="G4" s="4">
+        <v>10</v>
+      </c>
+      <c r="H4" s="4">
+        <v>6</v>
+      </c>
+      <c r="I4" s="4">
+        <v>7</v>
+      </c>
+      <c r="J4" s="4">
+        <v>200</v>
+      </c>
+      <c r="K4" s="4">
+        <v>200</v>
+      </c>
+      <c r="L4" s="4">
+        <v>8</v>
+      </c>
+      <c r="M4" s="4">
+        <v>8</v>
+      </c>
+      <c r="N4" s="4">
+        <v>7</v>
+      </c>
+      <c r="O4" s="4">
+        <v>8</v>
+      </c>
+      <c r="P4" s="4">
+        <v>8</v>
+      </c>
+      <c r="Q4" s="4">
+        <v>8</v>
+      </c>
+      <c r="R4" s="4">
+        <v>8</v>
+      </c>
+      <c r="S4" s="4">
+        <v>50</v>
+      </c>
+      <c r="T4" s="4">
+        <v>1</v>
+      </c>
+      <c r="U4" s="4">
+        <v>8</v>
+      </c>
+      <c r="V4" s="4">
+        <v>200</v>
+      </c>
+      <c r="W4" s="4">
+        <v>9</v>
+      </c>
+      <c r="X4" s="4">
+        <v>19</v>
+      </c>
+      <c r="Y4" s="4">
+        <v>8</v>
+      </c>
+      <c r="Z4" s="4">
+        <v>50</v>
+      </c>
+      <c r="AA4" s="4">
+        <v>50</v>
+      </c>
+      <c r="AB4" s="4">
+        <v>50</v>
+      </c>
+      <c r="AC4" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="AD4" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="AE4" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31" ht="32" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="D5" s="6">
+        <v>1</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="M5" s="6">
+        <v>39</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="O5" s="6">
+        <v>35</v>
+      </c>
+      <c r="P5" s="6">
+        <v>46</v>
+      </c>
+      <c r="Q5" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="T5" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="U5" s="6">
+        <v>1</v>
+      </c>
+      <c r="V5" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="W5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="X5" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y5" s="6">
+        <v>-7</v>
+      </c>
+      <c r="AA5">
+        <v>3</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC5" s="2">
+        <v>1</v>
+      </c>
+      <c r="AD5" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6" spans="1:31" ht="48" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="D6" s="6">
+        <v>2</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="M6" s="6">
+        <v>93</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="O6" s="6">
+        <v>35</v>
+      </c>
+      <c r="P6" s="6">
+        <v>115</v>
+      </c>
+      <c r="Q6" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="T6" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="U6" s="6">
+        <v>1</v>
+      </c>
+      <c r="V6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="W6" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="X6" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y6" s="6">
+        <v>-7</v>
+      </c>
+      <c r="AA6">
+        <v>2</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>100</v>
+      </c>
       <c r="AC6" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="AD6" t="s">
+        <v>101</v>
+      </c>
+      <c r="AD6" s="9" t="s">
         <v>92</v>
       </c>
       <c r="AE6" t="s">
         <v>93</v>
       </c>
-      <c r="AF6" t="s">
+    </row>
+    <row r="7" spans="1:31" ht="48" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E7" s="7" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="7" spans="1:32" ht="48" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C7" s="7" t="s">
+      <c r="F7" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="N7" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="O7" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="P7" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="T7" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="U7" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="K7" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="L7" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="M7" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="N7" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="O7" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="P7" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="Q7" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="T7" s="7" t="s">
+      <c r="V7" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="U7" s="7" t="s">
+      <c r="W7" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="X7" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y7" s="7" t="s">
         <v>104</v>
-      </c>
-      <c r="V7" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="W7" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="X7" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="Y7" s="7" t="s">
-        <v>105</v>
       </c>
       <c r="Z7" s="7"/>
       <c r="AA7" t="s">
+        <v>105</v>
+      </c>
+      <c r="AB7" t="s">
         <v>106</v>
-      </c>
-      <c r="AB7" t="s">
-        <v>107</v>
       </c>
       <c r="AC7" s="2">
         <v>3</v>
       </c>
-      <c r="AD7" s="9"/>
-      <c r="AE7" s="9" t="s">
+      <c r="AD7" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="AE7" t="s">
         <v>93</v>
-      </c>
-      <c r="AF7" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="8" spans="1:32" ht="48" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="R8" t="s">
-        <v>108</v>
-      </c>
-      <c r="S8" t="s">
-        <v>109</v>
-      </c>
-      <c r="U8" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="V8" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="W8" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="X8" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="Y8" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="Z8" s="7"/>
-      <c r="AB8" t="s">
-        <v>91</v>
-      </c>
-      <c r="AC8" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="AD8" t="s">
-        <v>92</v>
-      </c>
-      <c r="AE8" t="s">
-        <v>93</v>
-      </c>
-      <c r="AF8" t="s">
-        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
race instead of ethnic
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -457,18 +457,18 @@
   <dimension ref="A1:B2"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
+      <c r="A1" s="3" t="str">
         <v>Product</v>
       </c>
-      <c r="B1" s="2" t="str">
+      <c r="B1" s="3" t="str">
         <v>Version</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="3" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="3" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -484,26 +484,26 @@
   <dimension ref="A1:B3"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
+      <c r="A1" s="3" t="str">
         <v>Filename</v>
       </c>
-      <c r="B1" s="2" t="str">
+      <c r="B1" s="3" t="str">
         <v>Label</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="3" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="3" t="str">
         <v>Demographics</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="3" t="str">
         <v>suppdm.xpt</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="3" t="str">
         <v>Supplemental Qualifiers for Demographics</v>
       </c>
     </row>
@@ -519,103 +519,103 @@
   <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
+      <c r="A1" s="3" t="str">
         <v>Error group</v>
       </c>
-      <c r="B1" s="2" t="str">
+      <c r="B1" s="3" t="str">
         <v>Sheet</v>
       </c>
-      <c r="C1" s="2" t="str">
+      <c r="C1" s="3" t="str">
         <v>Error level</v>
       </c>
-      <c r="D1" s="2" t="str">
+      <c r="D1" s="3" t="str">
         <v>Row num</v>
       </c>
-      <c r="E1" s="2" t="str">
+      <c r="E1" s="3" t="str">
         <v>Variable</v>
       </c>
-      <c r="F1" s="2" t="str">
+      <c r="F1" s="3" t="str">
         <v>Error value</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="3" t="str">
         <v>Variable</v>
       </c>
-      <c r="D2" s="2" t="str">
+      <c r="D2" s="3" t="str">
         <v>N/A</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="3" t="str">
         <v>define_variable_name</v>
       </c>
-      <c r="F2" s="2" t="str">
-        <v>ETHNIC</v>
+      <c r="F2" s="3" t="str">
+        <v>RACE</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="3">
         <v>1</v>
       </c>
       <c r="B3" s="3" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="3" t="str">
         <v>Variable</v>
       </c>
-      <c r="D3" s="2" t="str">
+      <c r="D3" s="3" t="str">
         <v>N/A</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E3" s="3" t="str">
         <v>define_variable_codelist_coded_values</v>
       </c>
-      <c r="F3" s="2" t="str">
-        <v>HISPANIC OR LATINO</v>
+      <c r="F3" s="3" t="str">
+        <v>ASIAN,BLACK OR AFRICAN AMERICAN,NATIVE HAWAIIAN OR OTHER PACIFIC ISLANDER,WHITE</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
+      <c r="A4" s="3">
         <v>2</v>
       </c>
       <c r="B4" s="3" t="str">
         <v>suppdm.xpt</v>
       </c>
-      <c r="C4" s="2" t="str">
+      <c r="C4" s="3" t="str">
         <v>Variable</v>
       </c>
-      <c r="D4" s="2" t="str">
+      <c r="D4" s="3" t="str">
         <v>N/A</v>
       </c>
-      <c r="E4" s="2" t="str">
+      <c r="E4" s="3" t="str">
         <v>define_variable_name</v>
       </c>
-      <c r="F4" s="2" t="str">
-        <v>CETHNIC</v>
+      <c r="F4" s="3" t="str">
+        <v>CRACE</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2">
+      <c r="A5" s="3">
         <v>2</v>
       </c>
       <c r="B5" s="3" t="str">
         <v>suppdm.xpt</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C5" s="3" t="str">
         <v>Variable</v>
       </c>
-      <c r="D5" s="2" t="str">
+      <c r="D5" s="3" t="str">
         <v>N/A</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E5" s="3" t="str">
         <v>define_variable_codelist_coded_values</v>
       </c>
-      <c r="F5" s="2" t="str">
-        <v>HISPANIC OR LATINO</v>
+      <c r="F5" s="3" t="str">
+        <v>ASIAN,BLACK OR AFRICAN AMERICAN,NATIVE HAWAIIAN OR OTHER PACIFIC ISLANDER,WHITE"</v>
       </c>
     </row>
   </sheetData>
@@ -667,7 +667,7 @@
         <v>DTHFL</v>
       </c>
       <c r="M1" s="4" t="str">
-        <v>ETHNIC</v>
+        <v>RACE</v>
       </c>
     </row>
     <row r="2">
@@ -708,7 +708,7 @@
         <v>Subject Death Flag</v>
       </c>
       <c r="M2" s="6" t="str">
-        <v>Ethnicity</v>
+        <v>Race</v>
       </c>
     </row>
     <row r="3">
@@ -830,8 +830,8 @@
       <c r="L5" s="7" t="str">
         <v>Y</v>
       </c>
-      <c r="M5" s="2" t="str">
-        <v>HISPANIC OR LATINO</v>
+      <c r="M5" s="3" t="str">
+        <v>WHITE</v>
       </c>
     </row>
   </sheetData>
@@ -990,13 +990,13 @@
         <v>1</v>
       </c>
       <c r="F5" s="7" t="str">
-        <v>CETHNIC</v>
+        <v>CRACE</v>
       </c>
       <c r="G5" s="7" t="str">
-        <v>Ethnicity</v>
+        <v>Race</v>
       </c>
       <c r="H5" s="7" t="str">
-        <v>HISPANIC OR LATINO</v>
+        <v>WHITE</v>
       </c>
       <c r="I5" s="7" t="str">
         <v>CRF</v>

</xml_diff>

<commit_message>
added output variables and improved test cases
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D02EFB7-7C3F-CC41-ADD2-5AB80C1DFEDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B9BA9F0-E321-3445-B073-6053459672B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="216">
   <si>
     <t>Product</t>
   </si>
@@ -641,6 +641,36 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>STYPE1</t>
+  </si>
+  <si>
+    <t>STYPE2</t>
+  </si>
+  <si>
+    <t>OTHER</t>
+  </si>
+  <si>
+    <t>INTMODEL</t>
+  </si>
+  <si>
+    <t>Intervention Model</t>
+  </si>
+  <si>
+    <t>PARALLEL</t>
+  </si>
+  <si>
+    <t>C82639</t>
+  </si>
+  <si>
+    <t>Dataset</t>
+  </si>
+  <si>
+    <t>$STYPE_INTERVENTIONAL</t>
+  </si>
+  <si>
+    <t>Record</t>
   </si>
 </sst>
 </file>
@@ -676,7 +706,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -689,8 +719,14 @@
         <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -713,11 +749,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -730,11 +777,14 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1091,7 +1141,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CA1A07C-A03C-3740-B416-1DF5B7F6AA7A}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -1122,16 +1172,76 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>203</v>
-      </c>
-      <c r="D2" t="s">
+        <v>215</v>
+      </c>
+      <c r="D2">
+        <v>47</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D3">
+        <v>47</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>215</v>
+      </c>
+      <c r="D4">
+        <v>47</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>213</v>
+      </c>
+      <c r="D5" t="s">
         <v>205</v>
       </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" t="s">
-        <v>31</v>
+      <c r="E5" t="s">
+        <v>214</v>
+      </c>
+      <c r="F5" s="7">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1141,11 +1251,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -1285,7 +1395,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="64" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B5" s="4" t="s">
@@ -1714,17 +1824,16 @@
       <c r="C22" s="4">
         <v>1</v>
       </c>
-      <c r="D22" s="6"/>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="G22" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="H22" s="7" t="s">
+      <c r="H22" s="4" t="s">
         <v>198</v>
       </c>
       <c r="I22" s="4" t="s">
@@ -1747,19 +1856,20 @@
       <c r="C23" s="4">
         <v>1</v>
       </c>
-      <c r="D23" s="6"/>
-      <c r="E23" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="H23" s="6"/>
+      <c r="D23" t="s">
+        <v>207</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>211</v>
+      </c>
       <c r="I23" s="4" t="s">
-        <v>99</v>
+        <v>212</v>
       </c>
       <c r="J23" s="4" t="s">
         <v>40</v>
@@ -1778,60 +1888,69 @@
       <c r="C24" s="4">
         <v>1</v>
       </c>
+      <c r="D24" t="s">
+        <v>207</v>
+      </c>
       <c r="E24" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A25" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="4">
+        <v>1</v>
+      </c>
+      <c r="E25" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F25" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G25" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="J24" s="4" t="s">
+      <c r="J25" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A25" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C25" s="4">
-        <v>1</v>
-      </c>
-      <c r="E25" s="4" t="s">
+    <row r="26" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A26" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" s="4">
+        <v>1</v>
+      </c>
+      <c r="E26" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F26" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G26" s="4" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="112" x14ac:dyDescent="0.2">
-      <c r="A26" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C26" s="4">
-        <v>1</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="112" x14ac:dyDescent="0.2">
@@ -1842,10 +1961,10 @@
         <v>32</v>
       </c>
       <c r="C27" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>106</v>
@@ -1854,33 +1973,33 @@
         <v>107</v>
       </c>
       <c r="G27" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="112" x14ac:dyDescent="0.2">
+      <c r="A28" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" s="4">
+        <v>2</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="G28" s="4" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C28" s="4">
-        <v>1</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="365" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>31</v>
       </c>
@@ -1888,7 +2007,7 @@
         <v>32</v>
       </c>
       <c r="C29" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>105</v>
@@ -1900,18 +2019,18 @@
         <v>112</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="335" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="365" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C30" s="4" t="s">
-        <v>70</v>
+      <c r="C30" s="4">
+        <v>2</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>105</v>
@@ -1923,10 +2042,10 @@
         <v>112</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="128" x14ac:dyDescent="0.2">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="335" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>31</v>
       </c>
@@ -1934,10 +2053,10 @@
         <v>32</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>116</v>
+        <v>70</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>111</v>
@@ -1946,10 +2065,10 @@
         <v>112</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" ht="112" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>31</v>
       </c>
@@ -1957,7 +2076,7 @@
         <v>32</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>109</v>
@@ -1969,33 +2088,30 @@
         <v>112</v>
       </c>
       <c r="G32" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="112" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="G33" s="4" t="s">
         <v>119</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" ht="64" x14ac:dyDescent="0.2">
-      <c r="A33" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C33" s="4">
-        <v>1</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="G33" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="I33" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="J33" s="4" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="64" x14ac:dyDescent="0.2">
@@ -2009,42 +2125,39 @@
         <v>1</v>
       </c>
       <c r="E34" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J34" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+      <c r="A35" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C35" s="4">
+        <v>1</v>
+      </c>
+      <c r="E35" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="F35" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="G34" s="4" t="s">
+      <c r="G35" s="4" t="s">
         <v>127</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A35" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35" s="4">
-        <v>1</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="G35" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="I35" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J35" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K35" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="48" x14ac:dyDescent="0.2">
@@ -2058,88 +2171,97 @@
         <v>1</v>
       </c>
       <c r="E36" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J36" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K36" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C37" s="4">
+        <v>1</v>
+      </c>
+      <c r="E37" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="F36" s="4" t="s">
+      <c r="F37" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="G36" s="4" t="s">
+      <c r="G37" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A37" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C37" s="4">
-        <v>1</v>
-      </c>
-      <c r="E37" s="4" t="s">
+    <row r="38" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A38" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" s="4">
+        <v>1</v>
+      </c>
+      <c r="E38" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="F38" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="G38" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="I37" s="4" t="s">
+      <c r="I38" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="J37" s="4" t="s">
+      <c r="J38" s="4" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A38" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C38" s="4">
-        <v>1</v>
-      </c>
-      <c r="E38" s="4" t="s">
+    <row r="39" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A39" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C39" s="4">
+        <v>1</v>
+      </c>
+      <c r="E39" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="F38" s="4" t="s">
+      <c r="F39" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="G38" s="4" t="s">
+      <c r="G39" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="I38" s="4" t="s">
+      <c r="I39" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="J38" s="4" t="s">
+      <c r="J39" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K38" s="4" t="s">
+      <c r="K39" s="4" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A39" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C39" s="4">
-        <v>1</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="F39" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="G39" s="4" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="32" x14ac:dyDescent="0.2">
@@ -2153,13 +2275,13 @@
         <v>1</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="32" x14ac:dyDescent="0.2">
@@ -2173,160 +2295,154 @@
         <v>1</v>
       </c>
       <c r="E41" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A42" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C42" s="4">
+        <v>1</v>
+      </c>
+      <c r="E42" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="F41" s="4" t="s">
+      <c r="F42" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="G41" s="4" t="s">
+      <c r="G42" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="J41" s="4" t="s">
+      <c r="J42" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A42" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C42" s="4">
-        <v>1</v>
-      </c>
-      <c r="E42" s="4" t="s">
+    <row r="43" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A43" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C43" s="4">
+        <v>1</v>
+      </c>
+      <c r="E43" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="F42" s="4" t="s">
+      <c r="F43" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="G42" s="4" t="s">
+      <c r="G43" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="I42" s="4" t="s">
+      <c r="I43" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="J42" s="4" t="s">
+      <c r="J43" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K42" s="4" t="s">
+      <c r="K43" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="96" x14ac:dyDescent="0.2">
-      <c r="A43" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C43" s="4">
-        <v>1</v>
-      </c>
-      <c r="E43" s="4" t="s">
+    <row r="44" spans="1:11" ht="96" x14ac:dyDescent="0.2">
+      <c r="A44" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C44" s="4">
+        <v>1</v>
+      </c>
+      <c r="E44" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="F43" s="4" t="s">
+      <c r="F44" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="G43" s="4" t="s">
+      <c r="G44" s="4" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A44" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C44" s="4">
-        <v>1</v>
-      </c>
-      <c r="E44" s="4" t="s">
+    <row r="45" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A45" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C45" s="4">
+        <v>1</v>
+      </c>
+      <c r="E45" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="F44" s="4" t="s">
+      <c r="F45" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="G44" s="4" t="s">
+      <c r="G45" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="J44" s="4" t="s">
+      <c r="J45" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A45" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C45" s="4">
-        <v>1</v>
-      </c>
-      <c r="E45" s="4" t="s">
+    <row r="46" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A46" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C46" s="4">
+        <v>1</v>
+      </c>
+      <c r="E46" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="F45" s="4" t="s">
+      <c r="F46" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="G45" s="4" t="s">
+      <c r="G46" s="4" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A46" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C46" s="4">
-        <v>1</v>
-      </c>
-      <c r="E46" s="4" t="s">
+    <row r="47" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A47" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C47" s="4">
+        <v>1</v>
+      </c>
+      <c r="D47" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="E47" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="F46" s="4" t="s">
+      <c r="F47" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="G46" s="4" t="s">
+      <c r="G47" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="I46" s="4" t="s">
+      <c r="I47" s="4" t="s">
         <v>166</v>
-      </c>
-      <c r="J46" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K46" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A47" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C47" s="4">
-        <v>1</v>
-      </c>
-      <c r="E47" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="F47" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="G47" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="I47" s="4" t="s">
-        <v>170</v>
       </c>
       <c r="J47" s="4" t="s">
         <v>40</v>
@@ -2342,20 +2458,23 @@
       <c r="B48" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C48" s="4">
-        <v>1</v>
+      <c r="C48" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>207</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>63</v>
+        <v>208</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="J48" s="4" t="s">
         <v>40</v>
@@ -2364,7 +2483,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="112" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>31</v>
       </c>
@@ -2375,20 +2494,25 @@
         <v>1</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="H49" s="4"/>
-      <c r="I49" s="4"/>
-      <c r="J49" s="4"/>
-      <c r="K49" s="4"/>
-    </row>
-    <row r="50" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+        <v>169</v>
+      </c>
+      <c r="I49" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="J49" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K49" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>31</v>
       </c>
@@ -2399,16 +2523,16 @@
         <v>1</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>179</v>
+        <v>63</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="J50" s="4" t="s">
         <v>40</v>
@@ -2417,7 +2541,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="160" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>31</v>
       </c>
@@ -2428,16 +2552,20 @@
         <v>1</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+        <v>176</v>
+      </c>
+      <c r="H51" s="4"/>
+      <c r="I51" s="4"/>
+      <c r="J51" s="4"/>
+      <c r="K51" s="4"/>
+    </row>
+    <row r="52" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>31</v>
       </c>
@@ -2448,16 +2576,16 @@
         <v>1</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="J52" s="4" t="s">
         <v>40</v>
@@ -2466,7 +2594,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="96" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:11" ht="160" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
         <v>31</v>
       </c>
@@ -2477,22 +2605,16 @@
         <v>1</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="I53" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="J53" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
         <v>31</v>
       </c>
@@ -2503,16 +2625,16 @@
         <v>1</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>109</v>
+        <v>186</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="J54" s="4" t="s">
         <v>40</v>
@@ -2521,32 +2643,87 @@
         <v>41</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C55" s="4" t="s">
+      <c r="C55" s="4">
+        <v>1</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="I55" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J55" s="4" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A56" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C56" s="4">
+        <v>1</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="I56" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="J56" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K56" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A57" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C57" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="E55" s="4" t="s">
+      <c r="E57" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="F55" s="4" t="s">
+      <c r="F57" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="G55" s="4" t="s">
+      <c r="G57" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="I55" s="4" t="s">
+      <c r="I57" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="J55" s="4" t="s">
+      <c r="J57" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K55" s="4" t="s">
+      <c r="K57" s="4" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>

<commit_message>
changed grouping variable, added output variables and improved test cases
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE3F6EB-6645-6C43-BD39-E2D7D61D2DCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF1EE68C-8850-7A42-8604-E4FC993D8311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="217">
   <si>
     <t>Product</t>
   </si>
@@ -638,6 +638,42 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>C98389</t>
+  </si>
+  <si>
+    <t>NON-INT</t>
+  </si>
+  <si>
+    <t>STYPE1</t>
+  </si>
+  <si>
+    <t>STYPE2</t>
+  </si>
+  <si>
+    <t>TRT</t>
+  </si>
+  <si>
+    <t>Investigational Therapy or Treatment</t>
+  </si>
+  <si>
+    <t>Zanomaline</t>
+  </si>
+  <si>
+    <t>0XXX0X00XX</t>
+  </si>
+  <si>
+    <t>UNII</t>
+  </si>
+  <si>
+    <t>Dataset</t>
+  </si>
+  <si>
+    <t>$STYPE_INTERVENTIONAL</t>
+  </si>
+  <si>
+    <t>Record</t>
   </si>
 </sst>
 </file>
@@ -673,7 +709,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -684,6 +720,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -725,7 +767,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -741,6 +783,10 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1095,7 +1141,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3DD88E2-BA18-FE44-AA70-D0EB14B73457}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -1126,16 +1172,76 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D2">
+        <v>47</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>216</v>
+      </c>
+      <c r="D3">
+        <v>47</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>216</v>
+      </c>
+      <c r="D4">
+        <v>47</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>214</v>
+      </c>
+      <c r="D5" t="s">
         <v>204</v>
       </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" t="s">
-        <v>31</v>
+      <c r="E5" t="s">
+        <v>215</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1145,7 +1251,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:11" ht="32" x14ac:dyDescent="0.2">
@@ -2317,13 +2423,16 @@
       <c r="C47" s="4">
         <v>1</v>
       </c>
-      <c r="E47" s="4" t="s">
+      <c r="D47" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="E47" s="8" t="s">
         <v>167</v>
       </c>
       <c r="F47" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="G47" s="4" t="s">
+      <c r="G47" s="8" t="s">
         <v>169</v>
       </c>
       <c r="I47" s="4" t="s">
@@ -2336,27 +2445,30 @@
         <v>41</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C48" s="4">
-        <v>1</v>
+      <c r="C48" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D48" t="s">
+        <v>208</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>173</v>
+        <v>206</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>174</v>
+        <v>205</v>
       </c>
       <c r="J48" s="4" t="s">
         <v>40</v>
@@ -2365,7 +2477,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>31</v>
       </c>
@@ -2376,16 +2488,16 @@
         <v>1</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>63</v>
+        <v>173</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="J49" s="4" t="s">
         <v>40</v>
@@ -2394,7 +2506,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="112" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>31</v>
       </c>
@@ -2405,118 +2517,118 @@
         <v>1</v>
       </c>
       <c r="E50" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="I50" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J50" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K50" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="112" x14ac:dyDescent="0.2">
+      <c r="A51" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C51" s="4">
+        <v>1</v>
+      </c>
+      <c r="E51" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="F50" s="4" t="s">
+      <c r="F51" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="G50" s="4" t="s">
+      <c r="G51" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="H50" s="4"/>
-      <c r="I50" s="4"/>
-      <c r="J50" s="4"/>
-      <c r="K50" s="4"/>
-    </row>
-    <row r="51" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A51" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C51" s="4">
-        <v>1</v>
-      </c>
-      <c r="E51" s="4" t="s">
+      <c r="H51" s="4"/>
+      <c r="I51" s="4"/>
+      <c r="J51" s="4"/>
+      <c r="K51" s="4"/>
+    </row>
+    <row r="52" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A52" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C52" s="4">
+        <v>1</v>
+      </c>
+      <c r="E52" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F51" s="4" t="s">
+      <c r="F52" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="G51" s="4" t="s">
+      <c r="G52" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="I51" s="4" t="s">
+      <c r="I52" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="J51" s="4" t="s">
+      <c r="J52" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K51" s="4" t="s">
+      <c r="K52" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="160" x14ac:dyDescent="0.2">
-      <c r="A52" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C52" s="4">
-        <v>1</v>
-      </c>
-      <c r="E52" s="4" t="s">
+    <row r="53" spans="1:11" ht="160" x14ac:dyDescent="0.2">
+      <c r="A53" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C53" s="4">
+        <v>1</v>
+      </c>
+      <c r="E53" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="F52" s="4" t="s">
+      <c r="F53" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="G52" s="4" t="s">
+      <c r="G53" s="4" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="64" x14ac:dyDescent="0.2">
-      <c r="A53" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C53" s="4">
-        <v>1</v>
-      </c>
-      <c r="E53" s="4" t="s">
+    <row r="54" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+      <c r="A54" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C54" s="4">
+        <v>1</v>
+      </c>
+      <c r="E54" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="F53" s="4" t="s">
+      <c r="F54" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="G53" s="4" t="s">
+      <c r="G54" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="I53" s="4" t="s">
+      <c r="I54" s="4" t="s">
         <v>191</v>
-      </c>
-      <c r="J53" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K53" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A54" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C54" s="4">
-        <v>1</v>
-      </c>
-      <c r="E54" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="F54" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="G54" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="I54" s="4" t="s">
-        <v>194</v>
       </c>
       <c r="J54" s="4" t="s">
         <v>40</v>
@@ -2525,32 +2637,90 @@
         <v>41</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C55" s="4" t="s">
+      <c r="C55" s="4">
+        <v>1</v>
+      </c>
+      <c r="D55" t="s">
+        <v>208</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="I55" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="J55" s="4" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A56" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C56" s="4">
+        <v>1</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="I56" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="J56" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K56" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A57" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C57" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="E55" s="4" t="s">
+      <c r="E57" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="F55" s="4" t="s">
+      <c r="F57" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="G55" s="4" t="s">
+      <c r="G57" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="I55" s="4" t="s">
+      <c r="I57" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="J55" s="4" t="s">
+      <c r="J57" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K55" s="4" t="s">
+      <c r="K57" s="4" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>

<commit_message>
removed unneeded output variables
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D372D9B-844F-C64C-936F-94FDBC9E66BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE107DB4-549B-6C41-8664-8D1CC4469870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="217">
   <si>
     <t>Product</t>
   </si>
@@ -767,7 +767,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -784,6 +784,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1140,7 +1143,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44434EA3-6FA4-EA42-A583-C1F1881D4D81}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -1191,55 +1194,15 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>209</v>
-      </c>
-      <c r="D3">
-        <v>23</v>
+        <v>208</v>
+      </c>
+      <c r="D3" t="s">
+        <v>206</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>209</v>
-      </c>
-      <c r="D4">
-        <v>23</v>
-      </c>
-      <c r="E4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" t="s">
-        <v>208</v>
-      </c>
-      <c r="D5" t="s">
-        <v>206</v>
-      </c>
-      <c r="E5" t="s">
         <v>207</v>
       </c>
-      <c r="F5">
+      <c r="F3">
         <v>1</v>
       </c>
     </row>
@@ -1861,13 +1824,13 @@
       <c r="D23" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="8" t="s">
         <v>88</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G23" s="7" t="s">
+      <c r="G23" s="8" t="s">
         <v>38</v>
       </c>
       <c r="H23" s="4"/>

</xml_diff>

<commit_message>
change rule functionality to include all Trial Design datasets
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17B85662-5133-0746-A235-239505F51CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7042477-660D-C040-96D6-1286FEC5E807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-8560" windowWidth="51200" windowHeight="28200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="303">
   <si>
     <t>Product</t>
   </si>
@@ -930,13 +930,10 @@
     <t>Dataset</t>
   </si>
   <si>
-    <t>TA</t>
-  </si>
-  <si>
-    <t>TI</t>
-  </si>
-  <si>
-    <t>[ABSENT]</t>
+    <t>$missing_trial_design_domains</t>
+  </si>
+  <si>
+    <t>"TM", "TI", "TE","TD", "TA"</t>
   </si>
 </sst>
 </file>
@@ -1012,7 +1009,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1028,6 +1025,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1443,291 +1443,37 @@
         <v>301</v>
       </c>
       <c r="F2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C3" t="s">
-        <v>300</v>
-      </c>
-      <c r="D3" t="s">
-        <v>299</v>
-      </c>
-      <c r="E3" t="s">
-        <v>91</v>
-      </c>
-      <c r="F3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C4" t="s">
-        <v>300</v>
-      </c>
-      <c r="D4" t="s">
-        <v>299</v>
-      </c>
-      <c r="E4" t="s">
-        <v>302</v>
-      </c>
-      <c r="F4" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
-        <v>85</v>
-      </c>
-      <c r="C5" t="s">
-        <v>300</v>
-      </c>
-      <c r="D5" t="s">
-        <v>299</v>
-      </c>
-      <c r="E5" t="s">
-        <v>120</v>
-      </c>
-      <c r="F5" t="s">
-        <v>297</v>
-      </c>
+      <c r="F3" s="9"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="8">
-        <v>1</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>300</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>299</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>2</v>
-      </c>
-      <c r="B7" t="s">
-        <v>297</v>
-      </c>
-      <c r="C7" t="s">
-        <v>300</v>
-      </c>
-      <c r="D7" t="s">
-        <v>299</v>
-      </c>
-      <c r="E7" t="s">
-        <v>301</v>
-      </c>
-      <c r="F7" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>2</v>
-      </c>
-      <c r="B8" t="s">
-        <v>297</v>
-      </c>
-      <c r="C8" t="s">
-        <v>300</v>
-      </c>
-      <c r="D8" t="s">
-        <v>299</v>
-      </c>
-      <c r="E8" t="s">
-        <v>91</v>
-      </c>
-      <c r="F8" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>2</v>
-      </c>
-      <c r="B9" t="s">
-        <v>297</v>
-      </c>
-      <c r="C9" t="s">
-        <v>300</v>
-      </c>
-      <c r="D9" t="s">
-        <v>299</v>
-      </c>
-      <c r="E9" t="s">
-        <v>302</v>
-      </c>
-      <c r="F9" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>2</v>
-      </c>
-      <c r="B10" t="s">
-        <v>297</v>
-      </c>
-      <c r="C10" t="s">
-        <v>300</v>
-      </c>
-      <c r="D10" t="s">
-        <v>299</v>
-      </c>
-      <c r="E10" t="s">
-        <v>120</v>
-      </c>
-      <c r="F10" t="s">
-        <v>297</v>
-      </c>
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="8">
-        <v>2</v>
-      </c>
-      <c r="B11" t="s">
-        <v>297</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>300</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>299</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" t="s">
-        <v>300</v>
-      </c>
-      <c r="D12" t="s">
-        <v>299</v>
-      </c>
-      <c r="E12" t="s">
-        <v>301</v>
-      </c>
-      <c r="F12" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" t="s">
-        <v>300</v>
-      </c>
-      <c r="D13" t="s">
-        <v>299</v>
-      </c>
-      <c r="E13" t="s">
-        <v>91</v>
-      </c>
-      <c r="F13" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" t="s">
-        <v>300</v>
-      </c>
-      <c r="D14" t="s">
-        <v>299</v>
-      </c>
-      <c r="E14" t="s">
-        <v>302</v>
-      </c>
-      <c r="F14" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>3</v>
-      </c>
-      <c r="B15" t="s">
-        <v>6</v>
-      </c>
-      <c r="C15" t="s">
-        <v>300</v>
-      </c>
-      <c r="D15" t="s">
-        <v>299</v>
-      </c>
-      <c r="E15" t="s">
-        <v>120</v>
-      </c>
-      <c r="F15" t="s">
-        <v>297</v>
-      </c>
+      <c r="A11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="8">
-        <v>3</v>
-      </c>
-      <c r="B16" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>300</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>299</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>6</v>
-      </c>
+      <c r="A16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
small fix in the Excel files
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/negative/01/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7042477-660D-C040-96D6-1286FEC5E807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EF8CF48-4AB5-B944-8A8F-249CBFE7E505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-8560" windowWidth="51200" windowHeight="28200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -933,7 +933,7 @@
     <t>$missing_trial_design_domains</t>
   </si>
   <si>
-    <t>"TM", "TI", "TE","TD", "TA"</t>
+    <t>"TM", "TI","TD", "TA"</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
update error reporting and test cases
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29B6C1FC-41F1-6942-96D3-901D2EEEE03E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D3965D4-7948-A646-885C-9FC71FC84D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36400" yWindow="-2680" windowWidth="30240" windowHeight="18980" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51200" yWindow="-2260" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="63">
   <si>
     <t>Product</t>
   </si>
@@ -77,9 +77,6 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>dataset_name</t>
-  </si>
-  <si>
     <t>SV</t>
   </si>
   <si>
@@ -89,12 +86,6 @@
     <t>DOMAIN</t>
   </si>
   <si>
-    <t>variable_length</t>
-  </si>
-  <si>
-    <t>variable_value_length</t>
-  </si>
-  <si>
     <t>$max_variable_value_length</t>
   </si>
   <si>
@@ -182,9 +173,6 @@
     <t>CDISCPILOT01</t>
   </si>
   <si>
-    <t>CDISC001</t>
-  </si>
-  <si>
     <t>SCREENING</t>
   </si>
   <si>
@@ -221,7 +209,10 @@
     <t>Screening</t>
   </si>
   <si>
-    <t>CDISC002</t>
+    <t>CDISC1</t>
+  </si>
+  <si>
+    <t>CDISC00002</t>
   </si>
 </sst>
 </file>
@@ -627,9 +618,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -637,7 +628,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -656,9 +647,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -666,7 +657,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -674,7 +665,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -692,10 +683,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -715,7 +706,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -729,13 +720,13 @@
         <v>16</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="F2" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -749,13 +740,13 @@
         <v>16</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="F3" s="1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -772,10 +763,10 @@
         <v>21</v>
       </c>
       <c r="F4" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -792,13 +783,13 @@
         <v>22</v>
       </c>
       <c r="F5" s="1">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>1</v>
-      </c>
       <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
@@ -809,16 +800,16 @@
         <v>16</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="1">
+        <v>18</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>1</v>
-      </c>
       <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
@@ -829,15 +820,15 @@
         <v>16</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F7" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>6</v>
@@ -849,16 +840,437 @@
         <v>16</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F8" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>2</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="1">
         <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>3</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>3</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
+        <v>3</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
+        <v>3</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" s="4">
+        <v>4</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" s="4">
+        <v>4</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="4">
+        <v>4</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="4">
+        <v>4</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F17" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" s="4">
+        <v>5</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" s="4">
+        <v>5</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F19" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" s="4">
+        <v>5</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F20" s="4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" s="4">
+        <v>5</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F21" s="4">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="4">
+        <v>6</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" s="4">
+        <v>6</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F23" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" s="4">
+        <v>6</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" s="4">
+        <v>6</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" s="4">
+        <v>7</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A27" s="4">
+        <v>7</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F27" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" s="4">
+        <v>7</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F28" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" s="4">
+        <v>7</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F29" s="4">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:F8" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:F1 A5:E5 A2:E2 A3:E3 A4:E4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -866,128 +1278,128 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:L6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="J1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="J2" s="3" t="s">
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="B3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="L2" s="3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="15" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>50</v>
-      </c>
       <c r="F3" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="15" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
-        <v>12</v>
+        <v>120</v>
       </c>
       <c r="B4" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" s="3">
         <v>8</v>
@@ -1020,33 +1432,33 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D5" s="1">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D5" s="1">
-        <v>1</v>
-      </c>
-      <c r="E5" s="1">
-        <v>1</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="J5" s="1">
         <v>-28</v>
@@ -1055,36 +1467,36 @@
         <v>4</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="15" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D6" s="1">
-        <v>1</v>
-      </c>
-      <c r="E6" s="1">
-        <v>1</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="J6" s="1">
         <v>-28</v>
@@ -1093,14 +1505,14 @@
         <v>42</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L5" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:L3 A5:B5 D5:L5 D4:L4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1108,80 +1520,80 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B4" s="3">
         <v>3</v>
@@ -1202,47 +1614,47 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C5" s="1">
         <v>1</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E5" s="1">
         <v>13094209</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="G5" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C6" s="1">
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E6" s="1">
         <v>13094209</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="G6" s="1">
         <v>1</v>
@@ -1252,7 +1664,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:G3 A5:G5 A4:F4" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:G3 A5:G5 B4:F4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
changed negative case test value
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C72C1368-D9F5-4743-8F07-2FDBEC3C6BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED243EF7-5C70-264C-87FA-4D50B81DE580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="46">
   <si>
     <t>Product</t>
   </si>
@@ -158,13 +158,16 @@
   </si>
   <si>
     <t>CEROUS SALICYLATE</t>
+  </si>
+  <si>
+    <t>UNIITERM1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -187,11 +190,6 @@
     </font>
     <font>
       <i/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -249,9 +247,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -592,9 +590,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="21" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -602,7 +600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -621,9 +619,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="21" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -631,7 +629,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -650,9 +648,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="21" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -672,7 +670,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -692,7 +690,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -705,14 +703,14 @@
       <c r="D3" s="2">
         <v>5</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>23</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>1</v>
       </c>
@@ -728,14 +726,14 @@
       <c r="E4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="2">
-        <v>9999999999</v>
+      <c r="F4" s="5" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A4:F4 A1:F2" numberStoredAsText="1"/>
+    <ignoredError sqref="A4:E4 A1:F2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -743,9 +741,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="21" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -780,7 +778,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>27</v>
       </c>
@@ -815,7 +813,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>38</v>
       </c>
@@ -850,7 +848,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>10</v>
       </c>
@@ -885,7 +883,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>40</v>
       </c>
@@ -904,20 +902,20 @@
       <c r="F5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>44</v>
+      <c r="G5" s="6" t="s">
+        <v>45</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I5" s="5">
-        <v>9999999999</v>
+      <c r="I5" s="7" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:K4 A5:F5 H5:K5" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:K4 A5:F5 H5 J5:K5" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
removed grouping by TSGRPID, added informative output variables and changed sensitivity to dataset
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B9BA9F0-E321-3445-B073-6053459672B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CFAE84C-FD61-EC49-A861-0959A03B6D2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="210">
   <si>
     <t>Product</t>
   </si>
@@ -313,18 +313,6 @@
     <t>2019-03-01</t>
   </si>
   <si>
-    <t>INTTYPE</t>
-  </si>
-  <si>
-    <t>Intervention Type</t>
-  </si>
-  <si>
-    <t>DRUG</t>
-  </si>
-  <si>
-    <t>C1909</t>
-  </si>
-  <si>
     <t>LENGTH</t>
   </si>
   <si>
@@ -643,15 +631,6 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>STYPE1</t>
-  </si>
-  <si>
-    <t>STYPE2</t>
-  </si>
-  <si>
-    <t>OTHER</t>
-  </si>
-  <si>
     <t>INTMODEL</t>
   </si>
   <si>
@@ -670,7 +649,10 @@
     <t>$STYPE_INTERVENTIONAL</t>
   </si>
   <si>
-    <t>Record</t>
+    <t>$TSPARMCD_INTMODEL</t>
+  </si>
+  <si>
+    <t>$TSPARMCD_INTTYPE</t>
   </si>
 </sst>
 </file>
@@ -706,7 +688,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -719,14 +701,8 @@
         <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -749,22 +725,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -777,14 +742,10 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1105,7 +1066,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -1141,27 +1102,30 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CA1A07C-A03C-3740-B416-1DF5B7F6AA7A}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="5" max="5" width="21.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>200</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -1172,16 +1136,16 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>215</v>
-      </c>
-      <c r="D2">
-        <v>47</v>
+        <v>206</v>
+      </c>
+      <c r="D2" t="s">
+        <v>201</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>206</v>
+        <v>207</v>
+      </c>
+      <c r="F2" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -1192,16 +1156,16 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>215</v>
-      </c>
-      <c r="D3">
-        <v>47</v>
+        <v>206</v>
+      </c>
+      <c r="D3" t="s">
+        <v>201</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>163</v>
+        <v>208</v>
+      </c>
+      <c r="F3" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -1212,36 +1176,16 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>215</v>
-      </c>
-      <c r="D4">
-        <v>47</v>
+        <v>206</v>
+      </c>
+      <c r="D4" t="s">
+        <v>201</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" t="s">
-        <v>213</v>
-      </c>
-      <c r="D5" t="s">
-        <v>205</v>
-      </c>
-      <c r="E5" t="s">
-        <v>214</v>
-      </c>
-      <c r="F5" s="7">
-        <v>1</v>
+        <v>209</v>
+      </c>
+      <c r="F4" s="6">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1251,7 +1195,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K57"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:11" ht="32" x14ac:dyDescent="0.2">
@@ -1834,7 +1778,7 @@
         <v>92</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="I22" s="4" t="s">
         <v>93</v>
@@ -1856,20 +1800,17 @@
       <c r="C23" s="4">
         <v>1</v>
       </c>
-      <c r="D23" t="s">
-        <v>207</v>
-      </c>
       <c r="E23" s="4" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="J23" s="4" t="s">
         <v>40</v>
@@ -1888,9 +1829,6 @@
       <c r="C24" s="4">
         <v>1</v>
       </c>
-      <c r="D24" t="s">
-        <v>207</v>
-      </c>
       <c r="E24" s="4" t="s">
         <v>96</v>
       </c>
@@ -1900,57 +1838,51 @@
       <c r="G24" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="I24" s="4" t="s">
+      <c r="J24" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A25" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="4">
+        <v>1</v>
+      </c>
+      <c r="E25" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J24" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K24" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A25" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C25" s="4">
-        <v>1</v>
-      </c>
-      <c r="E25" s="4" t="s">
+      <c r="F25" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="G25" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="112" x14ac:dyDescent="0.2">
+      <c r="A26" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" s="4">
+        <v>1</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="E26" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="J25" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A26" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C26" s="4">
-        <v>1</v>
-      </c>
-      <c r="E26" s="4" t="s">
+      <c r="F26" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="G26" s="4" t="s">
         <v>104</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="112" x14ac:dyDescent="0.2">
@@ -1961,157 +1893,160 @@
         <v>32</v>
       </c>
       <c r="C27" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>105</v>
       </c>
       <c r="E27" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="G27" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="F27" s="4" t="s">
+    </row>
+    <row r="28" spans="1:11" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A28" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" s="4">
+        <v>1</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="F28" s="4" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" ht="112" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C28" s="4">
+      <c r="G28" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="365" x14ac:dyDescent="0.2">
+      <c r="A29" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C29" s="4">
         <v>2</v>
       </c>
-      <c r="D28" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="F28" s="4" t="s">
+      <c r="D29" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="F29" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="G29" s="4" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A29" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C29" s="4">
-        <v>1</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="E29" s="4" t="s">
+    <row r="30" spans="1:11" ht="335" x14ac:dyDescent="0.2">
+      <c r="A30" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="G30" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="F29" s="4" t="s">
+    </row>
+    <row r="31" spans="1:11" ht="128" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>112</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="365" x14ac:dyDescent="0.2">
-      <c r="A30" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C30" s="4">
-        <v>2</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="335" x14ac:dyDescent="0.2">
-      <c r="A31" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>70</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>105</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G31" s="4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="112" x14ac:dyDescent="0.2">
+      <c r="A32" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="G32" s="4" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="128" x14ac:dyDescent="0.2">
-      <c r="A32" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C32" s="4" t="s">
+    <row r="33" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" s="4">
+        <v>1</v>
+      </c>
+      <c r="E33" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="D32" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="G32" s="4" t="s">
+      <c r="F33" s="4" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" ht="112" x14ac:dyDescent="0.2">
-      <c r="A33" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C33" s="4" t="s">
+      <c r="G33" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="D33" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="G33" s="4" t="s">
+      <c r="I33" s="4" t="s">
         <v>119</v>
+      </c>
+      <c r="J33" s="4" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="64" x14ac:dyDescent="0.2">
@@ -2125,39 +2060,42 @@
         <v>1</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="I34" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="J34" s="4" t="s">
+    </row>
+    <row r="35" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A35" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C35" s="4">
+        <v>1</v>
+      </c>
+      <c r="E35" s="4" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" ht="64" x14ac:dyDescent="0.2">
-      <c r="A35" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35" s="4">
-        <v>1</v>
-      </c>
-      <c r="E35" s="4" t="s">
+      <c r="F35" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="F35" s="4" t="s">
-        <v>126</v>
-      </c>
       <c r="G35" s="4" t="s">
-        <v>127</v>
+        <v>44</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J35" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K35" s="4" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="48" x14ac:dyDescent="0.2">
@@ -2171,45 +2109,42 @@
         <v>1</v>
       </c>
       <c r="E36" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="G36" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="F36" s="4" t="s">
+    </row>
+    <row r="37" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C37" s="4">
+        <v>1</v>
+      </c>
+      <c r="E37" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="G36" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="I36" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J36" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K36" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A37" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C37" s="4">
-        <v>1</v>
-      </c>
-      <c r="E37" s="4" t="s">
+      <c r="F37" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="G37" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="I37" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="J37" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>31</v>
       </c>
@@ -2229,13 +2164,16 @@
         <v>135</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+      <c r="K38" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
         <v>31</v>
       </c>
@@ -2254,15 +2192,6 @@
       <c r="G39" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="I39" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="J39" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K39" s="4" t="s">
-        <v>41</v>
-      </c>
     </row>
     <row r="40" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
@@ -2275,13 +2204,13 @@
         <v>1</v>
       </c>
       <c r="E40" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="F40" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="F40" s="4" t="s">
+      <c r="G40" s="4" t="s">
         <v>142</v>
-      </c>
-      <c r="G40" s="4" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="32" x14ac:dyDescent="0.2">
@@ -2295,39 +2224,48 @@
         <v>1</v>
       </c>
       <c r="E41" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="F41" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="F41" s="4" t="s">
+      <c r="G41" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="G41" s="4" t="s">
+      <c r="J41" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A42" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C42" s="4">
+        <v>1</v>
+      </c>
+      <c r="E42" s="4" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="42" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A42" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C42" s="4">
-        <v>1</v>
-      </c>
-      <c r="E42" s="4" t="s">
+      <c r="F42" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="F42" s="4" t="s">
+      <c r="G42" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="G42" s="4" t="s">
+      <c r="I42" s="4" t="s">
         <v>149</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+      <c r="K42" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
         <v>31</v>
       </c>
@@ -2346,80 +2284,80 @@
       <c r="G43" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="I43" s="4" t="s">
+    </row>
+    <row r="44" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A44" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C44" s="4">
+        <v>1</v>
+      </c>
+      <c r="E44" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="J43" s="4" t="s">
+      <c r="F44" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="J44" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A45" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C45" s="4">
+        <v>1</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A46" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C46" s="4">
+        <v>1</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="G46" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="I46" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="J46" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K43" s="4" t="s">
+      <c r="K46" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="96" x14ac:dyDescent="0.2">
-      <c r="A44" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C44" s="4">
-        <v>1</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="F44" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="G44" s="4" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A45" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C45" s="4">
-        <v>1</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F45" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="G45" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="J45" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A46" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C46" s="4">
-        <v>1</v>
-      </c>
-      <c r="E46" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="F46" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="G46" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
         <v>31</v>
       </c>
@@ -2429,16 +2367,13 @@
       <c r="C47" s="4">
         <v>1</v>
       </c>
-      <c r="D47" s="8" t="s">
-        <v>206</v>
-      </c>
-      <c r="E47" s="9" t="s">
+      <c r="E47" s="4" t="s">
         <v>163</v>
       </c>
       <c r="F47" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="G47" s="9" t="s">
+      <c r="G47" s="4" t="s">
         <v>165</v>
       </c>
       <c r="I47" s="4" t="s">
@@ -2458,23 +2393,20 @@
       <c r="B48" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C48" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>207</v>
+      <c r="C48" s="4">
+        <v>1</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>208</v>
+        <v>63</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="J48" s="4" t="s">
         <v>40</v>
@@ -2483,7 +2415,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>31</v>
       </c>
@@ -2494,25 +2426,20 @@
         <v>1</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="I49" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="J49" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K49" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+        <v>172</v>
+      </c>
+      <c r="H49" s="4"/>
+      <c r="I49" s="4"/>
+      <c r="J49" s="4"/>
+      <c r="K49" s="4"/>
+    </row>
+    <row r="50" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>31</v>
       </c>
@@ -2523,16 +2450,16 @@
         <v>1</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>63</v>
+        <v>175</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="J50" s="4" t="s">
         <v>40</v>
@@ -2541,7 +2468,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="112" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11" ht="160" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>31</v>
       </c>
@@ -2552,20 +2479,16 @@
         <v>1</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="H51" s="4"/>
-      <c r="I51" s="4"/>
-      <c r="J51" s="4"/>
-      <c r="K51" s="4"/>
-    </row>
-    <row r="52" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>31</v>
       </c>
@@ -2576,16 +2499,16 @@
         <v>1</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="J52" s="4" t="s">
         <v>40</v>
@@ -2594,7 +2517,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="160" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
         <v>31</v>
       </c>
@@ -2605,16 +2528,22 @@
         <v>1</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+        <v>186</v>
+      </c>
+      <c r="I53" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="J53" s="4" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
         <v>31</v>
       </c>
@@ -2625,16 +2554,16 @@
         <v>1</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>186</v>
+        <v>105</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="J54" s="4" t="s">
         <v>40</v>
@@ -2643,87 +2572,32 @@
         <v>41</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="96" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C55" s="4">
-        <v>1</v>
+      <c r="C55" s="4" t="s">
+        <v>112</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>190</v>
+        <v>101</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A56" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C56" s="4">
-        <v>1</v>
-      </c>
-      <c r="E56" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="F56" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="G56" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I56" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="J56" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K56" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A57" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="E57" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="F57" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="G57" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="I57" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="J57" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K57" s="4" t="s">
+      <c r="K55" s="4" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>

<commit_message>
removed grouping by TSGRPID and STUDYID, added informative output variables and changed sensitivity to dataset
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{274EDFF5-DCF1-F148-89B6-D333C71F6697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19657EE1-6091-5743-A407-5564BE0594E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="208">
   <si>
     <t>Product</t>
   </si>
@@ -638,6 +638,15 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>Dataset</t>
+  </si>
+  <si>
+    <t>$STYPE_INTERVENTIONAL</t>
+  </si>
+  <si>
+    <t>$TSPARMCD_PCLAS</t>
   </si>
 </sst>
 </file>
@@ -1095,7 +1104,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99458E18-8BF7-F94F-B79C-D42E6729B92D}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -1126,16 +1135,36 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D2" t="s">
         <v>204</v>
       </c>
       <c r="E2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" t="s">
-        <v>31</v>
+        <v>206</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>205</v>
+      </c>
+      <c r="D3" t="s">
+        <v>204</v>
+      </c>
+      <c r="E3" t="s">
+        <v>207</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changing grouping variable and added informative output variables
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE107DB4-549B-6C41-8664-8D1CC4469870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82AE935E-8F27-194B-847D-6562E1A76656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="218">
   <si>
     <t>Product</t>
   </si>
@@ -674,13 +674,16 @@
   </si>
   <si>
     <t>Patients with Probable Mild to Moderate Alzheimers Disease</t>
+  </si>
+  <si>
+    <t>$TSPARMCD_TDIGRP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -704,6 +707,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -767,7 +777,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -786,6 +796,7 @@
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1143,7 +1154,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44434EA3-6FA4-EA42-A583-C1F1881D4D81}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -1187,23 +1198,63 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="A3" s="8">
+        <v>1</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="D3" s="8">
+        <v>23</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
         <v>208</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D4" t="s">
         <v>206</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E4" t="s">
         <v>207</v>
       </c>
-      <c r="F3">
-        <v>1</v>
+      <c r="F4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>208</v>
+      </c>
+      <c r="D5" t="s">
+        <v>206</v>
+      </c>
+      <c r="E5" t="s">
+        <v>217</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1755,7 +1806,7 @@
       <c r="C21" s="4">
         <v>1</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="9" t="s">
         <v>210</v>
       </c>
       <c r="E21" s="4" t="s">
@@ -1764,7 +1815,7 @@
       <c r="F21" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="G21" s="9" t="s">
         <v>38</v>
       </c>
       <c r="H21" s="4"/>
@@ -1788,7 +1839,7 @@
       <c r="C22" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="9" t="s">
         <v>211</v>
       </c>
       <c r="E22" s="4" t="s">
@@ -1797,7 +1848,7 @@
       <c r="F22" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="9" t="s">
         <v>44</v>
       </c>
       <c r="H22" s="4"/>
@@ -1824,13 +1875,13 @@
       <c r="D23" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="E23" s="8" t="s">
+      <c r="E23" s="4" t="s">
         <v>88</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G23" s="8" t="s">
+      <c r="G23" s="7" t="s">
         <v>38</v>
       </c>
       <c r="H23" s="4"/>

</xml_diff>

<commit_message>
added TS output variable
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{202BF879-8F75-7D48-AC09-D035B02B34AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2122F233-4B58-E54C-B326-01EEE564375A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="46">
   <si>
     <t>Product</t>
   </si>
@@ -157,7 +157,10 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>[ABSENT]</t>
+    <t>TS</t>
+  </si>
+  <si>
+    <t>Not in dataset</t>
   </si>
 </sst>
 </file>
@@ -627,10 +630,10 @@
         <v>43</v>
       </c>
       <c r="E2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
removed unnecessary check and changed test data accordingly
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{719F34A0-B324-9540-9D15-7CD587E3C89B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD37E90-F4CA-8F42-BAC7-46F51E3FDF53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="92">
   <si>
     <t>Product</t>
   </si>
@@ -300,9 +300,6 @@
   </si>
   <si>
     <t>Record</t>
-  </si>
-  <si>
-    <t>[ABSENT]</t>
   </si>
 </sst>
 </file>
@@ -455,7 +452,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -492,6 +489,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -854,7 +855,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F818558-05EF-6C45-AFB4-B21EE1959E05}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -884,7 +885,7 @@
       <c r="B2" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" t="s">
         <v>91</v>
       </c>
       <c r="D2" s="15">
@@ -904,8 +905,8 @@
       <c r="B3" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C3" s="15" t="s">
-        <v>88</v>
+      <c r="C3" t="s">
+        <v>91</v>
       </c>
       <c r="D3" s="15">
         <v>5</v>
@@ -914,7 +915,7 @@
         <v>75</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -924,7 +925,7 @@
       <c r="B4" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" t="s">
         <v>91</v>
       </c>
       <c r="D4" s="15">
@@ -944,8 +945,8 @@
       <c r="B5" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="15" t="s">
-        <v>88</v>
+      <c r="C5" t="s">
+        <v>91</v>
       </c>
       <c r="D5" s="15">
         <v>6</v>
@@ -954,87 +955,87 @@
         <v>75</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="15">
         <v>3</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="C6" s="15" t="s">
+      <c r="B6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" t="s">
         <v>91</v>
       </c>
-      <c r="D6" s="15">
-        <v>7</v>
+      <c r="D6">
+        <v>5</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="15">
         <v>3</v>
       </c>
-      <c r="B7" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="D7" s="15">
-        <v>7</v>
+      <c r="B7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" t="s">
+        <v>91</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
       </c>
       <c r="E7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F7" s="15" t="s">
-        <v>92</v>
+        <v>53</v>
+      </c>
+      <c r="F7" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="15">
         <v>4</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" s="15" t="s">
+      <c r="B8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" t="s">
         <v>91</v>
       </c>
-      <c r="D8" s="15">
-        <v>8</v>
+      <c r="D8">
+        <v>6</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F8" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="15">
         <v>4</v>
       </c>
-      <c r="B9" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="D9" s="15">
-        <v>8</v>
+      <c r="B9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" t="s">
+        <v>91</v>
+      </c>
+      <c r="D9">
+        <v>6</v>
       </c>
       <c r="E9" t="s">
-        <v>75</v>
-      </c>
-      <c r="F9" s="15" t="s">
-        <v>92</v>
+        <v>53</v>
+      </c>
+      <c r="F9" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -1048,7 +1049,7 @@
         <v>91</v>
       </c>
       <c r="D10">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
@@ -1068,92 +1069,12 @@
         <v>91</v>
       </c>
       <c r="D11">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E11" t="s">
         <v>53</v>
       </c>
       <c r="F11" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>6</v>
-      </c>
-      <c r="B12" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" t="s">
-        <v>91</v>
-      </c>
-      <c r="D12">
-        <v>6</v>
-      </c>
-      <c r="E12" t="s">
-        <v>10</v>
-      </c>
-      <c r="F12" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>6</v>
-      </c>
-      <c r="B13" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" t="s">
-        <v>91</v>
-      </c>
-      <c r="D13">
-        <v>6</v>
-      </c>
-      <c r="E13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F13" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>7</v>
-      </c>
-      <c r="B14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C14" t="s">
-        <v>91</v>
-      </c>
-      <c r="D14">
-        <v>7</v>
-      </c>
-      <c r="E14" t="s">
-        <v>10</v>
-      </c>
-      <c r="F14" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>7</v>
-      </c>
-      <c r="B15" t="s">
-        <v>47</v>
-      </c>
-      <c r="C15" t="s">
-        <v>91</v>
-      </c>
-      <c r="D15">
-        <v>7</v>
-      </c>
-      <c r="E15" t="s">
-        <v>53</v>
-      </c>
-      <c r="F15" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1164,13 +1085,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F748488-0D8F-E445-8E6B-6B1937D7843D}">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="6" max="6" width="11.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="11" t="s">
         <v>6</v>
       </c>
@@ -1195,14 +1116,17 @@
       <c r="H1" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="J1" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="K1" s="11" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="64" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
@@ -1228,13 +1152,16 @@
         <v>21</v>
       </c>
       <c r="I2" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="J2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>24</v>
       </c>
@@ -1265,8 +1192,11 @@
       <c r="J3" s="5" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="K3" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>40</v>
       </c>
@@ -1297,8 +1227,11 @@
       <c r="J4" s="5" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K4" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>26</v>
       </c>
@@ -1323,14 +1256,17 @@
       <c r="H5" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="I5" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="J5" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="K5" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>26</v>
       </c>
@@ -1355,14 +1291,17 @@
       <c r="H6" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="I6" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="J6" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="K6" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>76</v>
       </c>
@@ -1375,7 +1314,7 @@
       <c r="D7" s="7">
         <v>1</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="18" t="s">
         <v>77</v>
       </c>
       <c r="F7" s="8" t="s">
@@ -1387,14 +1326,17 @@
       <c r="H7" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="I7" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J7" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="K7" s="8" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>76</v>
       </c>
@@ -1407,7 +1349,7 @@
       <c r="D8" s="7">
         <v>2</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="19" t="s">
         <v>77</v>
       </c>
       <c r="F8" s="6" t="s">
@@ -1419,10 +1361,13 @@
       <c r="H8" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J8" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="J8" s="6" t="s">
+      <c r="K8" s="6" t="s">
         <v>83</v>
       </c>
     </row>

</xml_diff>

<commit_message>
introduced grouping to limit output length
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD37E90-F4CA-8F42-BAC7-46F51E3FDF53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDD69961-20D6-7F45-8C36-431659F71E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="95">
   <si>
     <t>Product</t>
   </si>
@@ -300,6 +300,15 @@
   </si>
   <si>
     <t>Record</t>
+  </si>
+  <si>
+    <t>ABC125</t>
+  </si>
+  <si>
+    <t>DRUG Z</t>
+  </si>
+  <si>
+    <t>STUDYDRUG3</t>
   </si>
 </sst>
 </file>
@@ -452,7 +461,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -489,10 +498,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -855,7 +861,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F818558-05EF-6C45-AFB4-B21EE1959E05}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -962,84 +968,84 @@
       <c r="A6" s="15">
         <v>3</v>
       </c>
-      <c r="B6" t="s">
-        <v>47</v>
+      <c r="B6" s="15" t="s">
+        <v>45</v>
       </c>
       <c r="C6" t="s">
         <v>91</v>
       </c>
-      <c r="D6">
-        <v>5</v>
+      <c r="D6" s="15">
+        <v>9</v>
       </c>
       <c r="E6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" t="s">
-        <v>66</v>
+        <v>32</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="15">
         <v>3</v>
       </c>
-      <c r="B7" t="s">
-        <v>47</v>
+      <c r="B7" s="15" t="s">
+        <v>45</v>
       </c>
       <c r="C7" t="s">
         <v>91</v>
       </c>
-      <c r="D7">
-        <v>5</v>
+      <c r="D7" s="15">
+        <v>9</v>
       </c>
       <c r="E7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F7" t="s">
-        <v>69</v>
+        <v>75</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="15">
         <v>4</v>
       </c>
-      <c r="B8" t="s">
-        <v>47</v>
+      <c r="B8" s="15" t="s">
+        <v>45</v>
       </c>
       <c r="C8" t="s">
         <v>91</v>
       </c>
-      <c r="D8">
-        <v>6</v>
+      <c r="D8" s="15">
+        <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" t="s">
-        <v>66</v>
+        <v>32</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="15">
         <v>4</v>
       </c>
-      <c r="B9" t="s">
-        <v>47</v>
+      <c r="B9" s="15" t="s">
+        <v>45</v>
       </c>
       <c r="C9" t="s">
         <v>91</v>
       </c>
-      <c r="D9">
-        <v>6</v>
+      <c r="D9" s="15">
+        <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F9" t="s">
-        <v>90</v>
+        <v>75</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10">
+      <c r="A10" s="15">
         <v>5</v>
       </c>
       <c r="B10" t="s">
@@ -1049,7 +1055,7 @@
         <v>91</v>
       </c>
       <c r="D10">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
@@ -1059,7 +1065,7 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11">
+      <c r="A11" s="15">
         <v>5</v>
       </c>
       <c r="B11" t="s">
@@ -1069,12 +1075,52 @@
         <v>91</v>
       </c>
       <c r="D11">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E11" t="s">
         <v>53</v>
       </c>
       <c r="F11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="15">
+        <v>6</v>
+      </c>
+      <c r="B12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" t="s">
+        <v>91</v>
+      </c>
+      <c r="D12">
+        <v>6</v>
+      </c>
+      <c r="E12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="15">
+        <v>6</v>
+      </c>
+      <c r="B13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D13">
+        <v>6</v>
+      </c>
+      <c r="E13" t="s">
+        <v>53</v>
+      </c>
+      <c r="F13" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1085,7 +1131,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F748488-0D8F-E445-8E6B-6B1937D7843D}">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="6" max="6" width="11.83203125" customWidth="1"/>
@@ -1314,7 +1360,7 @@
       <c r="D7" s="7">
         <v>1</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="8" t="s">
         <v>77</v>
       </c>
       <c r="F7" s="8" t="s">
@@ -1349,7 +1395,7 @@
       <c r="D8" s="7">
         <v>2</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="7" t="s">
         <v>77</v>
       </c>
       <c r="F8" s="6" t="s">
@@ -1368,6 +1414,146 @@
         <v>81</v>
       </c>
       <c r="K8" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="7">
+        <v>123103</v>
+      </c>
+      <c r="D9" s="7">
+        <v>1</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="G9" s="7">
+        <v>13</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="I9" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="7">
+        <v>123103</v>
+      </c>
+      <c r="D10" s="7">
+        <v>2</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G10" s="7">
+        <v>24</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="I10" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="7">
+        <v>123103</v>
+      </c>
+      <c r="D11" s="7">
+        <v>3</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="G11" s="7">
+        <v>133</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="7">
+        <v>123103</v>
+      </c>
+      <c r="D12" s="7">
+        <v>4</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G12" s="7">
+        <v>244</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="K12" s="6" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1679,7 +1865,7 @@
       <c r="E7" t="s">
         <v>65</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="18" t="s">
         <v>66</v>
       </c>
       <c r="G7" t="s">
@@ -1700,7 +1886,7 @@
       <c r="L7">
         <v>1195</v>
       </c>
-      <c r="M7" s="14" t="s">
+      <c r="M7" s="18" t="s">
         <v>90</v>
       </c>
       <c r="N7" t="s">

</xml_diff>

<commit_message>
better negative test cases per els comments
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -72,12 +72,8 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -97,12 +93,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -138,7 +128,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -148,7 +138,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -597,7 +586,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
+      <c r="A4" s="3">
         <v>1</v>
       </c>
       <c r="B4" s="3" t="str">
@@ -677,7 +666,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2">
+      <c r="A8" s="3">
         <v>3</v>
       </c>
       <c r="B8" s="3" t="str">
@@ -686,18 +675,18 @@
       <c r="C8" s="3" t="str">
         <v>Record</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="3">
         <v>7</v>
       </c>
       <c r="E8" s="3" t="str">
         <v>LBLOINC</v>
       </c>
       <c r="F8" s="3" t="str">
-        <v>100002-5</v>
+        <v>99932-5</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2">
+      <c r="A9" s="3">
         <v>3</v>
       </c>
       <c r="B9" s="3" t="str">
@@ -706,7 +695,7 @@
       <c r="C9" s="3" t="str">
         <v>Record</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="3">
         <v>7</v>
       </c>
       <c r="E9" s="3" t="str">
@@ -717,7 +706,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2">
+      <c r="A10" s="3">
         <v>3</v>
       </c>
       <c r="B10" s="3" t="str">
@@ -828,10 +817,10 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
       <c r="D2" s="6" t="str">
@@ -1110,7 +1099,7 @@
       <c r="R5" s="3" t="str">
         <v>Y</v>
       </c>
-      <c r="S5" s="2" t="str">
+      <c r="S5" s="3" t="str">
         <v/>
       </c>
       <c r="T5" s="3">
@@ -1128,7 +1117,7 @@
       <c r="X5" s="3">
         <v>-7</v>
       </c>
-      <c r="Y5" s="8" t="str">
+      <c r="Y5" s="7" t="str">
         <v>999999-9</v>
       </c>
     </row>
@@ -1205,7 +1194,7 @@
       <c r="X6" s="3">
         <v>-7</v>
       </c>
-      <c r="Y6" s="9" t="str">
+      <c r="Y6" s="8" t="str">
         <v>Health informatics pioneer and the father of LOINC</v>
       </c>
     </row>
@@ -1222,7 +1211,7 @@
       <c r="D7" s="3">
         <v>3</v>
       </c>
-      <c r="E7" s="7" t="str">
+      <c r="E7" s="8" t="str">
         <v>ALT</v>
       </c>
       <c r="F7" s="3" t="str">
@@ -1282,8 +1271,8 @@
       <c r="X7" s="3">
         <v>-7</v>
       </c>
-      <c r="Y7" s="9" t="str">
-        <v>100002-5</v>
+      <c r="Y7" s="7" t="str">
+        <v>99932-5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>